<commit_message>
generated from SC22EVO/MCB.json at 05bca40
</commit_message>
<xml_diff>
--- a/SC22EVO/artifacts/MCB.xlsx
+++ b/SC22EVO/artifacts/MCB.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="798" uniqueCount="173">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="810" uniqueCount="171">
   <si>
     <t>ID</t>
   </si>
@@ -391,7 +391,7 @@
     <t>0..31968.8</t>
   </si>
   <si>
-    <t>31.25 -</t>
+    <t>31.25  Ohm</t>
   </si>
   <si>
     <t>NTC2_Resistance</t>
@@ -472,10 +472,7 @@
     <t>Sens_Front_NTC</t>
   </si>
   <si>
-    <t>NTC__Resistance</t>
-  </si>
-  <si>
-    <t>0..1023</t>
+    <t>NTC_1_Resistance</t>
   </si>
   <si>
     <t>NTC_2_Resistance</t>
@@ -497,9 +494,6 @@
   </si>
   <si>
     <t>Sens_Rear_NTC</t>
-  </si>
-  <si>
-    <t>NTC_1_Resistance</t>
   </si>
   <si>
     <t>NTC_5_Resistance</t>
@@ -5057,7 +5051,7 @@
         <v>10</v>
       </c>
       <c r="K83" s="2">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="L83" s="2" t="s">
         <v>27</v>
@@ -5077,9 +5071,11 @@
       <c r="S83" s="2"/>
       <c r="T83" s="2"/>
       <c r="U83" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="V83" s="2"/>
+        <v>123</v>
+      </c>
+      <c r="V83" s="2" t="s">
+        <v>124</v>
+      </c>
     </row>
     <row r="84" spans="1:22" outlineLevel="1">
       <c r="A84" s="5" t="s">
@@ -5100,14 +5096,14 @@
         <v>2</v>
       </c>
       <c r="H84" s="6" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="I84" s="6"/>
       <c r="J84" s="6">
         <v>10</v>
       </c>
       <c r="K84" s="6">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="L84" s="6" t="s">
         <v>27</v>
@@ -5127,9 +5123,11 @@
       <c r="S84" s="6"/>
       <c r="T84" s="6"/>
       <c r="U84" s="6" t="s">
-        <v>152</v>
-      </c>
-      <c r="V84" s="6"/>
+        <v>123</v>
+      </c>
+      <c r="V84" s="6" t="s">
+        <v>124</v>
+      </c>
     </row>
     <row r="85" spans="1:22" outlineLevel="1">
       <c r="A85" s="5" t="s">
@@ -5150,14 +5148,14 @@
         <v>4</v>
       </c>
       <c r="H85" s="6" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="I85" s="6"/>
       <c r="J85" s="6">
         <v>10</v>
       </c>
       <c r="K85" s="6">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="L85" s="6" t="s">
         <v>27</v>
@@ -5177,9 +5175,11 @@
       <c r="S85" s="6"/>
       <c r="T85" s="6"/>
       <c r="U85" s="6" t="s">
-        <v>152</v>
-      </c>
-      <c r="V85" s="6"/>
+        <v>123</v>
+      </c>
+      <c r="V85" s="6" t="s">
+        <v>124</v>
+      </c>
     </row>
     <row r="86" spans="1:22" outlineLevel="1">
       <c r="A86" s="5" t="s">
@@ -5200,14 +5200,14 @@
         <v>6</v>
       </c>
       <c r="H86" s="6" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="I86" s="6"/>
       <c r="J86" s="6">
         <v>10</v>
       </c>
       <c r="K86" s="6">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="L86" s="6" t="s">
         <v>27</v>
@@ -5227,9 +5227,11 @@
       <c r="S86" s="6"/>
       <c r="T86" s="6"/>
       <c r="U86" s="6" t="s">
-        <v>152</v>
-      </c>
-      <c r="V86" s="6"/>
+        <v>123</v>
+      </c>
+      <c r="V86" s="6" t="s">
+        <v>124</v>
+      </c>
     </row>
     <row r="87" spans="1:22" outlineLevel="1">
       <c r="A87" s="5" t="s">
@@ -5250,14 +5252,14 @@
         <v>0</v>
       </c>
       <c r="H87" s="6" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="I87" s="6"/>
       <c r="J87" s="6">
         <v>10</v>
       </c>
       <c r="K87" s="6">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="L87" s="6" t="s">
         <v>27</v>
@@ -5277,9 +5279,11 @@
       <c r="S87" s="6"/>
       <c r="T87" s="6"/>
       <c r="U87" s="6" t="s">
-        <v>152</v>
-      </c>
-      <c r="V87" s="6"/>
+        <v>123</v>
+      </c>
+      <c r="V87" s="6" t="s">
+        <v>124</v>
+      </c>
     </row>
     <row r="88" spans="1:22" outlineLevel="1">
       <c r="A88" s="5" t="s">
@@ -5300,14 +5304,14 @@
         <v>2</v>
       </c>
       <c r="H88" s="6" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="I88" s="6"/>
       <c r="J88" s="6">
         <v>10</v>
       </c>
       <c r="K88" s="6">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="L88" s="6" t="s">
         <v>27</v>
@@ -5327,16 +5331,18 @@
       <c r="S88" s="6"/>
       <c r="T88" s="6"/>
       <c r="U88" s="6" t="s">
-        <v>152</v>
-      </c>
-      <c r="V88" s="6"/>
+        <v>123</v>
+      </c>
+      <c r="V88" s="6" t="s">
+        <v>124</v>
+      </c>
     </row>
     <row r="89" spans="1:22">
       <c r="A89" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="B89" s="2" t="s">
         <v>158</v>
-      </c>
-      <c r="B89" s="2" t="s">
-        <v>159</v>
       </c>
       <c r="C89" s="2">
         <v>0</v>
@@ -5350,14 +5356,14 @@
         <v>0</v>
       </c>
       <c r="H89" s="2" t="s">
-        <v>160</v>
+        <v>151</v>
       </c>
       <c r="I89" s="2"/>
       <c r="J89" s="2">
         <v>10</v>
       </c>
       <c r="K89" s="2">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="L89" s="2" t="s">
         <v>27</v>
@@ -5377,16 +5383,18 @@
       <c r="S89" s="2"/>
       <c r="T89" s="2"/>
       <c r="U89" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="V89" s="2"/>
+        <v>123</v>
+      </c>
+      <c r="V89" s="2" t="s">
+        <v>124</v>
+      </c>
     </row>
     <row r="90" spans="1:22" outlineLevel="1">
       <c r="A90" s="5" t="s">
+        <v>157</v>
+      </c>
+      <c r="B90" s="5" t="s">
         <v>158</v>
-      </c>
-      <c r="B90" s="5" t="s">
-        <v>159</v>
       </c>
       <c r="C90" s="5">
         <v>0</v>
@@ -5400,14 +5408,14 @@
         <v>2</v>
       </c>
       <c r="H90" s="6" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="I90" s="6"/>
       <c r="J90" s="6">
         <v>10</v>
       </c>
       <c r="K90" s="6">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="L90" s="6" t="s">
         <v>27</v>
@@ -5427,16 +5435,18 @@
       <c r="S90" s="6"/>
       <c r="T90" s="6"/>
       <c r="U90" s="6" t="s">
-        <v>152</v>
-      </c>
-      <c r="V90" s="6"/>
+        <v>123</v>
+      </c>
+      <c r="V90" s="6" t="s">
+        <v>124</v>
+      </c>
     </row>
     <row r="91" spans="1:22" outlineLevel="1">
       <c r="A91" s="5" t="s">
+        <v>157</v>
+      </c>
+      <c r="B91" s="5" t="s">
         <v>158</v>
-      </c>
-      <c r="B91" s="5" t="s">
-        <v>159</v>
       </c>
       <c r="C91" s="5">
         <v>0</v>
@@ -5450,14 +5460,14 @@
         <v>4</v>
       </c>
       <c r="H91" s="6" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="I91" s="6"/>
       <c r="J91" s="6">
         <v>10</v>
       </c>
       <c r="K91" s="6">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="L91" s="6" t="s">
         <v>27</v>
@@ -5477,16 +5487,18 @@
       <c r="S91" s="6"/>
       <c r="T91" s="6"/>
       <c r="U91" s="6" t="s">
-        <v>152</v>
-      </c>
-      <c r="V91" s="6"/>
+        <v>123</v>
+      </c>
+      <c r="V91" s="6" t="s">
+        <v>124</v>
+      </c>
     </row>
     <row r="92" spans="1:22" outlineLevel="1">
       <c r="A92" s="5" t="s">
+        <v>157</v>
+      </c>
+      <c r="B92" s="5" t="s">
         <v>158</v>
-      </c>
-      <c r="B92" s="5" t="s">
-        <v>159</v>
       </c>
       <c r="C92" s="5">
         <v>0</v>
@@ -5500,14 +5512,14 @@
         <v>6</v>
       </c>
       <c r="H92" s="6" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="I92" s="6"/>
       <c r="J92" s="6">
         <v>10</v>
       </c>
       <c r="K92" s="6">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="L92" s="6" t="s">
         <v>27</v>
@@ -5527,16 +5539,18 @@
       <c r="S92" s="6"/>
       <c r="T92" s="6"/>
       <c r="U92" s="6" t="s">
-        <v>152</v>
-      </c>
-      <c r="V92" s="6"/>
+        <v>123</v>
+      </c>
+      <c r="V92" s="6" t="s">
+        <v>124</v>
+      </c>
     </row>
     <row r="93" spans="1:22" outlineLevel="1">
       <c r="A93" s="5" t="s">
+        <v>157</v>
+      </c>
+      <c r="B93" s="5" t="s">
         <v>158</v>
-      </c>
-      <c r="B93" s="5" t="s">
-        <v>159</v>
       </c>
       <c r="C93" s="5">
         <v>0</v>
@@ -5550,14 +5564,14 @@
         <v>0</v>
       </c>
       <c r="H93" s="6" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="I93" s="6"/>
       <c r="J93" s="6">
         <v>10</v>
       </c>
       <c r="K93" s="6">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="L93" s="6" t="s">
         <v>27</v>
@@ -5577,16 +5591,18 @@
       <c r="S93" s="6"/>
       <c r="T93" s="6"/>
       <c r="U93" s="6" t="s">
-        <v>152</v>
-      </c>
-      <c r="V93" s="6"/>
+        <v>123</v>
+      </c>
+      <c r="V93" s="6" t="s">
+        <v>124</v>
+      </c>
     </row>
     <row r="94" spans="1:22" outlineLevel="1">
       <c r="A94" s="5" t="s">
+        <v>157</v>
+      </c>
+      <c r="B94" s="5" t="s">
         <v>158</v>
-      </c>
-      <c r="B94" s="5" t="s">
-        <v>159</v>
       </c>
       <c r="C94" s="5">
         <v>0</v>
@@ -5600,14 +5616,14 @@
         <v>2</v>
       </c>
       <c r="H94" s="6" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="I94" s="6"/>
       <c r="J94" s="6">
         <v>10</v>
       </c>
       <c r="K94" s="6">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="L94" s="6" t="s">
         <v>27</v>
@@ -5627,16 +5643,18 @@
       <c r="S94" s="6"/>
       <c r="T94" s="6"/>
       <c r="U94" s="6" t="s">
-        <v>152</v>
-      </c>
-      <c r="V94" s="6"/>
+        <v>123</v>
+      </c>
+      <c r="V94" s="6" t="s">
+        <v>124</v>
+      </c>
     </row>
     <row r="95" spans="1:22">
       <c r="A95" s="2" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="B95" s="2" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="C95" s="2">
         <v>0</v>
@@ -5650,7 +5668,7 @@
         <v>0</v>
       </c>
       <c r="H95" s="2" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="I95" s="2"/>
       <c r="J95" s="2">
@@ -5683,10 +5701,10 @@
     </row>
     <row r="96" spans="1:22" outlineLevel="1">
       <c r="A96" s="5" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="B96" s="5" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="C96" s="5">
         <v>0</v>
@@ -5700,7 +5718,7 @@
         <v>0</v>
       </c>
       <c r="H96" s="6" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="I96" s="6"/>
       <c r="J96" s="6">
@@ -5733,10 +5751,10 @@
     </row>
     <row r="97" spans="1:22">
       <c r="A97" s="2" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="B97" s="2" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="C97" s="2">
         <v>0</v>
@@ -5750,7 +5768,7 @@
         <v>0</v>
       </c>
       <c r="H97" s="2" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="I97" s="2"/>
       <c r="J97" s="2">
@@ -5781,10 +5799,10 @@
     </row>
     <row r="98" spans="1:22" outlineLevel="1">
       <c r="A98" s="5" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="B98" s="5" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="C98" s="5">
         <v>0</v>
@@ -5798,7 +5816,7 @@
         <v>1</v>
       </c>
       <c r="H98" s="6" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="I98" s="6"/>
       <c r="J98" s="6">
@@ -5829,10 +5847,10 @@
     </row>
     <row r="99" spans="1:22" outlineLevel="1">
       <c r="A99" s="5" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="B99" s="5" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="C99" s="5">
         <v>0</v>
@@ -5846,7 +5864,7 @@
         <v>2</v>
       </c>
       <c r="H99" s="6" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="I99" s="6"/>
       <c r="J99" s="6">
@@ -5877,10 +5895,10 @@
     </row>
     <row r="100" spans="1:22" outlineLevel="1">
       <c r="A100" s="5" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="B100" s="5" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="C100" s="5">
         <v>0</v>
@@ -5894,7 +5912,7 @@
         <v>3</v>
       </c>
       <c r="H100" s="6" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="I100" s="6"/>
       <c r="J100" s="6">

</xml_diff>

<commit_message>
generated from SC22EVO/MCB.json at 69beac6
</commit_message>
<xml_diff>
--- a/SC22EVO/artifacts/MCB.xlsx
+++ b/SC22EVO/artifacts/MCB.xlsx
@@ -352,10 +352,10 @@
     <t>Current_Sensor_Voltage</t>
   </si>
   <si>
-    <t>0..4980.66</t>
-  </si>
-  <si>
-    <t>0.076 -</t>
+    <t>-20..20.6317</t>
+  </si>
+  <si>
+    <t>0.00062 -</t>
   </si>
   <si>
     <t>LV_Total_Voltage_mV</t>
@@ -3677,7 +3677,7 @@
         <v>16</v>
       </c>
       <c r="K56" s="2">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="L56" s="2" t="s">
         <v>27</v>

</xml_diff>

<commit_message>
generated from SC22EVO/MCB.json at a5e95d8
</commit_message>
<xml_diff>
--- a/SC22EVO/artifacts/MCB.xlsx
+++ b/SC22EVO/artifacts/MCB.xlsx
@@ -349,13 +349,13 @@
     <t>BMSLV_BatteryPackGeneral</t>
   </si>
   <si>
-    <t>Current_Sensor_Voltage</t>
-  </si>
-  <si>
-    <t>-20..20.6317</t>
-  </si>
-  <si>
-    <t>0.00062 -</t>
+    <t>Current_Sensor_Voltage_mA</t>
+  </si>
+  <si>
+    <t>-20000..20631.7</t>
+  </si>
+  <si>
+    <t>0.62 -</t>
   </si>
   <si>
     <t>LV_Total_Voltage_mV</t>
@@ -3677,7 +3677,7 @@
         <v>16</v>
       </c>
       <c r="K56" s="2">
-        <v>20</v>
+        <v>20000</v>
       </c>
       <c r="L56" s="2" t="s">
         <v>27</v>

</xml_diff>

<commit_message>
generated from SC22EVO/MCB.json at 727e120
</commit_message>
<xml_diff>
--- a/SC22EVO/artifacts/MCB.xlsx
+++ b/SC22EVO/artifacts/MCB.xlsx
@@ -349,13 +349,13 @@
     <t>BMSLV_BatteryPackGeneral</t>
   </si>
   <si>
-    <t>Current_Sensor_Voltage_mA</t>
-  </si>
-  <si>
-    <t>-20000..20631.7</t>
-  </si>
-  <si>
-    <t>0.62 -</t>
+    <t>Current_Sensor_mV</t>
+  </si>
+  <si>
+    <t>0..4980.66</t>
+  </si>
+  <si>
+    <t>0.076 -</t>
   </si>
   <si>
     <t>LV_Total_Voltage_mV</t>
@@ -3677,7 +3677,7 @@
         <v>16</v>
       </c>
       <c r="K56" s="2">
-        <v>20000</v>
+        <v>0</v>
       </c>
       <c r="L56" s="2" t="s">
         <v>27</v>

</xml_diff>

<commit_message>
generated from SC22EVO/MCB.json at 23a8ea5
</commit_message>
<xml_diff>
--- a/SC22EVO/artifacts/MCB.xlsx
+++ b/SC22EVO/artifacts/MCB.xlsx
@@ -10,14 +10,14 @@
     <sheet name="K-Matrix " sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'K-Matrix '!$A$1:$AH$103</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'K-Matrix '!$A$1:$AH$104</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="826" uniqueCount="176">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="835" uniqueCount="177">
   <si>
     <t>ID</t>
   </si>
@@ -380,6 +380,9 @@
   </si>
   <si>
     <t>0.267 -</t>
+  </si>
+  <si>
+    <t>LV_Total_Voltage_Sum_mV</t>
   </si>
   <si>
     <t>103h</t>
@@ -933,7 +936,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W102"/>
+  <dimension ref="A1:W103"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="1"/>
   <cols>
     <col min="1" max="1" width="4.28515625" customWidth="1"/>
@@ -3478,7 +3481,7 @@
         <v>16</v>
       </c>
       <c r="K51" s="2">
-        <v>2000</v>
+        <v>-0.016</v>
       </c>
       <c r="L51" s="2" t="s">
         <v>28</v>
@@ -3531,7 +3534,7 @@
         <v>16</v>
       </c>
       <c r="K52" s="6">
-        <v>2000</v>
+        <v>-0.016</v>
       </c>
       <c r="L52" s="6" t="s">
         <v>28</v>
@@ -3584,7 +3587,7 @@
         <v>16</v>
       </c>
       <c r="K53" s="6">
-        <v>2000</v>
+        <v>-0.016</v>
       </c>
       <c r="L53" s="6" t="s">
         <v>28</v>
@@ -3637,7 +3640,7 @@
         <v>16</v>
       </c>
       <c r="K54" s="6">
-        <v>2000</v>
+        <v>-0.016</v>
       </c>
       <c r="L54" s="6" t="s">
         <v>28</v>
@@ -3690,7 +3693,7 @@
         <v>16</v>
       </c>
       <c r="K55" s="2">
-        <v>2000</v>
+        <v>-0.016</v>
       </c>
       <c r="L55" s="2" t="s">
         <v>28</v>
@@ -3743,7 +3746,7 @@
         <v>16</v>
       </c>
       <c r="K56" s="6">
-        <v>2000</v>
+        <v>-0.016</v>
       </c>
       <c r="L56" s="6" t="s">
         <v>28</v>
@@ -3796,7 +3799,7 @@
         <v>16</v>
       </c>
       <c r="K57" s="6">
-        <v>2000</v>
+        <v>-0.016</v>
       </c>
       <c r="L57" s="6" t="s">
         <v>28</v>
@@ -3902,7 +3905,7 @@
         <v>16</v>
       </c>
       <c r="K59" s="6">
-        <v>14000</v>
+        <v>0.122</v>
       </c>
       <c r="L59" s="6" t="s">
         <v>28</v>
@@ -3929,218 +3932,218 @@
         <v>120</v>
       </c>
     </row>
-    <row r="60" spans="1:23">
-      <c r="A60" s="2" t="s">
+    <row r="60" spans="1:23" outlineLevel="1">
+      <c r="A60" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="B60" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="C60" s="5">
+        <v>0</v>
+      </c>
+      <c r="D60" s="5"/>
+      <c r="E60" s="5"/>
+      <c r="F60" s="6">
+        <v>5</v>
+      </c>
+      <c r="G60" s="6">
+        <v>0</v>
+      </c>
+      <c r="H60" s="6" t="s">
         <v>121</v>
       </c>
-      <c r="B60" s="2" t="s">
+      <c r="I60" s="6"/>
+      <c r="J60" s="6">
+        <v>16</v>
+      </c>
+      <c r="K60" s="6">
+        <v>0.122</v>
+      </c>
+      <c r="L60" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="M60" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="N60" s="8"/>
+      <c r="O60" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="P60" s="8"/>
+      <c r="Q60" s="6"/>
+      <c r="R60" s="8"/>
+      <c r="S60" s="6"/>
+      <c r="T60" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="U60" s="6"/>
+      <c r="V60" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="W60" s="6" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="61" spans="1:23">
+      <c r="A61" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="C60" s="2">
-        <v>0</v>
-      </c>
-      <c r="D60" s="2"/>
-      <c r="E60" s="2"/>
-      <c r="F60" s="2">
-        <v>1</v>
-      </c>
-      <c r="G60" s="2">
-        <v>0</v>
-      </c>
-      <c r="H60" s="2" t="s">
+      <c r="B61" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="I60" s="2"/>
-      <c r="J60" s="2">
-        <v>1</v>
-      </c>
-      <c r="K60" s="2">
-        <v>0</v>
-      </c>
-      <c r="L60" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="M60" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="N60" s="4"/>
-      <c r="O60" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="P60" s="4"/>
-      <c r="Q60" s="2"/>
-      <c r="R60" s="4"/>
-      <c r="S60" s="2"/>
-      <c r="T60" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="U60" s="2"/>
-      <c r="V60" s="2"/>
-      <c r="W60" s="2"/>
-    </row>
-    <row r="61" spans="1:23" outlineLevel="1">
-      <c r="A61" s="5" t="s">
-        <v>121</v>
-      </c>
-      <c r="B61" s="5" t="s">
+      <c r="C61" s="2">
+        <v>0</v>
+      </c>
+      <c r="D61" s="2"/>
+      <c r="E61" s="2"/>
+      <c r="F61" s="2">
+        <v>1</v>
+      </c>
+      <c r="G61" s="2">
+        <v>0</v>
+      </c>
+      <c r="H61" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="I61" s="2"/>
+      <c r="J61" s="2">
+        <v>1</v>
+      </c>
+      <c r="K61" s="2">
+        <v>0</v>
+      </c>
+      <c r="L61" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="M61" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="N61" s="4"/>
+      <c r="O61" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="P61" s="4"/>
+      <c r="Q61" s="2"/>
+      <c r="R61" s="4"/>
+      <c r="S61" s="2"/>
+      <c r="T61" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="U61" s="2"/>
+      <c r="V61" s="2"/>
+      <c r="W61" s="2"/>
+    </row>
+    <row r="62" spans="1:23" outlineLevel="1">
+      <c r="A62" s="5" t="s">
         <v>122</v>
       </c>
-      <c r="C61" s="5">
-        <v>0</v>
-      </c>
-      <c r="D61" s="5"/>
-      <c r="E61" s="5"/>
-      <c r="F61" s="6">
-        <v>1</v>
-      </c>
-      <c r="G61" s="6">
-        <v>1</v>
-      </c>
-      <c r="H61" s="6" t="s">
-        <v>124</v>
-      </c>
-      <c r="I61" s="6"/>
-      <c r="J61" s="6">
+      <c r="B62" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="C62" s="5">
+        <v>0</v>
+      </c>
+      <c r="D62" s="5"/>
+      <c r="E62" s="5"/>
+      <c r="F62" s="6">
+        <v>1</v>
+      </c>
+      <c r="G62" s="6">
+        <v>1</v>
+      </c>
+      <c r="H62" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="I62" s="6"/>
+      <c r="J62" s="6">
         <v>8</v>
       </c>
-      <c r="K61" s="6">
-        <v>0</v>
-      </c>
-      <c r="L61" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="M61" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="N61" s="8"/>
-      <c r="O61" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="P61" s="8"/>
-      <c r="Q61" s="6"/>
-      <c r="R61" s="8"/>
-      <c r="S61" s="6"/>
-      <c r="T61" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="U61" s="6"/>
-      <c r="V61" s="6" t="s">
+      <c r="K62" s="6">
+        <v>0</v>
+      </c>
+      <c r="L62" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="M62" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="N62" s="8"/>
+      <c r="O62" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="P62" s="8"/>
+      <c r="Q62" s="6"/>
+      <c r="R62" s="8"/>
+      <c r="S62" s="6"/>
+      <c r="T62" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="U62" s="6"/>
+      <c r="V62" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="W61" s="6"/>
-    </row>
-    <row r="62" spans="1:23">
-      <c r="A62" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="B62" s="2" t="s">
+      <c r="W62" s="6"/>
+    </row>
+    <row r="63" spans="1:23">
+      <c r="A63" s="2" t="s">
         <v>126</v>
       </c>
-      <c r="C62" s="2">
-        <v>0</v>
-      </c>
-      <c r="D62" s="2"/>
-      <c r="E62" s="2"/>
-      <c r="F62" s="2">
-        <v>1</v>
-      </c>
-      <c r="G62" s="2">
-        <v>1</v>
-      </c>
-      <c r="H62" s="2" t="s">
+      <c r="B63" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="I62" s="2"/>
-      <c r="J62" s="2">
+      <c r="C63" s="2">
+        <v>0</v>
+      </c>
+      <c r="D63" s="2"/>
+      <c r="E63" s="2"/>
+      <c r="F63" s="2">
+        <v>1</v>
+      </c>
+      <c r="G63" s="2">
+        <v>1</v>
+      </c>
+      <c r="H63" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="I63" s="2"/>
+      <c r="J63" s="2">
         <v>10</v>
       </c>
-      <c r="K62" s="2">
-        <v>1000</v>
-      </c>
-      <c r="L62" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="M62" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="N62" s="4"/>
-      <c r="O62" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="P62" s="4"/>
-      <c r="Q62" s="2"/>
-      <c r="R62" s="4"/>
-      <c r="S62" s="2"/>
-      <c r="T62" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="U62" s="2"/>
-      <c r="V62" s="2" t="s">
-        <v>128</v>
-      </c>
-      <c r="W62" s="2" t="s">
+      <c r="K63" s="2">
+        <v>0</v>
+      </c>
+      <c r="L63" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="M63" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="N63" s="4"/>
+      <c r="O63" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="P63" s="4"/>
+      <c r="Q63" s="2"/>
+      <c r="R63" s="4"/>
+      <c r="S63" s="2"/>
+      <c r="T63" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="U63" s="2"/>
+      <c r="V63" s="2" t="s">
         <v>129</v>
       </c>
-    </row>
-    <row r="63" spans="1:23" outlineLevel="1">
-      <c r="A63" s="5" t="s">
-        <v>125</v>
-      </c>
-      <c r="B63" s="5" t="s">
-        <v>126</v>
-      </c>
-      <c r="C63" s="5">
-        <v>0</v>
-      </c>
-      <c r="D63" s="5"/>
-      <c r="E63" s="5"/>
-      <c r="F63" s="6">
-        <v>2</v>
-      </c>
-      <c r="G63" s="6">
-        <v>3</v>
-      </c>
-      <c r="H63" s="6" t="s">
+      <c r="W63" s="2" t="s">
         <v>130</v>
-      </c>
-      <c r="I63" s="6"/>
-      <c r="J63" s="6">
-        <v>10</v>
-      </c>
-      <c r="K63" s="6">
-        <v>1000</v>
-      </c>
-      <c r="L63" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="M63" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="N63" s="8"/>
-      <c r="O63" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="P63" s="8"/>
-      <c r="Q63" s="6"/>
-      <c r="R63" s="8"/>
-      <c r="S63" s="6"/>
-      <c r="T63" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="U63" s="6"/>
-      <c r="V63" s="6" t="s">
-        <v>128</v>
-      </c>
-      <c r="W63" s="6" t="s">
-        <v>129</v>
       </c>
     </row>
     <row r="64" spans="1:23" outlineLevel="1">
       <c r="A64" s="5" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B64" s="5" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C64" s="5">
         <v>0</v>
@@ -4148,10 +4151,10 @@
       <c r="D64" s="5"/>
       <c r="E64" s="5"/>
       <c r="F64" s="6">
+        <v>2</v>
+      </c>
+      <c r="G64" s="6">
         <v>3</v>
-      </c>
-      <c r="G64" s="6">
-        <v>5</v>
       </c>
       <c r="H64" s="6" t="s">
         <v>131</v>
@@ -4161,7 +4164,7 @@
         <v>10</v>
       </c>
       <c r="K64" s="6">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="L64" s="6" t="s">
         <v>28</v>
@@ -4182,18 +4185,18 @@
       </c>
       <c r="U64" s="6"/>
       <c r="V64" s="6" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="W64" s="6" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="65" spans="1:23" outlineLevel="1">
       <c r="A65" s="5" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B65" s="5" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C65" s="5">
         <v>0</v>
@@ -4201,10 +4204,10 @@
       <c r="D65" s="5"/>
       <c r="E65" s="5"/>
       <c r="F65" s="6">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G65" s="6">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="H65" s="6" t="s">
         <v>132</v>
@@ -4214,7 +4217,7 @@
         <v>10</v>
       </c>
       <c r="K65" s="6">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="L65" s="6" t="s">
         <v>28</v>
@@ -4235,18 +4238,18 @@
       </c>
       <c r="U65" s="6"/>
       <c r="V65" s="6" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="W65" s="6" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="66" spans="1:23" outlineLevel="1">
       <c r="A66" s="5" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B66" s="5" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C66" s="5">
         <v>0</v>
@@ -4254,10 +4257,10 @@
       <c r="D66" s="5"/>
       <c r="E66" s="5"/>
       <c r="F66" s="6">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G66" s="6">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="H66" s="6" t="s">
         <v>133</v>
@@ -4267,7 +4270,7 @@
         <v>10</v>
       </c>
       <c r="K66" s="6">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="L66" s="6" t="s">
         <v>28</v>
@@ -4288,18 +4291,18 @@
       </c>
       <c r="U66" s="6"/>
       <c r="V66" s="6" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="W66" s="6" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="67" spans="1:23" outlineLevel="1">
       <c r="A67" s="5" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B67" s="5" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C67" s="5">
         <v>0</v>
@@ -4307,10 +4310,10 @@
       <c r="D67" s="5"/>
       <c r="E67" s="5"/>
       <c r="F67" s="6">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G67" s="6">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="H67" s="6" t="s">
         <v>134</v>
@@ -4320,7 +4323,7 @@
         <v>10</v>
       </c>
       <c r="K67" s="6">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="L67" s="6" t="s">
         <v>28</v>
@@ -4341,124 +4344,124 @@
       </c>
       <c r="U67" s="6"/>
       <c r="V67" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="W67" s="6" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="68" spans="1:23" outlineLevel="1">
+      <c r="A68" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="B68" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="C68" s="5">
+        <v>0</v>
+      </c>
+      <c r="D68" s="5"/>
+      <c r="E68" s="5"/>
+      <c r="F68" s="6">
+        <v>7</v>
+      </c>
+      <c r="G68" s="6">
+        <v>6</v>
+      </c>
+      <c r="H68" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="I68" s="6"/>
+      <c r="J68" s="6">
+        <v>10</v>
+      </c>
+      <c r="K68" s="6">
+        <v>0</v>
+      </c>
+      <c r="L68" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="M68" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="N68" s="8"/>
+      <c r="O68" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="P68" s="8"/>
+      <c r="Q68" s="6"/>
+      <c r="R68" s="8"/>
+      <c r="S68" s="6"/>
+      <c r="T68" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="U68" s="6"/>
+      <c r="V68" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="W68" s="6" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="69" spans="1:23">
+      <c r="A69" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="B69" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="C69" s="2">
+        <v>0</v>
+      </c>
+      <c r="D69" s="2"/>
+      <c r="E69" s="2"/>
+      <c r="F69" s="2">
+        <v>1</v>
+      </c>
+      <c r="G69" s="2">
+        <v>1</v>
+      </c>
+      <c r="H69" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="W67" s="6" t="s">
+      <c r="I69" s="2"/>
+      <c r="J69" s="2">
+        <v>10</v>
+      </c>
+      <c r="K69" s="2">
+        <v>0</v>
+      </c>
+      <c r="L69" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="M69" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="N69" s="4"/>
+      <c r="O69" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="P69" s="4"/>
+      <c r="Q69" s="2"/>
+      <c r="R69" s="4"/>
+      <c r="S69" s="2"/>
+      <c r="T69" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="U69" s="2"/>
+      <c r="V69" s="2" t="s">
         <v>129</v>
       </c>
-    </row>
-    <row r="68" spans="1:23">
-      <c r="A68" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="B68" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="C68" s="2">
-        <v>0</v>
-      </c>
-      <c r="D68" s="2"/>
-      <c r="E68" s="2"/>
-      <c r="F68" s="2">
-        <v>1</v>
-      </c>
-      <c r="G68" s="2">
-        <v>1</v>
-      </c>
-      <c r="H68" s="2" t="s">
-        <v>127</v>
-      </c>
-      <c r="I68" s="2"/>
-      <c r="J68" s="2">
-        <v>10</v>
-      </c>
-      <c r="K68" s="2">
-        <v>1000</v>
-      </c>
-      <c r="L68" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="M68" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="N68" s="4"/>
-      <c r="O68" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="P68" s="4"/>
-      <c r="Q68" s="2"/>
-      <c r="R68" s="4"/>
-      <c r="S68" s="2"/>
-      <c r="T68" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="U68" s="2"/>
-      <c r="V68" s="2" t="s">
-        <v>128</v>
-      </c>
-      <c r="W68" s="2" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="69" spans="1:23" outlineLevel="1">
-      <c r="A69" s="5" t="s">
-        <v>135</v>
-      </c>
-      <c r="B69" s="5" t="s">
-        <v>136</v>
-      </c>
-      <c r="C69" s="5">
-        <v>0</v>
-      </c>
-      <c r="D69" s="5"/>
-      <c r="E69" s="5"/>
-      <c r="F69" s="6">
-        <v>2</v>
-      </c>
-      <c r="G69" s="6">
-        <v>3</v>
-      </c>
-      <c r="H69" s="6" t="s">
+      <c r="W69" s="2" t="s">
         <v>130</v>
-      </c>
-      <c r="I69" s="6"/>
-      <c r="J69" s="6">
-        <v>10</v>
-      </c>
-      <c r="K69" s="6">
-        <v>1000</v>
-      </c>
-      <c r="L69" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="M69" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="N69" s="8"/>
-      <c r="O69" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="P69" s="8"/>
-      <c r="Q69" s="6"/>
-      <c r="R69" s="8"/>
-      <c r="S69" s="6"/>
-      <c r="T69" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="U69" s="6"/>
-      <c r="V69" s="6" t="s">
-        <v>128</v>
-      </c>
-      <c r="W69" s="6" t="s">
-        <v>129</v>
       </c>
     </row>
     <row r="70" spans="1:23" outlineLevel="1">
       <c r="A70" s="5" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B70" s="5" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C70" s="5">
         <v>0</v>
@@ -4466,10 +4469,10 @@
       <c r="D70" s="5"/>
       <c r="E70" s="5"/>
       <c r="F70" s="6">
+        <v>2</v>
+      </c>
+      <c r="G70" s="6">
         <v>3</v>
-      </c>
-      <c r="G70" s="6">
-        <v>5</v>
       </c>
       <c r="H70" s="6" t="s">
         <v>131</v>
@@ -4479,7 +4482,7 @@
         <v>10</v>
       </c>
       <c r="K70" s="6">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="L70" s="6" t="s">
         <v>28</v>
@@ -4500,18 +4503,18 @@
       </c>
       <c r="U70" s="6"/>
       <c r="V70" s="6" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="W70" s="6" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="71" spans="1:23" outlineLevel="1">
       <c r="A71" s="5" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B71" s="5" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C71" s="5">
         <v>0</v>
@@ -4519,10 +4522,10 @@
       <c r="D71" s="5"/>
       <c r="E71" s="5"/>
       <c r="F71" s="6">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G71" s="6">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="H71" s="6" t="s">
         <v>132</v>
@@ -4532,7 +4535,7 @@
         <v>10</v>
       </c>
       <c r="K71" s="6">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="L71" s="6" t="s">
         <v>28</v>
@@ -4553,18 +4556,18 @@
       </c>
       <c r="U71" s="6"/>
       <c r="V71" s="6" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="W71" s="6" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="72" spans="1:23" outlineLevel="1">
       <c r="A72" s="5" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B72" s="5" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C72" s="5">
         <v>0</v>
@@ -4572,10 +4575,10 @@
       <c r="D72" s="5"/>
       <c r="E72" s="5"/>
       <c r="F72" s="6">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G72" s="6">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="H72" s="6" t="s">
         <v>133</v>
@@ -4585,7 +4588,7 @@
         <v>10</v>
       </c>
       <c r="K72" s="6">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="L72" s="6" t="s">
         <v>28</v>
@@ -4606,18 +4609,18 @@
       </c>
       <c r="U72" s="6"/>
       <c r="V72" s="6" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="W72" s="6" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="73" spans="1:23" outlineLevel="1">
       <c r="A73" s="5" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B73" s="5" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C73" s="5">
         <v>0</v>
@@ -4625,10 +4628,10 @@
       <c r="D73" s="5"/>
       <c r="E73" s="5"/>
       <c r="F73" s="6">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G73" s="6">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="H73" s="6" t="s">
         <v>134</v>
@@ -4638,7 +4641,7 @@
         <v>10</v>
       </c>
       <c r="K73" s="6">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="L73" s="6" t="s">
         <v>28</v>
@@ -4659,120 +4662,122 @@
       </c>
       <c r="U73" s="6"/>
       <c r="V73" s="6" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="W73" s="6" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="74" spans="1:23" outlineLevel="1">
+      <c r="A74" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="B74" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="C74" s="5">
+        <v>0</v>
+      </c>
+      <c r="D74" s="5"/>
+      <c r="E74" s="5"/>
+      <c r="F74" s="6">
+        <v>7</v>
+      </c>
+      <c r="G74" s="6">
+        <v>6</v>
+      </c>
+      <c r="H74" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="I74" s="6"/>
+      <c r="J74" s="6">
+        <v>10</v>
+      </c>
+      <c r="K74" s="6">
+        <v>0</v>
+      </c>
+      <c r="L74" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="M74" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="N74" s="8"/>
+      <c r="O74" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="P74" s="8"/>
+      <c r="Q74" s="6"/>
+      <c r="R74" s="8"/>
+      <c r="S74" s="6"/>
+      <c r="T74" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="U74" s="6"/>
+      <c r="V74" s="6" t="s">
         <v>129</v>
       </c>
-    </row>
-    <row r="74" spans="1:23">
-      <c r="A74" s="2" t="s">
-        <v>137</v>
-      </c>
-      <c r="B74" s="2" t="s">
+      <c r="W74" s="6" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="75" spans="1:23">
+      <c r="A75" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="C74" s="2">
-        <v>0</v>
-      </c>
-      <c r="D74" s="2"/>
-      <c r="E74" s="2"/>
-      <c r="F74" s="2">
-        <v>1</v>
-      </c>
-      <c r="G74" s="2">
-        <v>0</v>
-      </c>
-      <c r="H74" s="2" t="s">
+      <c r="B75" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="I74" s="2"/>
-      <c r="J74" s="2">
+      <c r="C75" s="2">
+        <v>0</v>
+      </c>
+      <c r="D75" s="2"/>
+      <c r="E75" s="2"/>
+      <c r="F75" s="2">
+        <v>1</v>
+      </c>
+      <c r="G75" s="2">
+        <v>0</v>
+      </c>
+      <c r="H75" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="I75" s="2"/>
+      <c r="J75" s="2">
         <v>16</v>
       </c>
-      <c r="K74" s="2">
-        <v>0</v>
-      </c>
-      <c r="L74" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="M74" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="N74" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="O74" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="P74" s="4"/>
-      <c r="Q74" s="2"/>
-      <c r="R74" s="4"/>
-      <c r="S74" s="2"/>
-      <c r="T74" s="4"/>
-      <c r="U74" s="2"/>
-      <c r="V74" s="2" t="s">
+      <c r="K75" s="2">
+        <v>0</v>
+      </c>
+      <c r="L75" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="M75" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="N75" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="O75" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="P75" s="4"/>
+      <c r="Q75" s="2"/>
+      <c r="R75" s="4"/>
+      <c r="S75" s="2"/>
+      <c r="T75" s="4"/>
+      <c r="U75" s="2"/>
+      <c r="V75" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="W74" s="2"/>
-    </row>
-    <row r="75" spans="1:23" outlineLevel="1">
-      <c r="A75" s="5" t="s">
-        <v>137</v>
-      </c>
-      <c r="B75" s="5" t="s">
-        <v>138</v>
-      </c>
-      <c r="C75" s="5">
-        <v>0</v>
-      </c>
-      <c r="D75" s="5"/>
-      <c r="E75" s="5"/>
-      <c r="F75" s="6">
-        <v>3</v>
-      </c>
-      <c r="G75" s="6">
-        <v>0</v>
-      </c>
-      <c r="H75" s="6" t="s">
-        <v>140</v>
-      </c>
-      <c r="I75" s="6"/>
-      <c r="J75" s="6">
-        <v>16</v>
-      </c>
-      <c r="K75" s="6">
-        <v>0</v>
-      </c>
-      <c r="L75" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="M75" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="N75" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="O75" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="P75" s="8"/>
-      <c r="Q75" s="6"/>
-      <c r="R75" s="8"/>
-      <c r="S75" s="6"/>
-      <c r="T75" s="8"/>
-      <c r="U75" s="6"/>
-      <c r="V75" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="W75" s="6"/>
+      <c r="W75" s="2"/>
     </row>
     <row r="76" spans="1:23" outlineLevel="1">
       <c r="A76" s="5" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B76" s="5" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C76" s="5">
         <v>0</v>
@@ -4780,7 +4785,7 @@
       <c r="D76" s="5"/>
       <c r="E76" s="5"/>
       <c r="F76" s="6">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G76" s="6">
         <v>0</v>
@@ -4820,10 +4825,10 @@
     </row>
     <row r="77" spans="1:23" outlineLevel="1">
       <c r="A77" s="5" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B77" s="5" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C77" s="5">
         <v>0</v>
@@ -4831,7 +4836,7 @@
       <c r="D77" s="5"/>
       <c r="E77" s="5"/>
       <c r="F77" s="6">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="G77" s="6">
         <v>0</v>
@@ -4869,114 +4874,114 @@
       </c>
       <c r="W77" s="6"/>
     </row>
-    <row r="78" spans="1:23">
-      <c r="A78" s="2" t="s">
+    <row r="78" spans="1:23" outlineLevel="1">
+      <c r="A78" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="B78" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="C78" s="5">
+        <v>0</v>
+      </c>
+      <c r="D78" s="5"/>
+      <c r="E78" s="5"/>
+      <c r="F78" s="6">
+        <v>7</v>
+      </c>
+      <c r="G78" s="6">
+        <v>0</v>
+      </c>
+      <c r="H78" s="6" t="s">
         <v>143</v>
       </c>
-      <c r="B78" s="2" t="s">
+      <c r="I78" s="6"/>
+      <c r="J78" s="6">
+        <v>16</v>
+      </c>
+      <c r="K78" s="6">
+        <v>0</v>
+      </c>
+      <c r="L78" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="M78" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="N78" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="O78" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="P78" s="8"/>
+      <c r="Q78" s="6"/>
+      <c r="R78" s="8"/>
+      <c r="S78" s="6"/>
+      <c r="T78" s="8"/>
+      <c r="U78" s="6"/>
+      <c r="V78" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="W78" s="6"/>
+    </row>
+    <row r="79" spans="1:23">
+      <c r="A79" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="C78" s="2">
-        <v>0</v>
-      </c>
-      <c r="D78" s="2"/>
-      <c r="E78" s="2"/>
-      <c r="F78" s="2">
-        <v>1</v>
-      </c>
-      <c r="G78" s="2">
-        <v>0</v>
-      </c>
-      <c r="H78" s="2" t="s">
+      <c r="B79" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="I78" s="2"/>
-      <c r="J78" s="2">
+      <c r="C79" s="2">
+        <v>0</v>
+      </c>
+      <c r="D79" s="2"/>
+      <c r="E79" s="2"/>
+      <c r="F79" s="2">
+        <v>1</v>
+      </c>
+      <c r="G79" s="2">
+        <v>0</v>
+      </c>
+      <c r="H79" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="I79" s="2"/>
+      <c r="J79" s="2">
         <v>16</v>
       </c>
-      <c r="K78" s="2">
-        <v>0</v>
-      </c>
-      <c r="L78" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="M78" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="N78" s="4"/>
-      <c r="O78" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="P78" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q78" s="2"/>
-      <c r="R78" s="4"/>
-      <c r="S78" s="2"/>
-      <c r="T78" s="4"/>
-      <c r="U78" s="2"/>
-      <c r="V78" s="2" t="s">
+      <c r="K79" s="2">
+        <v>0</v>
+      </c>
+      <c r="L79" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="M79" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="N79" s="4"/>
+      <c r="O79" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="P79" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q79" s="2"/>
+      <c r="R79" s="4"/>
+      <c r="S79" s="2"/>
+      <c r="T79" s="4"/>
+      <c r="U79" s="2"/>
+      <c r="V79" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="W78" s="2"/>
-    </row>
-    <row r="79" spans="1:23" outlineLevel="1">
-      <c r="A79" s="5" t="s">
-        <v>143</v>
-      </c>
-      <c r="B79" s="5" t="s">
-        <v>144</v>
-      </c>
-      <c r="C79" s="5">
-        <v>0</v>
-      </c>
-      <c r="D79" s="5"/>
-      <c r="E79" s="5"/>
-      <c r="F79" s="6">
-        <v>3</v>
-      </c>
-      <c r="G79" s="6">
-        <v>0</v>
-      </c>
-      <c r="H79" s="6" t="s">
-        <v>146</v>
-      </c>
-      <c r="I79" s="6"/>
-      <c r="J79" s="6">
-        <v>16</v>
-      </c>
-      <c r="K79" s="6">
-        <v>0</v>
-      </c>
-      <c r="L79" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="M79" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="N79" s="8"/>
-      <c r="O79" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="P79" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q79" s="6"/>
-      <c r="R79" s="8"/>
-      <c r="S79" s="6"/>
-      <c r="T79" s="8"/>
-      <c r="U79" s="6"/>
-      <c r="V79" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="W79" s="6"/>
+      <c r="W79" s="2"/>
     </row>
     <row r="80" spans="1:23" outlineLevel="1">
       <c r="A80" s="5" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B80" s="5" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C80" s="5">
         <v>0</v>
@@ -4984,7 +4989,7 @@
       <c r="D80" s="5"/>
       <c r="E80" s="5"/>
       <c r="F80" s="6">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G80" s="6">
         <v>0</v>
@@ -5024,10 +5029,10 @@
     </row>
     <row r="81" spans="1:23" outlineLevel="1">
       <c r="A81" s="5" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B81" s="5" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C81" s="5">
         <v>0</v>
@@ -5035,7 +5040,7 @@
       <c r="D81" s="5"/>
       <c r="E81" s="5"/>
       <c r="F81" s="6">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="G81" s="6">
         <v>0</v>
@@ -5073,112 +5078,112 @@
       </c>
       <c r="W81" s="6"/>
     </row>
-    <row r="82" spans="1:23">
-      <c r="A82" s="2" t="s">
+    <row r="82" spans="1:23" outlineLevel="1">
+      <c r="A82" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="B82" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="C82" s="5">
+        <v>0</v>
+      </c>
+      <c r="D82" s="5"/>
+      <c r="E82" s="5"/>
+      <c r="F82" s="6">
+        <v>7</v>
+      </c>
+      <c r="G82" s="6">
+        <v>0</v>
+      </c>
+      <c r="H82" s="6" t="s">
         <v>149</v>
       </c>
-      <c r="B82" s="2" t="s">
+      <c r="I82" s="6"/>
+      <c r="J82" s="6">
+        <v>16</v>
+      </c>
+      <c r="K82" s="6">
+        <v>0</v>
+      </c>
+      <c r="L82" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="M82" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="N82" s="8"/>
+      <c r="O82" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="P82" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q82" s="6"/>
+      <c r="R82" s="8"/>
+      <c r="S82" s="6"/>
+      <c r="T82" s="8"/>
+      <c r="U82" s="6"/>
+      <c r="V82" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="W82" s="6"/>
+    </row>
+    <row r="83" spans="1:23">
+      <c r="A83" s="2" t="s">
         <v>150</v>
       </c>
-      <c r="C82" s="2">
-        <v>0</v>
-      </c>
-      <c r="D82" s="2"/>
-      <c r="E82" s="2"/>
-      <c r="F82" s="2">
-        <v>1</v>
-      </c>
-      <c r="G82" s="2">
-        <v>0</v>
-      </c>
-      <c r="H82" s="2" t="s">
+      <c r="B83" s="2" t="s">
         <v>151</v>
       </c>
-      <c r="I82" s="2"/>
-      <c r="J82" s="2">
-        <v>1</v>
-      </c>
-      <c r="K82" s="2">
-        <v>0</v>
-      </c>
-      <c r="L82" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="M82" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="N82" s="4"/>
-      <c r="O82" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="P82" s="4"/>
-      <c r="Q82" s="2"/>
-      <c r="R82" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="S82" s="2"/>
-      <c r="T82" s="4"/>
-      <c r="U82" s="2"/>
-      <c r="V82" s="2"/>
-      <c r="W82" s="2"/>
-    </row>
-    <row r="83" spans="1:23" outlineLevel="1">
-      <c r="A83" s="5" t="s">
-        <v>149</v>
-      </c>
-      <c r="B83" s="5" t="s">
-        <v>150</v>
-      </c>
-      <c r="C83" s="5">
-        <v>0</v>
-      </c>
-      <c r="D83" s="5"/>
-      <c r="E83" s="5"/>
-      <c r="F83" s="6">
-        <v>2</v>
-      </c>
-      <c r="G83" s="6">
-        <v>0</v>
-      </c>
-      <c r="H83" s="6" t="s">
+      <c r="C83" s="2">
+        <v>0</v>
+      </c>
+      <c r="D83" s="2"/>
+      <c r="E83" s="2"/>
+      <c r="F83" s="2">
+        <v>1</v>
+      </c>
+      <c r="G83" s="2">
+        <v>0</v>
+      </c>
+      <c r="H83" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="I83" s="6"/>
-      <c r="J83" s="6">
-        <v>8</v>
-      </c>
-      <c r="K83" s="6">
-        <v>0</v>
-      </c>
-      <c r="L83" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="M83" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="N83" s="8"/>
-      <c r="O83" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="P83" s="8"/>
-      <c r="Q83" s="6"/>
-      <c r="R83" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="S83" s="6"/>
-      <c r="T83" s="8"/>
-      <c r="U83" s="6"/>
-      <c r="V83" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="W83" s="6"/>
+      <c r="I83" s="2"/>
+      <c r="J83" s="2">
+        <v>1</v>
+      </c>
+      <c r="K83" s="2">
+        <v>0</v>
+      </c>
+      <c r="L83" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="M83" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="N83" s="4"/>
+      <c r="O83" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="P83" s="4"/>
+      <c r="Q83" s="2"/>
+      <c r="R83" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="S83" s="2"/>
+      <c r="T83" s="4"/>
+      <c r="U83" s="2"/>
+      <c r="V83" s="2"/>
+      <c r="W83" s="2"/>
     </row>
     <row r="84" spans="1:23" outlineLevel="1">
       <c r="A84" s="5" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B84" s="5" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C84" s="5">
         <v>0</v>
@@ -5186,7 +5191,7 @@
       <c r="D84" s="5"/>
       <c r="E84" s="5"/>
       <c r="F84" s="6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G84" s="6">
         <v>0</v>
@@ -5224,118 +5229,116 @@
       </c>
       <c r="W84" s="6"/>
     </row>
-    <row r="85" spans="1:23">
-      <c r="A85" s="2" t="s">
+    <row r="85" spans="1:23" outlineLevel="1">
+      <c r="A85" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="B85" s="5" t="s">
+        <v>151</v>
+      </c>
+      <c r="C85" s="5">
+        <v>0</v>
+      </c>
+      <c r="D85" s="5"/>
+      <c r="E85" s="5"/>
+      <c r="F85" s="6">
+        <v>3</v>
+      </c>
+      <c r="G85" s="6">
+        <v>0</v>
+      </c>
+      <c r="H85" s="6" t="s">
         <v>154</v>
       </c>
-      <c r="B85" s="2" t="s">
+      <c r="I85" s="6"/>
+      <c r="J85" s="6">
+        <v>8</v>
+      </c>
+      <c r="K85" s="6">
+        <v>0</v>
+      </c>
+      <c r="L85" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="M85" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="N85" s="8"/>
+      <c r="O85" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="P85" s="8"/>
+      <c r="Q85" s="6"/>
+      <c r="R85" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="S85" s="6"/>
+      <c r="T85" s="8"/>
+      <c r="U85" s="6"/>
+      <c r="V85" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="W85" s="6"/>
+    </row>
+    <row r="86" spans="1:23">
+      <c r="A86" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="C85" s="2">
-        <v>0</v>
-      </c>
-      <c r="D85" s="2"/>
-      <c r="E85" s="2"/>
-      <c r="F85" s="2">
-        <v>1</v>
-      </c>
-      <c r="G85" s="2">
-        <v>0</v>
-      </c>
-      <c r="H85" s="2" t="s">
+      <c r="B86" s="2" t="s">
         <v>156</v>
       </c>
-      <c r="I85" s="2"/>
-      <c r="J85" s="2">
+      <c r="C86" s="2">
+        <v>0</v>
+      </c>
+      <c r="D86" s="2"/>
+      <c r="E86" s="2"/>
+      <c r="F86" s="2">
+        <v>1</v>
+      </c>
+      <c r="G86" s="2">
+        <v>0</v>
+      </c>
+      <c r="H86" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="I86" s="2"/>
+      <c r="J86" s="2">
         <v>10</v>
       </c>
-      <c r="K85" s="2">
-        <v>1000</v>
-      </c>
-      <c r="L85" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="M85" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="N85" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="O85" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="P85" s="4"/>
-      <c r="Q85" s="2"/>
-      <c r="R85" s="4"/>
-      <c r="S85" s="2"/>
-      <c r="T85" s="4"/>
-      <c r="U85" s="2"/>
-      <c r="V85" s="2" t="s">
-        <v>128</v>
-      </c>
-      <c r="W85" s="2" t="s">
+      <c r="K86" s="2">
+        <v>0</v>
+      </c>
+      <c r="L86" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="M86" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="N86" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="O86" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="P86" s="4"/>
+      <c r="Q86" s="2"/>
+      <c r="R86" s="4"/>
+      <c r="S86" s="2"/>
+      <c r="T86" s="4"/>
+      <c r="U86" s="2"/>
+      <c r="V86" s="2" t="s">
         <v>129</v>
       </c>
-    </row>
-    <row r="86" spans="1:23" outlineLevel="1">
-      <c r="A86" s="5" t="s">
-        <v>154</v>
-      </c>
-      <c r="B86" s="5" t="s">
-        <v>155</v>
-      </c>
-      <c r="C86" s="5">
-        <v>0</v>
-      </c>
-      <c r="D86" s="5"/>
-      <c r="E86" s="5"/>
-      <c r="F86" s="6">
-        <v>2</v>
-      </c>
-      <c r="G86" s="6">
-        <v>2</v>
-      </c>
-      <c r="H86" s="6" t="s">
-        <v>157</v>
-      </c>
-      <c r="I86" s="6"/>
-      <c r="J86" s="6">
-        <v>10</v>
-      </c>
-      <c r="K86" s="6">
-        <v>1000</v>
-      </c>
-      <c r="L86" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="M86" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="N86" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="O86" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="P86" s="8"/>
-      <c r="Q86" s="6"/>
-      <c r="R86" s="8"/>
-      <c r="S86" s="6"/>
-      <c r="T86" s="8"/>
-      <c r="U86" s="6"/>
-      <c r="V86" s="6" t="s">
-        <v>128</v>
-      </c>
-      <c r="W86" s="6" t="s">
-        <v>129</v>
+      <c r="W86" s="2" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="87" spans="1:23" outlineLevel="1">
       <c r="A87" s="5" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B87" s="5" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C87" s="5">
         <v>0</v>
@@ -5343,10 +5346,10 @@
       <c r="D87" s="5"/>
       <c r="E87" s="5"/>
       <c r="F87" s="6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G87" s="6">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H87" s="6" t="s">
         <v>158</v>
@@ -5356,7 +5359,7 @@
         <v>10</v>
       </c>
       <c r="K87" s="6">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="L87" s="6" t="s">
         <v>28</v>
@@ -5377,18 +5380,18 @@
       <c r="T87" s="8"/>
       <c r="U87" s="6"/>
       <c r="V87" s="6" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="W87" s="6" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="88" spans="1:23" outlineLevel="1">
       <c r="A88" s="5" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B88" s="5" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C88" s="5">
         <v>0</v>
@@ -5396,10 +5399,10 @@
       <c r="D88" s="5"/>
       <c r="E88" s="5"/>
       <c r="F88" s="6">
+        <v>3</v>
+      </c>
+      <c r="G88" s="6">
         <v>4</v>
-      </c>
-      <c r="G88" s="6">
-        <v>6</v>
       </c>
       <c r="H88" s="6" t="s">
         <v>159</v>
@@ -5409,7 +5412,7 @@
         <v>10</v>
       </c>
       <c r="K88" s="6">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="L88" s="6" t="s">
         <v>28</v>
@@ -5430,18 +5433,18 @@
       <c r="T88" s="8"/>
       <c r="U88" s="6"/>
       <c r="V88" s="6" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="W88" s="6" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="89" spans="1:23" outlineLevel="1">
       <c r="A89" s="5" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B89" s="5" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C89" s="5">
         <v>0</v>
@@ -5449,10 +5452,10 @@
       <c r="D89" s="5"/>
       <c r="E89" s="5"/>
       <c r="F89" s="6">
+        <v>4</v>
+      </c>
+      <c r="G89" s="6">
         <v>6</v>
-      </c>
-      <c r="G89" s="6">
-        <v>0</v>
       </c>
       <c r="H89" s="6" t="s">
         <v>160</v>
@@ -5462,7 +5465,7 @@
         <v>10</v>
       </c>
       <c r="K89" s="6">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="L89" s="6" t="s">
         <v>28</v>
@@ -5483,18 +5486,18 @@
       <c r="T89" s="8"/>
       <c r="U89" s="6"/>
       <c r="V89" s="6" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="W89" s="6" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="90" spans="1:23" outlineLevel="1">
       <c r="A90" s="5" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B90" s="5" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C90" s="5">
         <v>0</v>
@@ -5502,10 +5505,10 @@
       <c r="D90" s="5"/>
       <c r="E90" s="5"/>
       <c r="F90" s="6">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G90" s="6">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H90" s="6" t="s">
         <v>161</v>
@@ -5515,7 +5518,7 @@
         <v>10</v>
       </c>
       <c r="K90" s="6">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="L90" s="6" t="s">
         <v>28</v>
@@ -5536,124 +5539,124 @@
       <c r="T90" s="8"/>
       <c r="U90" s="6"/>
       <c r="V90" s="6" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="W90" s="6" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="91" spans="1:23" outlineLevel="1">
+      <c r="A91" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="B91" s="5" t="s">
+        <v>156</v>
+      </c>
+      <c r="C91" s="5">
+        <v>0</v>
+      </c>
+      <c r="D91" s="5"/>
+      <c r="E91" s="5"/>
+      <c r="F91" s="6">
+        <v>7</v>
+      </c>
+      <c r="G91" s="6">
+        <v>2</v>
+      </c>
+      <c r="H91" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="I91" s="6"/>
+      <c r="J91" s="6">
+        <v>10</v>
+      </c>
+      <c r="K91" s="6">
+        <v>0</v>
+      </c>
+      <c r="L91" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="M91" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="N91" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="O91" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="P91" s="8"/>
+      <c r="Q91" s="6"/>
+      <c r="R91" s="8"/>
+      <c r="S91" s="6"/>
+      <c r="T91" s="8"/>
+      <c r="U91" s="6"/>
+      <c r="V91" s="6" t="s">
         <v>129</v>
       </c>
-    </row>
-    <row r="91" spans="1:23">
-      <c r="A91" s="2" t="s">
-        <v>162</v>
-      </c>
-      <c r="B91" s="2" t="s">
+      <c r="W91" s="6" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="92" spans="1:23">
+      <c r="A92" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="C91" s="2">
-        <v>0</v>
-      </c>
-      <c r="D91" s="2"/>
-      <c r="E91" s="2"/>
-      <c r="F91" s="2">
-        <v>1</v>
-      </c>
-      <c r="G91" s="2">
-        <v>0</v>
-      </c>
-      <c r="H91" s="2" t="s">
-        <v>156</v>
-      </c>
-      <c r="I91" s="2"/>
-      <c r="J91" s="2">
+      <c r="B92" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="C92" s="2">
+        <v>0</v>
+      </c>
+      <c r="D92" s="2"/>
+      <c r="E92" s="2"/>
+      <c r="F92" s="2">
+        <v>1</v>
+      </c>
+      <c r="G92" s="2">
+        <v>0</v>
+      </c>
+      <c r="H92" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="I92" s="2"/>
+      <c r="J92" s="2">
         <v>10</v>
       </c>
-      <c r="K91" s="2">
-        <v>1000</v>
-      </c>
-      <c r="L91" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="M91" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="N91" s="4"/>
-      <c r="O91" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="P91" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q91" s="2"/>
-      <c r="R91" s="4"/>
-      <c r="S91" s="2"/>
-      <c r="T91" s="4"/>
-      <c r="U91" s="2"/>
-      <c r="V91" s="2" t="s">
-        <v>128</v>
-      </c>
-      <c r="W91" s="2" t="s">
+      <c r="K92" s="2">
+        <v>0</v>
+      </c>
+      <c r="L92" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="M92" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="N92" s="4"/>
+      <c r="O92" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="P92" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q92" s="2"/>
+      <c r="R92" s="4"/>
+      <c r="S92" s="2"/>
+      <c r="T92" s="4"/>
+      <c r="U92" s="2"/>
+      <c r="V92" s="2" t="s">
         <v>129</v>
       </c>
-    </row>
-    <row r="92" spans="1:23" outlineLevel="1">
-      <c r="A92" s="5" t="s">
-        <v>162</v>
-      </c>
-      <c r="B92" s="5" t="s">
-        <v>163</v>
-      </c>
-      <c r="C92" s="5">
-        <v>0</v>
-      </c>
-      <c r="D92" s="5"/>
-      <c r="E92" s="5"/>
-      <c r="F92" s="6">
-        <v>2</v>
-      </c>
-      <c r="G92" s="6">
-        <v>2</v>
-      </c>
-      <c r="H92" s="6" t="s">
-        <v>157</v>
-      </c>
-      <c r="I92" s="6"/>
-      <c r="J92" s="6">
-        <v>10</v>
-      </c>
-      <c r="K92" s="6">
-        <v>1000</v>
-      </c>
-      <c r="L92" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="M92" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="N92" s="8"/>
-      <c r="O92" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="P92" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q92" s="6"/>
-      <c r="R92" s="8"/>
-      <c r="S92" s="6"/>
-      <c r="T92" s="8"/>
-      <c r="U92" s="6"/>
-      <c r="V92" s="6" t="s">
-        <v>128</v>
-      </c>
-      <c r="W92" s="6" t="s">
-        <v>129</v>
+      <c r="W92" s="2" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="93" spans="1:23" outlineLevel="1">
       <c r="A93" s="5" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B93" s="5" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C93" s="5">
         <v>0</v>
@@ -5661,10 +5664,10 @@
       <c r="D93" s="5"/>
       <c r="E93" s="5"/>
       <c r="F93" s="6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G93" s="6">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H93" s="6" t="s">
         <v>158</v>
@@ -5674,7 +5677,7 @@
         <v>10</v>
       </c>
       <c r="K93" s="6">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="L93" s="6" t="s">
         <v>28</v>
@@ -5695,18 +5698,18 @@
       <c r="T93" s="8"/>
       <c r="U93" s="6"/>
       <c r="V93" s="6" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="W93" s="6" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="94" spans="1:23" outlineLevel="1">
       <c r="A94" s="5" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B94" s="5" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C94" s="5">
         <v>0</v>
@@ -5714,10 +5717,10 @@
       <c r="D94" s="5"/>
       <c r="E94" s="5"/>
       <c r="F94" s="6">
+        <v>3</v>
+      </c>
+      <c r="G94" s="6">
         <v>4</v>
-      </c>
-      <c r="G94" s="6">
-        <v>6</v>
       </c>
       <c r="H94" s="6" t="s">
         <v>159</v>
@@ -5727,7 +5730,7 @@
         <v>10</v>
       </c>
       <c r="K94" s="6">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="L94" s="6" t="s">
         <v>28</v>
@@ -5748,18 +5751,18 @@
       <c r="T94" s="8"/>
       <c r="U94" s="6"/>
       <c r="V94" s="6" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="W94" s="6" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="95" spans="1:23" outlineLevel="1">
       <c r="A95" s="5" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B95" s="5" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C95" s="5">
         <v>0</v>
@@ -5767,20 +5770,20 @@
       <c r="D95" s="5"/>
       <c r="E95" s="5"/>
       <c r="F95" s="6">
+        <v>4</v>
+      </c>
+      <c r="G95" s="6">
         <v>6</v>
       </c>
-      <c r="G95" s="6">
-        <v>0</v>
-      </c>
       <c r="H95" s="6" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="I95" s="6"/>
       <c r="J95" s="6">
         <v>10</v>
       </c>
       <c r="K95" s="6">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="L95" s="6" t="s">
         <v>28</v>
@@ -5801,18 +5804,18 @@
       <c r="T95" s="8"/>
       <c r="U95" s="6"/>
       <c r="V95" s="6" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="W95" s="6" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="96" spans="1:23" outlineLevel="1">
       <c r="A96" s="5" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B96" s="5" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C96" s="5">
         <v>0</v>
@@ -5820,10 +5823,10 @@
       <c r="D96" s="5"/>
       <c r="E96" s="5"/>
       <c r="F96" s="6">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G96" s="6">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H96" s="6" t="s">
         <v>165</v>
@@ -5833,7 +5836,7 @@
         <v>10</v>
       </c>
       <c r="K96" s="6">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="L96" s="6" t="s">
         <v>28</v>
@@ -5854,218 +5857,222 @@
       <c r="T96" s="8"/>
       <c r="U96" s="6"/>
       <c r="V96" s="6" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="W96" s="6" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="97" spans="1:23" outlineLevel="1">
+      <c r="A97" s="5" t="s">
+        <v>163</v>
+      </c>
+      <c r="B97" s="5" t="s">
+        <v>164</v>
+      </c>
+      <c r="C97" s="5">
+        <v>0</v>
+      </c>
+      <c r="D97" s="5"/>
+      <c r="E97" s="5"/>
+      <c r="F97" s="6">
+        <v>7</v>
+      </c>
+      <c r="G97" s="6">
+        <v>2</v>
+      </c>
+      <c r="H97" s="6" t="s">
+        <v>166</v>
+      </c>
+      <c r="I97" s="6"/>
+      <c r="J97" s="6">
+        <v>10</v>
+      </c>
+      <c r="K97" s="6">
+        <v>0</v>
+      </c>
+      <c r="L97" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="M97" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="N97" s="8"/>
+      <c r="O97" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="P97" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q97" s="6"/>
+      <c r="R97" s="8"/>
+      <c r="S97" s="6"/>
+      <c r="T97" s="8"/>
+      <c r="U97" s="6"/>
+      <c r="V97" s="6" t="s">
         <v>129</v>
       </c>
-    </row>
-    <row r="97" spans="1:23">
-      <c r="A97" s="2" t="s">
-        <v>166</v>
-      </c>
-      <c r="B97" s="2" t="s">
+      <c r="W97" s="6" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="98" spans="1:23">
+      <c r="A98" s="2" t="s">
         <v>167</v>
       </c>
-      <c r="C97" s="2">
-        <v>0</v>
-      </c>
-      <c r="D97" s="2"/>
-      <c r="E97" s="2"/>
-      <c r="F97" s="2">
-        <v>1</v>
-      </c>
-      <c r="G97" s="2">
-        <v>0</v>
-      </c>
-      <c r="H97" s="2" t="s">
+      <c r="B98" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="I97" s="2"/>
-      <c r="J97" s="2">
+      <c r="C98" s="2">
+        <v>0</v>
+      </c>
+      <c r="D98" s="2"/>
+      <c r="E98" s="2"/>
+      <c r="F98" s="2">
+        <v>1</v>
+      </c>
+      <c r="G98" s="2">
+        <v>0</v>
+      </c>
+      <c r="H98" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="I98" s="2"/>
+      <c r="J98" s="2">
         <v>16</v>
       </c>
-      <c r="K97" s="2">
-        <v>0</v>
-      </c>
-      <c r="L97" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="M97" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="N97" s="4"/>
-      <c r="O97" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="P97" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q97" s="2"/>
-      <c r="R97" s="4"/>
-      <c r="S97" s="2"/>
-      <c r="T97" s="4"/>
-      <c r="U97" s="2"/>
-      <c r="V97" s="2" t="s">
+      <c r="K98" s="2">
+        <v>0</v>
+      </c>
+      <c r="L98" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="M98" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="N98" s="4"/>
+      <c r="O98" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="P98" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q98" s="2"/>
+      <c r="R98" s="4"/>
+      <c r="S98" s="2"/>
+      <c r="T98" s="4"/>
+      <c r="U98" s="2"/>
+      <c r="V98" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="W97" s="2"/>
-    </row>
-    <row r="98" spans="1:23" outlineLevel="1">
-      <c r="A98" s="5" t="s">
-        <v>166</v>
-      </c>
-      <c r="B98" s="5" t="s">
+      <c r="W98" s="2"/>
+    </row>
+    <row r="99" spans="1:23" outlineLevel="1">
+      <c r="A99" s="5" t="s">
         <v>167</v>
       </c>
-      <c r="C98" s="5">
-        <v>0</v>
-      </c>
-      <c r="D98" s="5"/>
-      <c r="E98" s="5"/>
-      <c r="F98" s="6">
+      <c r="B99" s="5" t="s">
+        <v>168</v>
+      </c>
+      <c r="C99" s="5">
+        <v>0</v>
+      </c>
+      <c r="D99" s="5"/>
+      <c r="E99" s="5"/>
+      <c r="F99" s="6">
         <v>3</v>
       </c>
-      <c r="G98" s="6">
-        <v>0</v>
-      </c>
-      <c r="H98" s="6" t="s">
-        <v>169</v>
-      </c>
-      <c r="I98" s="6"/>
-      <c r="J98" s="6">
+      <c r="G99" s="6">
+        <v>0</v>
+      </c>
+      <c r="H99" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="I99" s="6"/>
+      <c r="J99" s="6">
         <v>16</v>
       </c>
-      <c r="K98" s="6">
-        <v>0</v>
-      </c>
-      <c r="L98" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="M98" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="N98" s="8"/>
-      <c r="O98" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="P98" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q98" s="6"/>
-      <c r="R98" s="8"/>
-      <c r="S98" s="6"/>
-      <c r="T98" s="8"/>
-      <c r="U98" s="6"/>
-      <c r="V98" s="6" t="s">
+      <c r="K99" s="6">
+        <v>0</v>
+      </c>
+      <c r="L99" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="M99" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="N99" s="8"/>
+      <c r="O99" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="P99" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q99" s="6"/>
+      <c r="R99" s="8"/>
+      <c r="S99" s="6"/>
+      <c r="T99" s="8"/>
+      <c r="U99" s="6"/>
+      <c r="V99" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="W98" s="6"/>
-    </row>
-    <row r="99" spans="1:23">
-      <c r="A99" s="2" t="s">
-        <v>170</v>
-      </c>
-      <c r="B99" s="2" t="s">
+      <c r="W99" s="6"/>
+    </row>
+    <row r="100" spans="1:23">
+      <c r="A100" s="2" t="s">
         <v>171</v>
       </c>
-      <c r="C99" s="2">
-        <v>0</v>
-      </c>
-      <c r="D99" s="2"/>
-      <c r="E99" s="2"/>
-      <c r="F99" s="2">
-        <v>1</v>
-      </c>
-      <c r="G99" s="2">
-        <v>0</v>
-      </c>
-      <c r="H99" s="2" t="s">
+      <c r="B100" s="2" t="s">
         <v>172</v>
       </c>
-      <c r="I99" s="2"/>
-      <c r="J99" s="2">
-        <v>1</v>
-      </c>
-      <c r="K99" s="2">
-        <v>0</v>
-      </c>
-      <c r="L99" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="M99" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="N99" s="4"/>
-      <c r="O99" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="P99" s="4"/>
-      <c r="Q99" s="2"/>
-      <c r="R99" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="S99" s="2"/>
-      <c r="T99" s="4"/>
-      <c r="U99" s="2"/>
-      <c r="V99" s="2"/>
-      <c r="W99" s="2"/>
-    </row>
-    <row r="100" spans="1:23" outlineLevel="1">
-      <c r="A100" s="5" t="s">
-        <v>170</v>
-      </c>
-      <c r="B100" s="5" t="s">
-        <v>171</v>
-      </c>
-      <c r="C100" s="5">
-        <v>0</v>
-      </c>
-      <c r="D100" s="5"/>
-      <c r="E100" s="5"/>
-      <c r="F100" s="6">
-        <v>1</v>
-      </c>
-      <c r="G100" s="6">
-        <v>1</v>
-      </c>
-      <c r="H100" s="6" t="s">
+      <c r="C100" s="2">
+        <v>0</v>
+      </c>
+      <c r="D100" s="2"/>
+      <c r="E100" s="2"/>
+      <c r="F100" s="2">
+        <v>1</v>
+      </c>
+      <c r="G100" s="2">
+        <v>0</v>
+      </c>
+      <c r="H100" s="2" t="s">
         <v>173</v>
       </c>
-      <c r="I100" s="6"/>
-      <c r="J100" s="6">
-        <v>1</v>
-      </c>
-      <c r="K100" s="6">
-        <v>0</v>
-      </c>
-      <c r="L100" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="M100" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="N100" s="8"/>
-      <c r="O100" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="P100" s="8"/>
-      <c r="Q100" s="6"/>
-      <c r="R100" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="S100" s="6"/>
-      <c r="T100" s="8"/>
-      <c r="U100" s="6"/>
-      <c r="V100" s="6"/>
-      <c r="W100" s="6"/>
+      <c r="I100" s="2"/>
+      <c r="J100" s="2">
+        <v>1</v>
+      </c>
+      <c r="K100" s="2">
+        <v>0</v>
+      </c>
+      <c r="L100" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="M100" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="N100" s="4"/>
+      <c r="O100" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="P100" s="4"/>
+      <c r="Q100" s="2"/>
+      <c r="R100" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="S100" s="2"/>
+      <c r="T100" s="4"/>
+      <c r="U100" s="2"/>
+      <c r="V100" s="2"/>
+      <c r="W100" s="2"/>
     </row>
     <row r="101" spans="1:23" outlineLevel="1">
       <c r="A101" s="5" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B101" s="5" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C101" s="5">
         <v>0</v>
@@ -6076,7 +6083,7 @@
         <v>1</v>
       </c>
       <c r="G101" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H101" s="6" t="s">
         <v>174</v>
@@ -6111,10 +6118,10 @@
     </row>
     <row r="102" spans="1:23" outlineLevel="1">
       <c r="A102" s="5" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B102" s="5" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C102" s="5">
         <v>0</v>
@@ -6125,7 +6132,7 @@
         <v>1</v>
       </c>
       <c r="G102" s="6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H102" s="6" t="s">
         <v>175</v>
@@ -6158,8 +6165,57 @@
       <c r="V102" s="6"/>
       <c r="W102" s="6"/>
     </row>
+    <row r="103" spans="1:23" outlineLevel="1">
+      <c r="A103" s="5" t="s">
+        <v>171</v>
+      </c>
+      <c r="B103" s="5" t="s">
+        <v>172</v>
+      </c>
+      <c r="C103" s="5">
+        <v>0</v>
+      </c>
+      <c r="D103" s="5"/>
+      <c r="E103" s="5"/>
+      <c r="F103" s="6">
+        <v>1</v>
+      </c>
+      <c r="G103" s="6">
+        <v>3</v>
+      </c>
+      <c r="H103" s="6" t="s">
+        <v>176</v>
+      </c>
+      <c r="I103" s="6"/>
+      <c r="J103" s="6">
+        <v>1</v>
+      </c>
+      <c r="K103" s="6">
+        <v>0</v>
+      </c>
+      <c r="L103" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="M103" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="N103" s="8"/>
+      <c r="O103" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="P103" s="8"/>
+      <c r="Q103" s="6"/>
+      <c r="R103" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="S103" s="6"/>
+      <c r="T103" s="8"/>
+      <c r="U103" s="6"/>
+      <c r="V103" s="6"/>
+      <c r="W103" s="6"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AH103"/>
+  <autoFilter ref="A1:AH104"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
generated from SC22EVO/MCB.json at 230988d
</commit_message>
<xml_diff>
--- a/SC22EVO/artifacts/MCB.xlsx
+++ b/SC22EVO/artifacts/MCB.xlsx
@@ -10,14 +10,14 @@
     <sheet name="K-Matrix " sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'K-Matrix '!$A$1:$AH$104</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'K-Matrix '!$A$1:$AH$110</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="835" uniqueCount="177">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="883" uniqueCount="191">
   <si>
     <t>ID</t>
   </si>
@@ -70,15 +70,15 @@
     <t>tlb_bat</t>
   </si>
   <si>
+    <t>bms_lv</t>
+  </si>
+  <si>
     <t>dash</t>
   </si>
   <si>
     <t>bmslv</t>
   </si>
   <si>
-    <t>bms_lv</t>
-  </si>
-  <si>
     <t>Value</t>
   </si>
   <si>
@@ -245,6 +245,48 @@
   </si>
   <si>
     <t>Imp_isAnyImp_Latched</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 14h</t>
+  </si>
+  <si>
+    <t>BMSLV_Helo</t>
+  </si>
+  <si>
+    <t>time</t>
+  </si>
+  <si>
+    <t>0..1.84467e+19</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 15h</t>
+  </si>
+  <si>
+    <t>Sens_Front_Helo</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 16h</t>
+  </si>
+  <si>
+    <t>Sens_Rear_Helo</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 17h</t>
+  </si>
+  <si>
+    <t>Steering_Helo</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 18h</t>
+  </si>
+  <si>
+    <t>TLB_Battery_Helo</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 19h</t>
+  </si>
+  <si>
+    <t>dSpaxe_Helo</t>
   </si>
   <si>
     <t xml:space="preserve"> 25h</t>
@@ -936,7 +978,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W103"/>
+  <dimension ref="A1:W109"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="1"/>
   <cols>
     <col min="1" max="1" width="4.28515625" customWidth="1"/>
@@ -2835,7 +2877,7 @@
       </c>
       <c r="I38" s="2"/>
       <c r="J38" s="2">
-        <v>8</v>
+        <v>64</v>
       </c>
       <c r="K38" s="2">
         <v>0</v>
@@ -2847,13 +2889,13 @@
         <v>29</v>
       </c>
       <c r="N38" s="4"/>
-      <c r="O38" s="9" t="s">
-        <v>25</v>
+      <c r="O38" s="2" t="s">
+        <v>26</v>
       </c>
       <c r="P38" s="4"/>
       <c r="Q38" s="2"/>
-      <c r="R38" s="4" t="s">
-        <v>26</v>
+      <c r="R38" s="3" t="s">
+        <v>25</v>
       </c>
       <c r="S38" s="2"/>
       <c r="T38" s="4"/>
@@ -2882,11 +2924,11 @@
         <v>0</v>
       </c>
       <c r="H39" s="2" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="I39" s="2"/>
       <c r="J39" s="2">
-        <v>8</v>
+        <v>64</v>
       </c>
       <c r="K39" s="2">
         <v>0</v>
@@ -2910,16 +2952,16 @@
       <c r="T39" s="4"/>
       <c r="U39" s="2"/>
       <c r="V39" s="2" t="s">
-        <v>54</v>
+        <v>79</v>
       </c>
       <c r="W39" s="2"/>
     </row>
     <row r="40" spans="1:23">
       <c r="A40" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B40" s="2" t="s">
         <v>83</v>
-      </c>
-      <c r="B40" s="2" t="s">
-        <v>84</v>
       </c>
       <c r="C40" s="2">
         <v>0</v>
@@ -2933,11 +2975,11 @@
         <v>0</v>
       </c>
       <c r="H40" s="2" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="I40" s="2"/>
       <c r="J40" s="2">
-        <v>1</v>
+        <v>64</v>
       </c>
       <c r="K40" s="2">
         <v>0</v>
@@ -2952,219 +2994,229 @@
       <c r="O40" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="P40" s="3" t="s">
-        <v>25</v>
-      </c>
+      <c r="P40" s="4"/>
       <c r="Q40" s="2"/>
-      <c r="R40" s="4"/>
+      <c r="R40" s="3" t="s">
+        <v>25</v>
+      </c>
       <c r="S40" s="2"/>
       <c r="T40" s="4"/>
       <c r="U40" s="2"/>
-      <c r="V40" s="2"/>
+      <c r="V40" s="2" t="s">
+        <v>79</v>
+      </c>
       <c r="W40" s="2"/>
     </row>
-    <row r="41" spans="1:23" outlineLevel="1">
-      <c r="A41" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="B41" s="5" t="s">
+    <row r="41" spans="1:23">
+      <c r="A41" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="C41" s="5">
-        <v>0</v>
-      </c>
-      <c r="D41" s="5"/>
-      <c r="E41" s="5"/>
-      <c r="F41" s="6">
-        <v>1</v>
-      </c>
-      <c r="G41" s="6">
-        <v>1</v>
-      </c>
-      <c r="H41" s="6" t="s">
+      <c r="B41" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="C41" s="2">
+        <v>0</v>
+      </c>
+      <c r="D41" s="2"/>
+      <c r="E41" s="2"/>
+      <c r="F41" s="2">
+        <v>1</v>
+      </c>
+      <c r="G41" s="2">
+        <v>0</v>
+      </c>
+      <c r="H41" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="I41" s="2"/>
+      <c r="J41" s="2">
+        <v>64</v>
+      </c>
+      <c r="K41" s="2">
+        <v>0</v>
+      </c>
+      <c r="L41" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="M41" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="N41" s="4"/>
+      <c r="O41" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="P41" s="4"/>
+      <c r="Q41" s="2"/>
+      <c r="R41" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="S41" s="2"/>
+      <c r="T41" s="4"/>
+      <c r="U41" s="2"/>
+      <c r="V41" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="W41" s="2"/>
+    </row>
+    <row r="42" spans="1:23">
+      <c r="A42" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="I41" s="6"/>
-      <c r="J41" s="6">
-        <v>1</v>
-      </c>
-      <c r="K41" s="6">
-        <v>0</v>
-      </c>
-      <c r="L41" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="M41" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="N41" s="8"/>
-      <c r="O41" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="P41" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q41" s="6"/>
-      <c r="R41" s="8"/>
-      <c r="S41" s="6"/>
-      <c r="T41" s="8"/>
-      <c r="U41" s="6"/>
-      <c r="V41" s="6"/>
-      <c r="W41" s="6"/>
-    </row>
-    <row r="42" spans="1:23" outlineLevel="1">
-      <c r="A42" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="B42" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="C42" s="5">
-        <v>0</v>
-      </c>
-      <c r="D42" s="5"/>
-      <c r="E42" s="5"/>
-      <c r="F42" s="6">
-        <v>1</v>
-      </c>
-      <c r="G42" s="6">
-        <v>2</v>
-      </c>
-      <c r="H42" s="6" t="s">
+      <c r="B42" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="I42" s="6"/>
-      <c r="J42" s="6">
-        <v>1</v>
-      </c>
-      <c r="K42" s="6">
-        <v>0</v>
-      </c>
-      <c r="L42" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="M42" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="N42" s="8"/>
-      <c r="O42" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="P42" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q42" s="6"/>
-      <c r="R42" s="8"/>
-      <c r="S42" s="6"/>
-      <c r="T42" s="8"/>
-      <c r="U42" s="6"/>
-      <c r="V42" s="6"/>
-      <c r="W42" s="6"/>
-    </row>
-    <row r="43" spans="1:23" outlineLevel="1">
-      <c r="A43" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="B43" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="C43" s="5">
-        <v>0</v>
-      </c>
-      <c r="D43" s="5"/>
-      <c r="E43" s="5"/>
-      <c r="F43" s="6">
-        <v>1</v>
-      </c>
-      <c r="G43" s="6">
-        <v>3</v>
-      </c>
-      <c r="H43" s="6" t="s">
+      <c r="C42" s="2">
+        <v>0</v>
+      </c>
+      <c r="D42" s="2"/>
+      <c r="E42" s="2"/>
+      <c r="F42" s="2">
+        <v>1</v>
+      </c>
+      <c r="G42" s="2">
+        <v>0</v>
+      </c>
+      <c r="H42" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="I42" s="2"/>
+      <c r="J42" s="2">
+        <v>64</v>
+      </c>
+      <c r="K42" s="2">
+        <v>0</v>
+      </c>
+      <c r="L42" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="M42" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="N42" s="4"/>
+      <c r="O42" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="P42" s="4"/>
+      <c r="Q42" s="2"/>
+      <c r="R42" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="S42" s="2"/>
+      <c r="T42" s="4"/>
+      <c r="U42" s="2"/>
+      <c r="V42" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="W42" s="2"/>
+    </row>
+    <row r="43" spans="1:23">
+      <c r="A43" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="I43" s="6"/>
-      <c r="J43" s="6">
-        <v>1</v>
-      </c>
-      <c r="K43" s="6">
-        <v>0</v>
-      </c>
-      <c r="L43" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="M43" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="N43" s="8"/>
-      <c r="O43" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="P43" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q43" s="6"/>
-      <c r="R43" s="8"/>
-      <c r="S43" s="6"/>
-      <c r="T43" s="8"/>
-      <c r="U43" s="6"/>
-      <c r="V43" s="6"/>
-      <c r="W43" s="6"/>
-    </row>
-    <row r="44" spans="1:23" outlineLevel="1">
-      <c r="A44" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="B44" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="C44" s="5">
-        <v>0</v>
-      </c>
-      <c r="D44" s="5"/>
-      <c r="E44" s="5"/>
-      <c r="F44" s="6">
-        <v>1</v>
-      </c>
-      <c r="G44" s="6">
-        <v>4</v>
-      </c>
-      <c r="H44" s="6" t="s">
+      <c r="B43" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="I44" s="6"/>
-      <c r="J44" s="6">
-        <v>1</v>
-      </c>
-      <c r="K44" s="6">
-        <v>0</v>
-      </c>
-      <c r="L44" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="M44" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="N44" s="8"/>
-      <c r="O44" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="P44" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q44" s="6"/>
-      <c r="R44" s="8"/>
-      <c r="S44" s="6"/>
-      <c r="T44" s="8"/>
-      <c r="U44" s="6"/>
-      <c r="V44" s="6"/>
-      <c r="W44" s="6"/>
+      <c r="C43" s="2">
+        <v>0</v>
+      </c>
+      <c r="D43" s="2"/>
+      <c r="E43" s="2"/>
+      <c r="F43" s="2">
+        <v>1</v>
+      </c>
+      <c r="G43" s="2">
+        <v>0</v>
+      </c>
+      <c r="H43" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="I43" s="2"/>
+      <c r="J43" s="2">
+        <v>64</v>
+      </c>
+      <c r="K43" s="2">
+        <v>0</v>
+      </c>
+      <c r="L43" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="M43" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="N43" s="4"/>
+      <c r="O43" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="P43" s="4"/>
+      <c r="Q43" s="2"/>
+      <c r="R43" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="S43" s="2"/>
+      <c r="T43" s="4"/>
+      <c r="U43" s="2"/>
+      <c r="V43" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="W43" s="2"/>
+    </row>
+    <row r="44" spans="1:23">
+      <c r="A44" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="C44" s="2">
+        <v>0</v>
+      </c>
+      <c r="D44" s="2"/>
+      <c r="E44" s="2"/>
+      <c r="F44" s="2">
+        <v>1</v>
+      </c>
+      <c r="G44" s="2">
+        <v>0</v>
+      </c>
+      <c r="H44" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="I44" s="2"/>
+      <c r="J44" s="2">
+        <v>8</v>
+      </c>
+      <c r="K44" s="2">
+        <v>0</v>
+      </c>
+      <c r="L44" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="M44" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="N44" s="4"/>
+      <c r="O44" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="P44" s="4"/>
+      <c r="Q44" s="2"/>
+      <c r="R44" s="4"/>
+      <c r="S44" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="T44" s="4"/>
+      <c r="U44" s="2"/>
+      <c r="V44" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="W44" s="2"/>
     </row>
     <row r="45" spans="1:23">
       <c r="A45" s="2" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="C45" s="2">
         <v>0</v>
@@ -3178,11 +3230,11 @@
         <v>0</v>
       </c>
       <c r="H45" s="2" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="I45" s="2"/>
       <c r="J45" s="2">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="K45" s="2">
         <v>0</v>
@@ -3193,76 +3245,78 @@
       <c r="M45" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="N45" s="3" t="s">
-        <v>25</v>
-      </c>
+      <c r="N45" s="4"/>
       <c r="O45" s="2" t="s">
         <v>26</v>
       </c>
       <c r="P45" s="4"/>
       <c r="Q45" s="2"/>
       <c r="R45" s="4"/>
-      <c r="S45" s="2"/>
+      <c r="S45" s="9" t="s">
+        <v>25</v>
+      </c>
       <c r="T45" s="4"/>
       <c r="U45" s="2"/>
-      <c r="V45" s="2"/>
+      <c r="V45" s="2" t="s">
+        <v>54</v>
+      </c>
       <c r="W45" s="2"/>
     </row>
-    <row r="46" spans="1:23" outlineLevel="1">
-      <c r="A46" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="B46" s="5" t="s">
-        <v>91</v>
-      </c>
-      <c r="C46" s="5">
-        <v>0</v>
-      </c>
-      <c r="D46" s="5"/>
-      <c r="E46" s="5"/>
-      <c r="F46" s="6">
-        <v>1</v>
-      </c>
-      <c r="G46" s="6">
-        <v>1</v>
-      </c>
-      <c r="H46" s="6" t="s">
-        <v>93</v>
-      </c>
-      <c r="I46" s="6"/>
-      <c r="J46" s="6">
-        <v>1</v>
-      </c>
-      <c r="K46" s="6">
-        <v>0</v>
-      </c>
-      <c r="L46" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="M46" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="N46" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="O46" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="P46" s="8"/>
-      <c r="Q46" s="6"/>
-      <c r="R46" s="8"/>
-      <c r="S46" s="6"/>
-      <c r="T46" s="8"/>
-      <c r="U46" s="6"/>
-      <c r="V46" s="6"/>
-      <c r="W46" s="6"/>
+    <row r="46" spans="1:23">
+      <c r="A46" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="C46" s="2">
+        <v>0</v>
+      </c>
+      <c r="D46" s="2"/>
+      <c r="E46" s="2"/>
+      <c r="F46" s="2">
+        <v>1</v>
+      </c>
+      <c r="G46" s="2">
+        <v>0</v>
+      </c>
+      <c r="H46" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="I46" s="2"/>
+      <c r="J46" s="2">
+        <v>1</v>
+      </c>
+      <c r="K46" s="2">
+        <v>0</v>
+      </c>
+      <c r="L46" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="M46" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="N46" s="4"/>
+      <c r="O46" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="P46" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q46" s="2"/>
+      <c r="R46" s="4"/>
+      <c r="S46" s="2"/>
+      <c r="T46" s="4"/>
+      <c r="U46" s="2"/>
+      <c r="V46" s="2"/>
+      <c r="W46" s="2"/>
     </row>
     <row r="47" spans="1:23" outlineLevel="1">
       <c r="A47" s="5" t="s">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="B47" s="5" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="C47" s="5">
         <v>0</v>
@@ -3273,10 +3327,10 @@
         <v>1</v>
       </c>
       <c r="G47" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H47" s="6" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="I47" s="6"/>
       <c r="J47" s="6">
@@ -3291,13 +3345,13 @@
       <c r="M47" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="N47" s="7" t="s">
-        <v>25</v>
-      </c>
+      <c r="N47" s="8"/>
       <c r="O47" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="P47" s="8"/>
+      <c r="P47" s="7" t="s">
+        <v>25</v>
+      </c>
       <c r="Q47" s="6"/>
       <c r="R47" s="8"/>
       <c r="S47" s="6"/>
@@ -3308,10 +3362,10 @@
     </row>
     <row r="48" spans="1:23" outlineLevel="1">
       <c r="A48" s="5" t="s">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="B48" s="5" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="C48" s="5">
         <v>0</v>
@@ -3322,10 +3376,10 @@
         <v>1</v>
       </c>
       <c r="G48" s="6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H48" s="6" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="I48" s="6"/>
       <c r="J48" s="6">
@@ -3340,13 +3394,13 @@
       <c r="M48" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="N48" s="7" t="s">
-        <v>25</v>
-      </c>
+      <c r="N48" s="8"/>
       <c r="O48" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="P48" s="8"/>
+      <c r="P48" s="7" t="s">
+        <v>25</v>
+      </c>
       <c r="Q48" s="6"/>
       <c r="R48" s="8"/>
       <c r="S48" s="6"/>
@@ -3355,63 +3409,61 @@
       <c r="V48" s="6"/>
       <c r="W48" s="6"/>
     </row>
-    <row r="49" spans="1:23">
-      <c r="A49" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="B49" s="2" t="s">
+    <row r="49" spans="1:23" outlineLevel="1">
+      <c r="A49" s="5" t="s">
         <v>97</v>
       </c>
-      <c r="C49" s="2">
-        <v>0</v>
-      </c>
-      <c r="D49" s="2"/>
-      <c r="E49" s="2"/>
-      <c r="F49" s="2">
-        <v>1</v>
-      </c>
-      <c r="G49" s="2">
-        <v>0</v>
-      </c>
-      <c r="H49" s="2" t="s">
+      <c r="B49" s="5" t="s">
         <v>98</v>
       </c>
-      <c r="I49" s="2"/>
-      <c r="J49" s="2">
-        <v>15</v>
-      </c>
-      <c r="K49" s="2">
-        <v>0</v>
-      </c>
-      <c r="L49" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="M49" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="N49" s="4"/>
-      <c r="O49" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="P49" s="4"/>
-      <c r="Q49" s="2"/>
-      <c r="R49" s="4"/>
-      <c r="S49" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="T49" s="4"/>
-      <c r="U49" s="2"/>
-      <c r="V49" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="W49" s="2"/>
+      <c r="C49" s="5">
+        <v>0</v>
+      </c>
+      <c r="D49" s="5"/>
+      <c r="E49" s="5"/>
+      <c r="F49" s="6">
+        <v>1</v>
+      </c>
+      <c r="G49" s="6">
+        <v>3</v>
+      </c>
+      <c r="H49" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="I49" s="6"/>
+      <c r="J49" s="6">
+        <v>1</v>
+      </c>
+      <c r="K49" s="6">
+        <v>0</v>
+      </c>
+      <c r="L49" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="M49" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="N49" s="8"/>
+      <c r="O49" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="P49" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q49" s="6"/>
+      <c r="R49" s="8"/>
+      <c r="S49" s="6"/>
+      <c r="T49" s="8"/>
+      <c r="U49" s="6"/>
+      <c r="V49" s="6"/>
+      <c r="W49" s="6"/>
     </row>
     <row r="50" spans="1:23" outlineLevel="1">
       <c r="A50" s="5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B50" s="5" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C50" s="5">
         <v>0</v>
@@ -3419,13 +3471,13 @@
       <c r="D50" s="5"/>
       <c r="E50" s="5"/>
       <c r="F50" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G50" s="6">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="H50" s="6" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="I50" s="6"/>
       <c r="J50" s="6">
@@ -3441,15 +3493,15 @@
         <v>29</v>
       </c>
       <c r="N50" s="8"/>
-      <c r="O50" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="P50" s="8"/>
+      <c r="O50" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="P50" s="7" t="s">
+        <v>25</v>
+      </c>
       <c r="Q50" s="6"/>
       <c r="R50" s="8"/>
-      <c r="S50" s="6" t="s">
-        <v>26</v>
-      </c>
+      <c r="S50" s="6"/>
       <c r="T50" s="8"/>
       <c r="U50" s="6"/>
       <c r="V50" s="6"/>
@@ -3457,10 +3509,10 @@
     </row>
     <row r="51" spans="1:23">
       <c r="A51" s="2" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="C51" s="2">
         <v>0</v>
@@ -3474,14 +3526,14 @@
         <v>0</v>
       </c>
       <c r="H51" s="2" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="I51" s="2"/>
       <c r="J51" s="2">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="K51" s="2">
-        <v>-0.016</v>
+        <v>0</v>
       </c>
       <c r="L51" s="2" t="s">
         <v>28</v>
@@ -3489,7 +3541,9 @@
       <c r="M51" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="N51" s="4"/>
+      <c r="N51" s="3" t="s">
+        <v>25</v>
+      </c>
       <c r="O51" s="2" t="s">
         <v>26</v>
       </c>
@@ -3497,23 +3551,17 @@
       <c r="Q51" s="2"/>
       <c r="R51" s="4"/>
       <c r="S51" s="2"/>
-      <c r="T51" s="3" t="s">
-        <v>25</v>
-      </c>
+      <c r="T51" s="4"/>
       <c r="U51" s="2"/>
-      <c r="V51" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="W51" s="2" t="s">
-        <v>104</v>
-      </c>
+      <c r="V51" s="2"/>
+      <c r="W51" s="2"/>
     </row>
     <row r="52" spans="1:23" outlineLevel="1">
       <c r="A52" s="5" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="B52" s="5" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="C52" s="5">
         <v>0</v>
@@ -3521,20 +3569,20 @@
       <c r="D52" s="5"/>
       <c r="E52" s="5"/>
       <c r="F52" s="6">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G52" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H52" s="6" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="I52" s="6"/>
       <c r="J52" s="6">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="K52" s="6">
-        <v>-0.016</v>
+        <v>0</v>
       </c>
       <c r="L52" s="6" t="s">
         <v>28</v>
@@ -3542,7 +3590,9 @@
       <c r="M52" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="N52" s="8"/>
+      <c r="N52" s="7" t="s">
+        <v>25</v>
+      </c>
       <c r="O52" s="6" t="s">
         <v>26</v>
       </c>
@@ -3550,23 +3600,17 @@
       <c r="Q52" s="6"/>
       <c r="R52" s="8"/>
       <c r="S52" s="6"/>
-      <c r="T52" s="7" t="s">
-        <v>25</v>
-      </c>
+      <c r="T52" s="8"/>
       <c r="U52" s="6"/>
-      <c r="V52" s="6" t="s">
-        <v>103</v>
-      </c>
-      <c r="W52" s="6" t="s">
-        <v>104</v>
-      </c>
+      <c r="V52" s="6"/>
+      <c r="W52" s="6"/>
     </row>
     <row r="53" spans="1:23" outlineLevel="1">
       <c r="A53" s="5" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="B53" s="5" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="C53" s="5">
         <v>0</v>
@@ -3574,20 +3618,20 @@
       <c r="D53" s="5"/>
       <c r="E53" s="5"/>
       <c r="F53" s="6">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G53" s="6">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H53" s="6" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="I53" s="6"/>
       <c r="J53" s="6">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="K53" s="6">
-        <v>-0.016</v>
+        <v>0</v>
       </c>
       <c r="L53" s="6" t="s">
         <v>28</v>
@@ -3595,7 +3639,9 @@
       <c r="M53" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="N53" s="8"/>
+      <c r="N53" s="7" t="s">
+        <v>25</v>
+      </c>
       <c r="O53" s="6" t="s">
         <v>26</v>
       </c>
@@ -3603,23 +3649,17 @@
       <c r="Q53" s="6"/>
       <c r="R53" s="8"/>
       <c r="S53" s="6"/>
-      <c r="T53" s="7" t="s">
-        <v>25</v>
-      </c>
+      <c r="T53" s="8"/>
       <c r="U53" s="6"/>
-      <c r="V53" s="6" t="s">
-        <v>103</v>
-      </c>
-      <c r="W53" s="6" t="s">
-        <v>104</v>
-      </c>
+      <c r="V53" s="6"/>
+      <c r="W53" s="6"/>
     </row>
     <row r="54" spans="1:23" outlineLevel="1">
       <c r="A54" s="5" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="B54" s="5" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="C54" s="5">
         <v>0</v>
@@ -3627,20 +3667,20 @@
       <c r="D54" s="5"/>
       <c r="E54" s="5"/>
       <c r="F54" s="6">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="G54" s="6">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H54" s="6" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="I54" s="6"/>
       <c r="J54" s="6">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="K54" s="6">
-        <v>-0.016</v>
+        <v>0</v>
       </c>
       <c r="L54" s="6" t="s">
         <v>28</v>
@@ -3648,7 +3688,9 @@
       <c r="M54" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="N54" s="8"/>
+      <c r="N54" s="7" t="s">
+        <v>25</v>
+      </c>
       <c r="O54" s="6" t="s">
         <v>26</v>
       </c>
@@ -3656,23 +3698,17 @@
       <c r="Q54" s="6"/>
       <c r="R54" s="8"/>
       <c r="S54" s="6"/>
-      <c r="T54" s="7" t="s">
-        <v>25</v>
-      </c>
+      <c r="T54" s="8"/>
       <c r="U54" s="6"/>
-      <c r="V54" s="6" t="s">
-        <v>103</v>
-      </c>
-      <c r="W54" s="6" t="s">
-        <v>104</v>
-      </c>
+      <c r="V54" s="6"/>
+      <c r="W54" s="6"/>
     </row>
     <row r="55" spans="1:23">
       <c r="A55" s="2" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C55" s="2">
         <v>0</v>
@@ -3686,14 +3722,14 @@
         <v>0</v>
       </c>
       <c r="H55" s="2" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="I55" s="2"/>
       <c r="J55" s="2">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="K55" s="2">
-        <v>-0.016</v>
+        <v>0</v>
       </c>
       <c r="L55" s="2" t="s">
         <v>28</v>
@@ -3702,30 +3738,28 @@
         <v>29</v>
       </c>
       <c r="N55" s="4"/>
-      <c r="O55" s="2" t="s">
-        <v>26</v>
+      <c r="O55" s="9" t="s">
+        <v>25</v>
       </c>
       <c r="P55" s="4"/>
       <c r="Q55" s="2"/>
       <c r="R55" s="4"/>
       <c r="S55" s="2"/>
-      <c r="T55" s="3" t="s">
-        <v>25</v>
+      <c r="T55" s="4" t="s">
+        <v>26</v>
       </c>
       <c r="U55" s="2"/>
       <c r="V55" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="W55" s="2" t="s">
-        <v>104</v>
-      </c>
+        <v>30</v>
+      </c>
+      <c r="W55" s="2"/>
     </row>
     <row r="56" spans="1:23" outlineLevel="1">
       <c r="A56" s="5" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B56" s="5" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C56" s="5">
         <v>0</v>
@@ -3733,20 +3767,20 @@
       <c r="D56" s="5"/>
       <c r="E56" s="5"/>
       <c r="F56" s="6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G56" s="6">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="H56" s="6" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="I56" s="6"/>
       <c r="J56" s="6">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="K56" s="6">
-        <v>-0.016</v>
+        <v>0</v>
       </c>
       <c r="L56" s="6" t="s">
         <v>28</v>
@@ -3755,136 +3789,132 @@
         <v>29</v>
       </c>
       <c r="N56" s="8"/>
-      <c r="O56" s="6" t="s">
-        <v>26</v>
+      <c r="O56" s="10" t="s">
+        <v>25</v>
       </c>
       <c r="P56" s="8"/>
       <c r="Q56" s="6"/>
       <c r="R56" s="8"/>
       <c r="S56" s="6"/>
-      <c r="T56" s="7" t="s">
-        <v>25</v>
+      <c r="T56" s="8" t="s">
+        <v>26</v>
       </c>
       <c r="U56" s="6"/>
-      <c r="V56" s="6" t="s">
-        <v>103</v>
-      </c>
-      <c r="W56" s="6" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="57" spans="1:23" outlineLevel="1">
-      <c r="A57" s="5" t="s">
-        <v>108</v>
-      </c>
-      <c r="B57" s="5" t="s">
-        <v>109</v>
-      </c>
-      <c r="C57" s="5">
-        <v>0</v>
-      </c>
-      <c r="D57" s="5"/>
-      <c r="E57" s="5"/>
-      <c r="F57" s="6">
-        <v>5</v>
-      </c>
-      <c r="G57" s="6">
-        <v>0</v>
-      </c>
-      <c r="H57" s="6" t="s">
-        <v>112</v>
-      </c>
-      <c r="I57" s="6"/>
-      <c r="J57" s="6">
+      <c r="V56" s="6"/>
+      <c r="W56" s="6"/>
+    </row>
+    <row r="57" spans="1:23">
+      <c r="A57" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="B57" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="C57" s="2">
+        <v>0</v>
+      </c>
+      <c r="D57" s="2"/>
+      <c r="E57" s="2"/>
+      <c r="F57" s="2">
+        <v>1</v>
+      </c>
+      <c r="G57" s="2">
+        <v>0</v>
+      </c>
+      <c r="H57" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="I57" s="2"/>
+      <c r="J57" s="2">
         <v>16</v>
       </c>
-      <c r="K57" s="6">
+      <c r="K57" s="2">
         <v>-0.016</v>
       </c>
-      <c r="L57" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="M57" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="N57" s="8"/>
-      <c r="O57" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="P57" s="8"/>
-      <c r="Q57" s="6"/>
-      <c r="R57" s="8"/>
-      <c r="S57" s="6"/>
-      <c r="T57" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="U57" s="6"/>
-      <c r="V57" s="6" t="s">
-        <v>103</v>
-      </c>
-      <c r="W57" s="6" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="58" spans="1:23">
-      <c r="A58" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="B58" s="2" t="s">
+      <c r="L57" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="M57" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="N57" s="4"/>
+      <c r="O57" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="P57" s="4"/>
+      <c r="Q57" s="2"/>
+      <c r="R57" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="S57" s="2"/>
+      <c r="T57" s="4"/>
+      <c r="U57" s="2"/>
+      <c r="V57" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="W57" s="2" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="58" spans="1:23" outlineLevel="1">
+      <c r="A58" s="5" t="s">
         <v>114</v>
       </c>
-      <c r="C58" s="2">
-        <v>0</v>
-      </c>
-      <c r="D58" s="2"/>
-      <c r="E58" s="2"/>
-      <c r="F58" s="2">
-        <v>1</v>
-      </c>
-      <c r="G58" s="2">
-        <v>0</v>
-      </c>
-      <c r="H58" s="2" t="s">
+      <c r="B58" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="I58" s="2"/>
-      <c r="J58" s="2">
+      <c r="C58" s="5">
+        <v>0</v>
+      </c>
+      <c r="D58" s="5"/>
+      <c r="E58" s="5"/>
+      <c r="F58" s="6">
+        <v>3</v>
+      </c>
+      <c r="G58" s="6">
+        <v>0</v>
+      </c>
+      <c r="H58" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="I58" s="6"/>
+      <c r="J58" s="6">
         <v>16</v>
       </c>
-      <c r="K58" s="2">
-        <v>0</v>
-      </c>
-      <c r="L58" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="M58" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="N58" s="4"/>
-      <c r="O58" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="P58" s="4"/>
-      <c r="Q58" s="2"/>
-      <c r="R58" s="4"/>
-      <c r="S58" s="2"/>
-      <c r="T58" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="U58" s="2"/>
-      <c r="V58" s="2" t="s">
-        <v>116</v>
-      </c>
-      <c r="W58" s="2" t="s">
+      <c r="K58" s="6">
+        <v>-0.016</v>
+      </c>
+      <c r="L58" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="M58" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="N58" s="8"/>
+      <c r="O58" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="P58" s="8"/>
+      <c r="Q58" s="6"/>
+      <c r="R58" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="S58" s="6"/>
+      <c r="T58" s="8"/>
+      <c r="U58" s="6"/>
+      <c r="V58" s="6" t="s">
         <v>117</v>
+      </c>
+      <c r="W58" s="6" t="s">
+        <v>118</v>
       </c>
     </row>
     <row r="59" spans="1:23" outlineLevel="1">
       <c r="A59" s="5" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B59" s="5" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C59" s="5">
         <v>0</v>
@@ -3892,20 +3922,20 @@
       <c r="D59" s="5"/>
       <c r="E59" s="5"/>
       <c r="F59" s="6">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G59" s="6">
         <v>0</v>
       </c>
       <c r="H59" s="6" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="I59" s="6"/>
       <c r="J59" s="6">
         <v>16</v>
       </c>
       <c r="K59" s="6">
-        <v>0.122</v>
+        <v>-0.016</v>
       </c>
       <c r="L59" s="6" t="s">
         <v>28</v>
@@ -3919,25 +3949,25 @@
       </c>
       <c r="P59" s="8"/>
       <c r="Q59" s="6"/>
-      <c r="R59" s="8"/>
+      <c r="R59" s="7" t="s">
+        <v>25</v>
+      </c>
       <c r="S59" s="6"/>
-      <c r="T59" s="7" t="s">
-        <v>25</v>
-      </c>
+      <c r="T59" s="8"/>
       <c r="U59" s="6"/>
       <c r="V59" s="6" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="W59" s="6" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
     </row>
     <row r="60" spans="1:23" outlineLevel="1">
       <c r="A60" s="5" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B60" s="5" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C60" s="5">
         <v>0</v>
@@ -3945,7 +3975,7 @@
       <c r="D60" s="5"/>
       <c r="E60" s="5"/>
       <c r="F60" s="6">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G60" s="6">
         <v>0</v>
@@ -3958,7 +3988,7 @@
         <v>16</v>
       </c>
       <c r="K60" s="6">
-        <v>0.122</v>
+        <v>-0.016</v>
       </c>
       <c r="L60" s="6" t="s">
         <v>28</v>
@@ -3972,17 +4002,17 @@
       </c>
       <c r="P60" s="8"/>
       <c r="Q60" s="6"/>
-      <c r="R60" s="8"/>
+      <c r="R60" s="7" t="s">
+        <v>25</v>
+      </c>
       <c r="S60" s="6"/>
-      <c r="T60" s="7" t="s">
-        <v>25</v>
-      </c>
+      <c r="T60" s="8"/>
       <c r="U60" s="6"/>
       <c r="V60" s="6" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="W60" s="6" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
     </row>
     <row r="61" spans="1:23">
@@ -4008,10 +4038,10 @@
       </c>
       <c r="I61" s="2"/>
       <c r="J61" s="2">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="K61" s="2">
-        <v>0</v>
+        <v>-0.016</v>
       </c>
       <c r="L61" s="2" t="s">
         <v>28</v>
@@ -4025,14 +4055,18 @@
       </c>
       <c r="P61" s="4"/>
       <c r="Q61" s="2"/>
-      <c r="R61" s="4"/>
+      <c r="R61" s="3" t="s">
+        <v>25</v>
+      </c>
       <c r="S61" s="2"/>
-      <c r="T61" s="3" t="s">
-        <v>25</v>
-      </c>
+      <c r="T61" s="4"/>
       <c r="U61" s="2"/>
-      <c r="V61" s="2"/>
-      <c r="W61" s="2"/>
+      <c r="V61" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="W61" s="2" t="s">
+        <v>118</v>
+      </c>
     </row>
     <row r="62" spans="1:23" outlineLevel="1">
       <c r="A62" s="5" t="s">
@@ -4047,20 +4081,20 @@
       <c r="D62" s="5"/>
       <c r="E62" s="5"/>
       <c r="F62" s="6">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G62" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H62" s="6" t="s">
         <v>125</v>
       </c>
       <c r="I62" s="6"/>
       <c r="J62" s="6">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="K62" s="6">
-        <v>0</v>
+        <v>-0.016</v>
       </c>
       <c r="L62" s="6" t="s">
         <v>28</v>
@@ -4074,129 +4108,131 @@
       </c>
       <c r="P62" s="8"/>
       <c r="Q62" s="6"/>
-      <c r="R62" s="8"/>
+      <c r="R62" s="7" t="s">
+        <v>25</v>
+      </c>
       <c r="S62" s="6"/>
-      <c r="T62" s="7" t="s">
-        <v>25</v>
-      </c>
+      <c r="T62" s="8"/>
       <c r="U62" s="6"/>
       <c r="V62" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="W62" s="6"/>
-    </row>
-    <row r="63" spans="1:23">
-      <c r="A63" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="W62" s="6" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="63" spans="1:23" outlineLevel="1">
+      <c r="A63" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="B63" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="C63" s="5">
+        <v>0</v>
+      </c>
+      <c r="D63" s="5"/>
+      <c r="E63" s="5"/>
+      <c r="F63" s="6">
+        <v>5</v>
+      </c>
+      <c r="G63" s="6">
+        <v>0</v>
+      </c>
+      <c r="H63" s="6" t="s">
         <v>126</v>
       </c>
-      <c r="B63" s="2" t="s">
+      <c r="I63" s="6"/>
+      <c r="J63" s="6">
+        <v>16</v>
+      </c>
+      <c r="K63" s="6">
+        <v>-0.016</v>
+      </c>
+      <c r="L63" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="M63" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="N63" s="8"/>
+      <c r="O63" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="P63" s="8"/>
+      <c r="Q63" s="6"/>
+      <c r="R63" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="S63" s="6"/>
+      <c r="T63" s="8"/>
+      <c r="U63" s="6"/>
+      <c r="V63" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="W63" s="6" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="64" spans="1:23">
+      <c r="A64" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="C63" s="2">
-        <v>0</v>
-      </c>
-      <c r="D63" s="2"/>
-      <c r="E63" s="2"/>
-      <c r="F63" s="2">
-        <v>1</v>
-      </c>
-      <c r="G63" s="2">
-        <v>1</v>
-      </c>
-      <c r="H63" s="2" t="s">
+      <c r="B64" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="I63" s="2"/>
-      <c r="J63" s="2">
-        <v>10</v>
-      </c>
-      <c r="K63" s="2">
-        <v>0</v>
-      </c>
-      <c r="L63" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="M63" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="N63" s="4"/>
-      <c r="O63" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="P63" s="4"/>
-      <c r="Q63" s="2"/>
-      <c r="R63" s="4"/>
-      <c r="S63" s="2"/>
-      <c r="T63" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="U63" s="2"/>
-      <c r="V63" s="2" t="s">
+      <c r="C64" s="2">
+        <v>0</v>
+      </c>
+      <c r="D64" s="2"/>
+      <c r="E64" s="2"/>
+      <c r="F64" s="2">
+        <v>1</v>
+      </c>
+      <c r="G64" s="2">
+        <v>0</v>
+      </c>
+      <c r="H64" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="W63" s="2" t="s">
+      <c r="I64" s="2"/>
+      <c r="J64" s="2">
+        <v>16</v>
+      </c>
+      <c r="K64" s="2">
+        <v>0</v>
+      </c>
+      <c r="L64" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="M64" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="N64" s="4"/>
+      <c r="O64" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="P64" s="4"/>
+      <c r="Q64" s="2"/>
+      <c r="R64" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="S64" s="2"/>
+      <c r="T64" s="4"/>
+      <c r="U64" s="2"/>
+      <c r="V64" s="2" t="s">
         <v>130</v>
       </c>
-    </row>
-    <row r="64" spans="1:23" outlineLevel="1">
-      <c r="A64" s="5" t="s">
-        <v>126</v>
-      </c>
-      <c r="B64" s="5" t="s">
-        <v>127</v>
-      </c>
-      <c r="C64" s="5">
-        <v>0</v>
-      </c>
-      <c r="D64" s="5"/>
-      <c r="E64" s="5"/>
-      <c r="F64" s="6">
-        <v>2</v>
-      </c>
-      <c r="G64" s="6">
-        <v>3</v>
-      </c>
-      <c r="H64" s="6" t="s">
+      <c r="W64" s="2" t="s">
         <v>131</v>
-      </c>
-      <c r="I64" s="6"/>
-      <c r="J64" s="6">
-        <v>10</v>
-      </c>
-      <c r="K64" s="6">
-        <v>0</v>
-      </c>
-      <c r="L64" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="M64" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="N64" s="8"/>
-      <c r="O64" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="P64" s="8"/>
-      <c r="Q64" s="6"/>
-      <c r="R64" s="8"/>
-      <c r="S64" s="6"/>
-      <c r="T64" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="U64" s="6"/>
-      <c r="V64" s="6" t="s">
-        <v>129</v>
-      </c>
-      <c r="W64" s="6" t="s">
-        <v>130</v>
       </c>
     </row>
     <row r="65" spans="1:23" outlineLevel="1">
       <c r="A65" s="5" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B65" s="5" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C65" s="5">
         <v>0</v>
@@ -4207,17 +4243,17 @@
         <v>3</v>
       </c>
       <c r="G65" s="6">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="H65" s="6" t="s">
         <v>132</v>
       </c>
       <c r="I65" s="6"/>
       <c r="J65" s="6">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="K65" s="6">
-        <v>0</v>
+        <v>0.122</v>
       </c>
       <c r="L65" s="6" t="s">
         <v>28</v>
@@ -4231,25 +4267,25 @@
       </c>
       <c r="P65" s="8"/>
       <c r="Q65" s="6"/>
-      <c r="R65" s="8"/>
+      <c r="R65" s="7" t="s">
+        <v>25</v>
+      </c>
       <c r="S65" s="6"/>
-      <c r="T65" s="7" t="s">
-        <v>25</v>
-      </c>
+      <c r="T65" s="8"/>
       <c r="U65" s="6"/>
       <c r="V65" s="6" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="W65" s="6" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
     </row>
     <row r="66" spans="1:23" outlineLevel="1">
       <c r="A66" s="5" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B66" s="5" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C66" s="5">
         <v>0</v>
@@ -4257,20 +4293,20 @@
       <c r="D66" s="5"/>
       <c r="E66" s="5"/>
       <c r="F66" s="6">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G66" s="6">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="H66" s="6" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="I66" s="6"/>
       <c r="J66" s="6">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="K66" s="6">
-        <v>0</v>
+        <v>0.122</v>
       </c>
       <c r="L66" s="6" t="s">
         <v>28</v>
@@ -4284,78 +4320,74 @@
       </c>
       <c r="P66" s="8"/>
       <c r="Q66" s="6"/>
-      <c r="R66" s="8"/>
+      <c r="R66" s="7" t="s">
+        <v>25</v>
+      </c>
       <c r="S66" s="6"/>
-      <c r="T66" s="7" t="s">
-        <v>25</v>
-      </c>
+      <c r="T66" s="8"/>
       <c r="U66" s="6"/>
       <c r="V66" s="6" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="W66" s="6" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="67" spans="1:23" outlineLevel="1">
-      <c r="A67" s="5" t="s">
-        <v>126</v>
-      </c>
-      <c r="B67" s="5" t="s">
-        <v>127</v>
-      </c>
-      <c r="C67" s="5">
-        <v>0</v>
-      </c>
-      <c r="D67" s="5"/>
-      <c r="E67" s="5"/>
-      <c r="F67" s="6">
-        <v>6</v>
-      </c>
-      <c r="G67" s="6">
-        <v>1</v>
-      </c>
-      <c r="H67" s="6" t="s">
         <v>134</v>
       </c>
-      <c r="I67" s="6"/>
-      <c r="J67" s="6">
-        <v>10</v>
-      </c>
-      <c r="K67" s="6">
-        <v>0</v>
-      </c>
-      <c r="L67" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="M67" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="N67" s="8"/>
-      <c r="O67" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="P67" s="8"/>
-      <c r="Q67" s="6"/>
-      <c r="R67" s="8"/>
-      <c r="S67" s="6"/>
-      <c r="T67" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="U67" s="6"/>
-      <c r="V67" s="6" t="s">
-        <v>129</v>
-      </c>
-      <c r="W67" s="6" t="s">
-        <v>130</v>
-      </c>
+    </row>
+    <row r="67" spans="1:23">
+      <c r="A67" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="B67" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="C67" s="2">
+        <v>0</v>
+      </c>
+      <c r="D67" s="2"/>
+      <c r="E67" s="2"/>
+      <c r="F67" s="2">
+        <v>1</v>
+      </c>
+      <c r="G67" s="2">
+        <v>0</v>
+      </c>
+      <c r="H67" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="I67" s="2"/>
+      <c r="J67" s="2">
+        <v>1</v>
+      </c>
+      <c r="K67" s="2">
+        <v>0</v>
+      </c>
+      <c r="L67" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="M67" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="N67" s="4"/>
+      <c r="O67" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="P67" s="4"/>
+      <c r="Q67" s="2"/>
+      <c r="R67" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="S67" s="2"/>
+      <c r="T67" s="4"/>
+      <c r="U67" s="2"/>
+      <c r="V67" s="2"/>
+      <c r="W67" s="2"/>
     </row>
     <row r="68" spans="1:23" outlineLevel="1">
       <c r="A68" s="5" t="s">
-        <v>126</v>
+        <v>136</v>
       </c>
       <c r="B68" s="5" t="s">
-        <v>127</v>
+        <v>137</v>
       </c>
       <c r="C68" s="5">
         <v>0</v>
@@ -4363,17 +4395,17 @@
       <c r="D68" s="5"/>
       <c r="E68" s="5"/>
       <c r="F68" s="6">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="G68" s="6">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="H68" s="6" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="I68" s="6"/>
       <c r="J68" s="6">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="K68" s="6">
         <v>0</v>
@@ -4390,25 +4422,23 @@
       </c>
       <c r="P68" s="8"/>
       <c r="Q68" s="6"/>
-      <c r="R68" s="8"/>
+      <c r="R68" s="7" t="s">
+        <v>25</v>
+      </c>
       <c r="S68" s="6"/>
-      <c r="T68" s="7" t="s">
-        <v>25</v>
-      </c>
+      <c r="T68" s="8"/>
       <c r="U68" s="6"/>
       <c r="V68" s="6" t="s">
-        <v>129</v>
-      </c>
-      <c r="W68" s="6" t="s">
-        <v>130</v>
-      </c>
+        <v>54</v>
+      </c>
+      <c r="W68" s="6"/>
     </row>
     <row r="69" spans="1:23">
       <c r="A69" s="2" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="C69" s="2">
         <v>0</v>
@@ -4422,7 +4452,7 @@
         <v>1</v>
       </c>
       <c r="H69" s="2" t="s">
-        <v>128</v>
+        <v>142</v>
       </c>
       <c r="I69" s="2"/>
       <c r="J69" s="2">
@@ -4443,25 +4473,25 @@
       </c>
       <c r="P69" s="4"/>
       <c r="Q69" s="2"/>
-      <c r="R69" s="4"/>
+      <c r="R69" s="3" t="s">
+        <v>25</v>
+      </c>
       <c r="S69" s="2"/>
-      <c r="T69" s="3" t="s">
-        <v>25</v>
-      </c>
+      <c r="T69" s="4"/>
       <c r="U69" s="2"/>
       <c r="V69" s="2" t="s">
-        <v>129</v>
+        <v>143</v>
       </c>
       <c r="W69" s="2" t="s">
-        <v>130</v>
+        <v>144</v>
       </c>
     </row>
     <row r="70" spans="1:23" outlineLevel="1">
       <c r="A70" s="5" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="B70" s="5" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="C70" s="5">
         <v>0</v>
@@ -4475,7 +4505,7 @@
         <v>3</v>
       </c>
       <c r="H70" s="6" t="s">
-        <v>131</v>
+        <v>145</v>
       </c>
       <c r="I70" s="6"/>
       <c r="J70" s="6">
@@ -4496,25 +4526,25 @@
       </c>
       <c r="P70" s="8"/>
       <c r="Q70" s="6"/>
-      <c r="R70" s="8"/>
+      <c r="R70" s="7" t="s">
+        <v>25</v>
+      </c>
       <c r="S70" s="6"/>
-      <c r="T70" s="7" t="s">
-        <v>25</v>
-      </c>
+      <c r="T70" s="8"/>
       <c r="U70" s="6"/>
       <c r="V70" s="6" t="s">
-        <v>129</v>
+        <v>143</v>
       </c>
       <c r="W70" s="6" t="s">
-        <v>130</v>
+        <v>144</v>
       </c>
     </row>
     <row r="71" spans="1:23" outlineLevel="1">
       <c r="A71" s="5" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="B71" s="5" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="C71" s="5">
         <v>0</v>
@@ -4528,7 +4558,7 @@
         <v>5</v>
       </c>
       <c r="H71" s="6" t="s">
-        <v>132</v>
+        <v>146</v>
       </c>
       <c r="I71" s="6"/>
       <c r="J71" s="6">
@@ -4549,25 +4579,25 @@
       </c>
       <c r="P71" s="8"/>
       <c r="Q71" s="6"/>
-      <c r="R71" s="8"/>
+      <c r="R71" s="7" t="s">
+        <v>25</v>
+      </c>
       <c r="S71" s="6"/>
-      <c r="T71" s="7" t="s">
-        <v>25</v>
-      </c>
+      <c r="T71" s="8"/>
       <c r="U71" s="6"/>
       <c r="V71" s="6" t="s">
-        <v>129</v>
+        <v>143</v>
       </c>
       <c r="W71" s="6" t="s">
-        <v>130</v>
+        <v>144</v>
       </c>
     </row>
     <row r="72" spans="1:23" outlineLevel="1">
       <c r="A72" s="5" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="B72" s="5" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="C72" s="5">
         <v>0</v>
@@ -4581,7 +4611,7 @@
         <v>7</v>
       </c>
       <c r="H72" s="6" t="s">
-        <v>133</v>
+        <v>147</v>
       </c>
       <c r="I72" s="6"/>
       <c r="J72" s="6">
@@ -4602,25 +4632,25 @@
       </c>
       <c r="P72" s="8"/>
       <c r="Q72" s="6"/>
-      <c r="R72" s="8"/>
+      <c r="R72" s="7" t="s">
+        <v>25</v>
+      </c>
       <c r="S72" s="6"/>
-      <c r="T72" s="7" t="s">
-        <v>25</v>
-      </c>
+      <c r="T72" s="8"/>
       <c r="U72" s="6"/>
       <c r="V72" s="6" t="s">
-        <v>129</v>
+        <v>143</v>
       </c>
       <c r="W72" s="6" t="s">
-        <v>130</v>
+        <v>144</v>
       </c>
     </row>
     <row r="73" spans="1:23" outlineLevel="1">
       <c r="A73" s="5" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="B73" s="5" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="C73" s="5">
         <v>0</v>
@@ -4634,7 +4664,7 @@
         <v>1</v>
       </c>
       <c r="H73" s="6" t="s">
-        <v>134</v>
+        <v>148</v>
       </c>
       <c r="I73" s="6"/>
       <c r="J73" s="6">
@@ -4655,25 +4685,25 @@
       </c>
       <c r="P73" s="8"/>
       <c r="Q73" s="6"/>
-      <c r="R73" s="8"/>
+      <c r="R73" s="7" t="s">
+        <v>25</v>
+      </c>
       <c r="S73" s="6"/>
-      <c r="T73" s="7" t="s">
-        <v>25</v>
-      </c>
+      <c r="T73" s="8"/>
       <c r="U73" s="6"/>
       <c r="V73" s="6" t="s">
-        <v>129</v>
+        <v>143</v>
       </c>
       <c r="W73" s="6" t="s">
-        <v>130</v>
+        <v>144</v>
       </c>
     </row>
     <row r="74" spans="1:23" outlineLevel="1">
       <c r="A74" s="5" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="B74" s="5" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="C74" s="5">
         <v>0</v>
@@ -4687,7 +4717,7 @@
         <v>6</v>
       </c>
       <c r="H74" s="6" t="s">
-        <v>135</v>
+        <v>149</v>
       </c>
       <c r="I74" s="6"/>
       <c r="J74" s="6">
@@ -4708,25 +4738,25 @@
       </c>
       <c r="P74" s="8"/>
       <c r="Q74" s="6"/>
-      <c r="R74" s="8"/>
+      <c r="R74" s="7" t="s">
+        <v>25</v>
+      </c>
       <c r="S74" s="6"/>
-      <c r="T74" s="7" t="s">
-        <v>25</v>
-      </c>
+      <c r="T74" s="8"/>
       <c r="U74" s="6"/>
       <c r="V74" s="6" t="s">
-        <v>129</v>
+        <v>143</v>
       </c>
       <c r="W74" s="6" t="s">
-        <v>130</v>
+        <v>144</v>
       </c>
     </row>
     <row r="75" spans="1:23">
       <c r="A75" s="2" t="s">
-        <v>138</v>
+        <v>150</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>139</v>
+        <v>151</v>
       </c>
       <c r="C75" s="2">
         <v>0</v>
@@ -4737,14 +4767,14 @@
         <v>1</v>
       </c>
       <c r="G75" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H75" s="2" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="I75" s="2"/>
       <c r="J75" s="2">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="K75" s="2">
         <v>0</v>
@@ -4755,29 +4785,31 @@
       <c r="M75" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="N75" s="3" t="s">
-        <v>25</v>
-      </c>
+      <c r="N75" s="4"/>
       <c r="O75" s="2" t="s">
         <v>26</v>
       </c>
       <c r="P75" s="4"/>
       <c r="Q75" s="2"/>
-      <c r="R75" s="4"/>
+      <c r="R75" s="3" t="s">
+        <v>25</v>
+      </c>
       <c r="S75" s="2"/>
       <c r="T75" s="4"/>
       <c r="U75" s="2"/>
       <c r="V75" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="W75" s="2"/>
+        <v>143</v>
+      </c>
+      <c r="W75" s="2" t="s">
+        <v>144</v>
+      </c>
     </row>
     <row r="76" spans="1:23" outlineLevel="1">
       <c r="A76" s="5" t="s">
-        <v>138</v>
+        <v>150</v>
       </c>
       <c r="B76" s="5" t="s">
-        <v>139</v>
+        <v>151</v>
       </c>
       <c r="C76" s="5">
         <v>0</v>
@@ -4785,17 +4817,17 @@
       <c r="D76" s="5"/>
       <c r="E76" s="5"/>
       <c r="F76" s="6">
+        <v>2</v>
+      </c>
+      <c r="G76" s="6">
         <v>3</v>
       </c>
-      <c r="G76" s="6">
-        <v>0</v>
-      </c>
       <c r="H76" s="6" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="I76" s="6"/>
       <c r="J76" s="6">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="K76" s="6">
         <v>0</v>
@@ -4806,29 +4838,31 @@
       <c r="M76" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="N76" s="7" t="s">
-        <v>25</v>
-      </c>
+      <c r="N76" s="8"/>
       <c r="O76" s="6" t="s">
         <v>26</v>
       </c>
       <c r="P76" s="8"/>
       <c r="Q76" s="6"/>
-      <c r="R76" s="8"/>
+      <c r="R76" s="7" t="s">
+        <v>25</v>
+      </c>
       <c r="S76" s="6"/>
       <c r="T76" s="8"/>
       <c r="U76" s="6"/>
       <c r="V76" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="W76" s="6"/>
+        <v>143</v>
+      </c>
+      <c r="W76" s="6" t="s">
+        <v>144</v>
+      </c>
     </row>
     <row r="77" spans="1:23" outlineLevel="1">
       <c r="A77" s="5" t="s">
-        <v>138</v>
+        <v>150</v>
       </c>
       <c r="B77" s="5" t="s">
-        <v>139</v>
+        <v>151</v>
       </c>
       <c r="C77" s="5">
         <v>0</v>
@@ -4836,17 +4870,17 @@
       <c r="D77" s="5"/>
       <c r="E77" s="5"/>
       <c r="F77" s="6">
+        <v>3</v>
+      </c>
+      <c r="G77" s="6">
         <v>5</v>
       </c>
-      <c r="G77" s="6">
-        <v>0</v>
-      </c>
       <c r="H77" s="6" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="I77" s="6"/>
       <c r="J77" s="6">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="K77" s="6">
         <v>0</v>
@@ -4857,29 +4891,31 @@
       <c r="M77" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="N77" s="7" t="s">
-        <v>25</v>
-      </c>
+      <c r="N77" s="8"/>
       <c r="O77" s="6" t="s">
         <v>26</v>
       </c>
       <c r="P77" s="8"/>
       <c r="Q77" s="6"/>
-      <c r="R77" s="8"/>
+      <c r="R77" s="7" t="s">
+        <v>25</v>
+      </c>
       <c r="S77" s="6"/>
       <c r="T77" s="8"/>
       <c r="U77" s="6"/>
       <c r="V77" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="W77" s="6"/>
+        <v>143</v>
+      </c>
+      <c r="W77" s="6" t="s">
+        <v>144</v>
+      </c>
     </row>
     <row r="78" spans="1:23" outlineLevel="1">
       <c r="A78" s="5" t="s">
-        <v>138</v>
+        <v>150</v>
       </c>
       <c r="B78" s="5" t="s">
-        <v>139</v>
+        <v>151</v>
       </c>
       <c r="C78" s="5">
         <v>0</v>
@@ -4887,17 +4923,17 @@
       <c r="D78" s="5"/>
       <c r="E78" s="5"/>
       <c r="F78" s="6">
+        <v>4</v>
+      </c>
+      <c r="G78" s="6">
         <v>7</v>
       </c>
-      <c r="G78" s="6">
-        <v>0</v>
-      </c>
       <c r="H78" s="6" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="I78" s="6"/>
       <c r="J78" s="6">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="K78" s="6">
         <v>0</v>
@@ -4908,80 +4944,84 @@
       <c r="M78" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="N78" s="7" t="s">
-        <v>25</v>
-      </c>
+      <c r="N78" s="8"/>
       <c r="O78" s="6" t="s">
         <v>26</v>
       </c>
       <c r="P78" s="8"/>
       <c r="Q78" s="6"/>
-      <c r="R78" s="8"/>
+      <c r="R78" s="7" t="s">
+        <v>25</v>
+      </c>
       <c r="S78" s="6"/>
       <c r="T78" s="8"/>
       <c r="U78" s="6"/>
       <c r="V78" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="W78" s="6"/>
-    </row>
-    <row r="79" spans="1:23">
-      <c r="A79" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="W78" s="6" t="s">
         <v>144</v>
       </c>
-      <c r="B79" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="C79" s="2">
-        <v>0</v>
-      </c>
-      <c r="D79" s="2"/>
-      <c r="E79" s="2"/>
-      <c r="F79" s="2">
-        <v>1</v>
-      </c>
-      <c r="G79" s="2">
-        <v>0</v>
-      </c>
-      <c r="H79" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="I79" s="2"/>
-      <c r="J79" s="2">
-        <v>16</v>
-      </c>
-      <c r="K79" s="2">
-        <v>0</v>
-      </c>
-      <c r="L79" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="M79" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="N79" s="4"/>
-      <c r="O79" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="P79" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q79" s="2"/>
-      <c r="R79" s="4"/>
-      <c r="S79" s="2"/>
-      <c r="T79" s="4"/>
-      <c r="U79" s="2"/>
-      <c r="V79" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="W79" s="2"/>
+    </row>
+    <row r="79" spans="1:23" outlineLevel="1">
+      <c r="A79" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="B79" s="5" t="s">
+        <v>151</v>
+      </c>
+      <c r="C79" s="5">
+        <v>0</v>
+      </c>
+      <c r="D79" s="5"/>
+      <c r="E79" s="5"/>
+      <c r="F79" s="6">
+        <v>6</v>
+      </c>
+      <c r="G79" s="6">
+        <v>1</v>
+      </c>
+      <c r="H79" s="6" t="s">
+        <v>148</v>
+      </c>
+      <c r="I79" s="6"/>
+      <c r="J79" s="6">
+        <v>10</v>
+      </c>
+      <c r="K79" s="6">
+        <v>0</v>
+      </c>
+      <c r="L79" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="M79" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="N79" s="8"/>
+      <c r="O79" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="P79" s="8"/>
+      <c r="Q79" s="6"/>
+      <c r="R79" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="S79" s="6"/>
+      <c r="T79" s="8"/>
+      <c r="U79" s="6"/>
+      <c r="V79" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="W79" s="6" t="s">
+        <v>144</v>
+      </c>
     </row>
     <row r="80" spans="1:23" outlineLevel="1">
       <c r="A80" s="5" t="s">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="B80" s="5" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="C80" s="5">
         <v>0</v>
@@ -4989,17 +5029,17 @@
       <c r="D80" s="5"/>
       <c r="E80" s="5"/>
       <c r="F80" s="6">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="G80" s="6">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H80" s="6" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="I80" s="6"/>
       <c r="J80" s="6">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="K80" s="6">
         <v>0</v>
@@ -5014,76 +5054,78 @@
       <c r="O80" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="P80" s="7" t="s">
-        <v>25</v>
-      </c>
+      <c r="P80" s="8"/>
       <c r="Q80" s="6"/>
-      <c r="R80" s="8"/>
+      <c r="R80" s="7" t="s">
+        <v>25</v>
+      </c>
       <c r="S80" s="6"/>
       <c r="T80" s="8"/>
       <c r="U80" s="6"/>
       <c r="V80" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="W80" s="6" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="81" spans="1:23">
+      <c r="A81" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="B81" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="C81" s="2">
+        <v>0</v>
+      </c>
+      <c r="D81" s="2"/>
+      <c r="E81" s="2"/>
+      <c r="F81" s="2">
+        <v>1</v>
+      </c>
+      <c r="G81" s="2">
+        <v>0</v>
+      </c>
+      <c r="H81" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="I81" s="2"/>
+      <c r="J81" s="2">
+        <v>16</v>
+      </c>
+      <c r="K81" s="2">
+        <v>0</v>
+      </c>
+      <c r="L81" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="M81" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="N81" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="O81" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="P81" s="4"/>
+      <c r="Q81" s="2"/>
+      <c r="R81" s="4"/>
+      <c r="S81" s="2"/>
+      <c r="T81" s="4"/>
+      <c r="U81" s="2"/>
+      <c r="V81" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="W80" s="6"/>
-    </row>
-    <row r="81" spans="1:23" outlineLevel="1">
-      <c r="A81" s="5" t="s">
-        <v>144</v>
-      </c>
-      <c r="B81" s="5" t="s">
-        <v>145</v>
-      </c>
-      <c r="C81" s="5">
-        <v>0</v>
-      </c>
-      <c r="D81" s="5"/>
-      <c r="E81" s="5"/>
-      <c r="F81" s="6">
-        <v>5</v>
-      </c>
-      <c r="G81" s="6">
-        <v>0</v>
-      </c>
-      <c r="H81" s="6" t="s">
-        <v>148</v>
-      </c>
-      <c r="I81" s="6"/>
-      <c r="J81" s="6">
-        <v>16</v>
-      </c>
-      <c r="K81" s="6">
-        <v>0</v>
-      </c>
-      <c r="L81" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="M81" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="N81" s="8"/>
-      <c r="O81" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="P81" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q81" s="6"/>
-      <c r="R81" s="8"/>
-      <c r="S81" s="6"/>
-      <c r="T81" s="8"/>
-      <c r="U81" s="6"/>
-      <c r="V81" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="W81" s="6"/>
+      <c r="W81" s="2"/>
     </row>
     <row r="82" spans="1:23" outlineLevel="1">
       <c r="A82" s="5" t="s">
-        <v>144</v>
+        <v>152</v>
       </c>
       <c r="B82" s="5" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="C82" s="5">
         <v>0</v>
@@ -5091,13 +5133,13 @@
       <c r="D82" s="5"/>
       <c r="E82" s="5"/>
       <c r="F82" s="6">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="G82" s="6">
         <v>0</v>
       </c>
       <c r="H82" s="6" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
       <c r="I82" s="6"/>
       <c r="J82" s="6">
@@ -5112,13 +5154,13 @@
       <c r="M82" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="N82" s="8"/>
+      <c r="N82" s="7" t="s">
+        <v>25</v>
+      </c>
       <c r="O82" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="P82" s="7" t="s">
-        <v>25</v>
-      </c>
+      <c r="P82" s="8"/>
       <c r="Q82" s="6"/>
       <c r="R82" s="8"/>
       <c r="S82" s="6"/>
@@ -5129,61 +5171,63 @@
       </c>
       <c r="W82" s="6"/>
     </row>
-    <row r="83" spans="1:23">
-      <c r="A83" s="2" t="s">
-        <v>150</v>
-      </c>
-      <c r="B83" s="2" t="s">
-        <v>151</v>
-      </c>
-      <c r="C83" s="2">
-        <v>0</v>
-      </c>
-      <c r="D83" s="2"/>
-      <c r="E83" s="2"/>
-      <c r="F83" s="2">
-        <v>1</v>
-      </c>
-      <c r="G83" s="2">
-        <v>0</v>
-      </c>
-      <c r="H83" s="2" t="s">
+    <row r="83" spans="1:23" outlineLevel="1">
+      <c r="A83" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="I83" s="2"/>
-      <c r="J83" s="2">
-        <v>1</v>
-      </c>
-      <c r="K83" s="2">
-        <v>0</v>
-      </c>
-      <c r="L83" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="M83" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="N83" s="4"/>
-      <c r="O83" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="P83" s="4"/>
-      <c r="Q83" s="2"/>
-      <c r="R83" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="S83" s="2"/>
-      <c r="T83" s="4"/>
-      <c r="U83" s="2"/>
-      <c r="V83" s="2"/>
-      <c r="W83" s="2"/>
+      <c r="B83" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="C83" s="5">
+        <v>0</v>
+      </c>
+      <c r="D83" s="5"/>
+      <c r="E83" s="5"/>
+      <c r="F83" s="6">
+        <v>5</v>
+      </c>
+      <c r="G83" s="6">
+        <v>0</v>
+      </c>
+      <c r="H83" s="6" t="s">
+        <v>156</v>
+      </c>
+      <c r="I83" s="6"/>
+      <c r="J83" s="6">
+        <v>16</v>
+      </c>
+      <c r="K83" s="6">
+        <v>0</v>
+      </c>
+      <c r="L83" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="M83" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="N83" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="O83" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="P83" s="8"/>
+      <c r="Q83" s="6"/>
+      <c r="R83" s="8"/>
+      <c r="S83" s="6"/>
+      <c r="T83" s="8"/>
+      <c r="U83" s="6"/>
+      <c r="V83" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="W83" s="6"/>
     </row>
     <row r="84" spans="1:23" outlineLevel="1">
       <c r="A84" s="5" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B84" s="5" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="C84" s="5">
         <v>0</v>
@@ -5191,17 +5235,17 @@
       <c r="D84" s="5"/>
       <c r="E84" s="5"/>
       <c r="F84" s="6">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="G84" s="6">
         <v>0</v>
       </c>
       <c r="H84" s="6" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="I84" s="6"/>
       <c r="J84" s="6">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="K84" s="6">
         <v>0</v>
@@ -5212,133 +5256,131 @@
       <c r="M84" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="N84" s="8"/>
-      <c r="O84" s="10" t="s">
-        <v>25</v>
+      <c r="N84" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="O84" s="6" t="s">
+        <v>26</v>
       </c>
       <c r="P84" s="8"/>
       <c r="Q84" s="6"/>
-      <c r="R84" s="8" t="s">
-        <v>26</v>
-      </c>
+      <c r="R84" s="8"/>
       <c r="S84" s="6"/>
       <c r="T84" s="8"/>
       <c r="U84" s="6"/>
       <c r="V84" s="6" t="s">
-        <v>54</v>
+        <v>30</v>
       </c>
       <c r="W84" s="6"/>
     </row>
-    <row r="85" spans="1:23" outlineLevel="1">
-      <c r="A85" s="5" t="s">
-        <v>150</v>
-      </c>
-      <c r="B85" s="5" t="s">
-        <v>151</v>
-      </c>
-      <c r="C85" s="5">
-        <v>0</v>
-      </c>
-      <c r="D85" s="5"/>
-      <c r="E85" s="5"/>
-      <c r="F85" s="6">
+    <row r="85" spans="1:23">
+      <c r="A85" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="B85" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="C85" s="2">
+        <v>0</v>
+      </c>
+      <c r="D85" s="2"/>
+      <c r="E85" s="2"/>
+      <c r="F85" s="2">
+        <v>1</v>
+      </c>
+      <c r="G85" s="2">
+        <v>0</v>
+      </c>
+      <c r="H85" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="I85" s="2"/>
+      <c r="J85" s="2">
+        <v>16</v>
+      </c>
+      <c r="K85" s="2">
+        <v>0</v>
+      </c>
+      <c r="L85" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="M85" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="N85" s="4"/>
+      <c r="O85" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="P85" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q85" s="2"/>
+      <c r="R85" s="4"/>
+      <c r="S85" s="2"/>
+      <c r="T85" s="4"/>
+      <c r="U85" s="2"/>
+      <c r="V85" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="W85" s="2"/>
+    </row>
+    <row r="86" spans="1:23" outlineLevel="1">
+      <c r="A86" s="5" t="s">
+        <v>158</v>
+      </c>
+      <c r="B86" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="C86" s="5">
+        <v>0</v>
+      </c>
+      <c r="D86" s="5"/>
+      <c r="E86" s="5"/>
+      <c r="F86" s="6">
         <v>3</v>
       </c>
-      <c r="G85" s="6">
-        <v>0</v>
-      </c>
-      <c r="H85" s="6" t="s">
-        <v>154</v>
-      </c>
-      <c r="I85" s="6"/>
-      <c r="J85" s="6">
-        <v>8</v>
-      </c>
-      <c r="K85" s="6">
-        <v>0</v>
-      </c>
-      <c r="L85" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="M85" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="N85" s="8"/>
-      <c r="O85" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="P85" s="8"/>
-      <c r="Q85" s="6"/>
-      <c r="R85" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="S85" s="6"/>
-      <c r="T85" s="8"/>
-      <c r="U85" s="6"/>
-      <c r="V85" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="W85" s="6"/>
-    </row>
-    <row r="86" spans="1:23">
-      <c r="A86" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="B86" s="2" t="s">
-        <v>156</v>
-      </c>
-      <c r="C86" s="2">
-        <v>0</v>
-      </c>
-      <c r="D86" s="2"/>
-      <c r="E86" s="2"/>
-      <c r="F86" s="2">
-        <v>1</v>
-      </c>
-      <c r="G86" s="2">
-        <v>0</v>
-      </c>
-      <c r="H86" s="2" t="s">
-        <v>157</v>
-      </c>
-      <c r="I86" s="2"/>
-      <c r="J86" s="2">
-        <v>10</v>
-      </c>
-      <c r="K86" s="2">
-        <v>0</v>
-      </c>
-      <c r="L86" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="M86" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="N86" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="O86" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="P86" s="4"/>
-      <c r="Q86" s="2"/>
-      <c r="R86" s="4"/>
-      <c r="S86" s="2"/>
-      <c r="T86" s="4"/>
-      <c r="U86" s="2"/>
-      <c r="V86" s="2" t="s">
-        <v>129</v>
-      </c>
-      <c r="W86" s="2" t="s">
-        <v>130</v>
-      </c>
+      <c r="G86" s="6">
+        <v>0</v>
+      </c>
+      <c r="H86" s="6" t="s">
+        <v>161</v>
+      </c>
+      <c r="I86" s="6"/>
+      <c r="J86" s="6">
+        <v>16</v>
+      </c>
+      <c r="K86" s="6">
+        <v>0</v>
+      </c>
+      <c r="L86" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="M86" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="N86" s="8"/>
+      <c r="O86" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="P86" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q86" s="6"/>
+      <c r="R86" s="8"/>
+      <c r="S86" s="6"/>
+      <c r="T86" s="8"/>
+      <c r="U86" s="6"/>
+      <c r="V86" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="W86" s="6"/>
     </row>
     <row r="87" spans="1:23" outlineLevel="1">
       <c r="A87" s="5" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="B87" s="5" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="C87" s="5">
         <v>0</v>
@@ -5346,17 +5388,17 @@
       <c r="D87" s="5"/>
       <c r="E87" s="5"/>
       <c r="F87" s="6">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G87" s="6">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H87" s="6" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="I87" s="6"/>
       <c r="J87" s="6">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="K87" s="6">
         <v>0</v>
@@ -5367,31 +5409,29 @@
       <c r="M87" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="N87" s="7" t="s">
-        <v>25</v>
-      </c>
+      <c r="N87" s="8"/>
       <c r="O87" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="P87" s="8"/>
+      <c r="P87" s="7" t="s">
+        <v>25</v>
+      </c>
       <c r="Q87" s="6"/>
       <c r="R87" s="8"/>
       <c r="S87" s="6"/>
       <c r="T87" s="8"/>
       <c r="U87" s="6"/>
       <c r="V87" s="6" t="s">
-        <v>129</v>
-      </c>
-      <c r="W87" s="6" t="s">
-        <v>130</v>
-      </c>
+        <v>30</v>
+      </c>
+      <c r="W87" s="6"/>
     </row>
     <row r="88" spans="1:23" outlineLevel="1">
       <c r="A88" s="5" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="B88" s="5" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="C88" s="5">
         <v>0</v>
@@ -5399,17 +5439,17 @@
       <c r="D88" s="5"/>
       <c r="E88" s="5"/>
       <c r="F88" s="6">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="G88" s="6">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H88" s="6" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="I88" s="6"/>
       <c r="J88" s="6">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="K88" s="6">
         <v>0</v>
@@ -5420,84 +5460,78 @@
       <c r="M88" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="N88" s="7" t="s">
-        <v>25</v>
-      </c>
+      <c r="N88" s="8"/>
       <c r="O88" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="P88" s="8"/>
+      <c r="P88" s="7" t="s">
+        <v>25</v>
+      </c>
       <c r="Q88" s="6"/>
       <c r="R88" s="8"/>
       <c r="S88" s="6"/>
       <c r="T88" s="8"/>
       <c r="U88" s="6"/>
       <c r="V88" s="6" t="s">
-        <v>129</v>
-      </c>
-      <c r="W88" s="6" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="89" spans="1:23" outlineLevel="1">
-      <c r="A89" s="5" t="s">
-        <v>155</v>
-      </c>
-      <c r="B89" s="5" t="s">
-        <v>156</v>
-      </c>
-      <c r="C89" s="5">
-        <v>0</v>
-      </c>
-      <c r="D89" s="5"/>
-      <c r="E89" s="5"/>
-      <c r="F89" s="6">
-        <v>4</v>
-      </c>
-      <c r="G89" s="6">
-        <v>6</v>
-      </c>
-      <c r="H89" s="6" t="s">
-        <v>160</v>
-      </c>
-      <c r="I89" s="6"/>
-      <c r="J89" s="6">
-        <v>10</v>
-      </c>
-      <c r="K89" s="6">
-        <v>0</v>
-      </c>
-      <c r="L89" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="M89" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="N89" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="O89" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="P89" s="8"/>
-      <c r="Q89" s="6"/>
-      <c r="R89" s="8"/>
-      <c r="S89" s="6"/>
-      <c r="T89" s="8"/>
-      <c r="U89" s="6"/>
-      <c r="V89" s="6" t="s">
-        <v>129</v>
-      </c>
-      <c r="W89" s="6" t="s">
-        <v>130</v>
-      </c>
+        <v>30</v>
+      </c>
+      <c r="W88" s="6"/>
+    </row>
+    <row r="89" spans="1:23">
+      <c r="A89" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="B89" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="C89" s="2">
+        <v>0</v>
+      </c>
+      <c r="D89" s="2"/>
+      <c r="E89" s="2"/>
+      <c r="F89" s="2">
+        <v>1</v>
+      </c>
+      <c r="G89" s="2">
+        <v>0</v>
+      </c>
+      <c r="H89" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="I89" s="2"/>
+      <c r="J89" s="2">
+        <v>1</v>
+      </c>
+      <c r="K89" s="2">
+        <v>0</v>
+      </c>
+      <c r="L89" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="M89" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="N89" s="4"/>
+      <c r="O89" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="P89" s="4"/>
+      <c r="Q89" s="2"/>
+      <c r="R89" s="4"/>
+      <c r="S89" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="T89" s="4"/>
+      <c r="U89" s="2"/>
+      <c r="V89" s="2"/>
+      <c r="W89" s="2"/>
     </row>
     <row r="90" spans="1:23" outlineLevel="1">
       <c r="A90" s="5" t="s">
-        <v>155</v>
+        <v>164</v>
       </c>
       <c r="B90" s="5" t="s">
-        <v>156</v>
+        <v>165</v>
       </c>
       <c r="C90" s="5">
         <v>0</v>
@@ -5505,17 +5539,17 @@
       <c r="D90" s="5"/>
       <c r="E90" s="5"/>
       <c r="F90" s="6">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G90" s="6">
         <v>0</v>
       </c>
       <c r="H90" s="6" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="I90" s="6"/>
       <c r="J90" s="6">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="K90" s="6">
         <v>0</v>
@@ -5526,31 +5560,29 @@
       <c r="M90" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="N90" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="O90" s="6" t="s">
-        <v>26</v>
+      <c r="N90" s="8"/>
+      <c r="O90" s="10" t="s">
+        <v>25</v>
       </c>
       <c r="P90" s="8"/>
       <c r="Q90" s="6"/>
       <c r="R90" s="8"/>
-      <c r="S90" s="6"/>
+      <c r="S90" s="6" t="s">
+        <v>26</v>
+      </c>
       <c r="T90" s="8"/>
       <c r="U90" s="6"/>
       <c r="V90" s="6" t="s">
-        <v>129</v>
-      </c>
-      <c r="W90" s="6" t="s">
-        <v>130</v>
-      </c>
+        <v>54</v>
+      </c>
+      <c r="W90" s="6"/>
     </row>
     <row r="91" spans="1:23" outlineLevel="1">
       <c r="A91" s="5" t="s">
-        <v>155</v>
+        <v>164</v>
       </c>
       <c r="B91" s="5" t="s">
-        <v>156</v>
+        <v>165</v>
       </c>
       <c r="C91" s="5">
         <v>0</v>
@@ -5558,17 +5590,17 @@
       <c r="D91" s="5"/>
       <c r="E91" s="5"/>
       <c r="F91" s="6">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="G91" s="6">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H91" s="6" t="s">
-        <v>162</v>
+        <v>168</v>
       </c>
       <c r="I91" s="6"/>
       <c r="J91" s="6">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="K91" s="6">
         <v>0</v>
@@ -5579,31 +5611,29 @@
       <c r="M91" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="N91" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="O91" s="6" t="s">
-        <v>26</v>
+      <c r="N91" s="8"/>
+      <c r="O91" s="10" t="s">
+        <v>25</v>
       </c>
       <c r="P91" s="8"/>
       <c r="Q91" s="6"/>
       <c r="R91" s="8"/>
-      <c r="S91" s="6"/>
+      <c r="S91" s="6" t="s">
+        <v>26</v>
+      </c>
       <c r="T91" s="8"/>
       <c r="U91" s="6"/>
       <c r="V91" s="6" t="s">
-        <v>129</v>
-      </c>
-      <c r="W91" s="6" t="s">
-        <v>130</v>
-      </c>
+        <v>54</v>
+      </c>
+      <c r="W91" s="6"/>
     </row>
     <row r="92" spans="1:23">
       <c r="A92" s="2" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="B92" s="2" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
       <c r="C92" s="2">
         <v>0</v>
@@ -5617,7 +5647,7 @@
         <v>0</v>
       </c>
       <c r="H92" s="2" t="s">
-        <v>157</v>
+        <v>171</v>
       </c>
       <c r="I92" s="2"/>
       <c r="J92" s="2">
@@ -5632,31 +5662,31 @@
       <c r="M92" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="N92" s="4"/>
+      <c r="N92" s="3" t="s">
+        <v>25</v>
+      </c>
       <c r="O92" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="P92" s="3" t="s">
-        <v>25</v>
-      </c>
+      <c r="P92" s="4"/>
       <c r="Q92" s="2"/>
       <c r="R92" s="4"/>
       <c r="S92" s="2"/>
       <c r="T92" s="4"/>
       <c r="U92" s="2"/>
       <c r="V92" s="2" t="s">
-        <v>129</v>
+        <v>143</v>
       </c>
       <c r="W92" s="2" t="s">
-        <v>130</v>
+        <v>144</v>
       </c>
     </row>
     <row r="93" spans="1:23" outlineLevel="1">
       <c r="A93" s="5" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="B93" s="5" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
       <c r="C93" s="5">
         <v>0</v>
@@ -5670,7 +5700,7 @@
         <v>2</v>
       </c>
       <c r="H93" s="6" t="s">
-        <v>158</v>
+        <v>172</v>
       </c>
       <c r="I93" s="6"/>
       <c r="J93" s="6">
@@ -5685,31 +5715,31 @@
       <c r="M93" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="N93" s="8"/>
+      <c r="N93" s="7" t="s">
+        <v>25</v>
+      </c>
       <c r="O93" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="P93" s="7" t="s">
-        <v>25</v>
-      </c>
+      <c r="P93" s="8"/>
       <c r="Q93" s="6"/>
       <c r="R93" s="8"/>
       <c r="S93" s="6"/>
       <c r="T93" s="8"/>
       <c r="U93" s="6"/>
       <c r="V93" s="6" t="s">
-        <v>129</v>
+        <v>143</v>
       </c>
       <c r="W93" s="6" t="s">
-        <v>130</v>
+        <v>144</v>
       </c>
     </row>
     <row r="94" spans="1:23" outlineLevel="1">
       <c r="A94" s="5" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="B94" s="5" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
       <c r="C94" s="5">
         <v>0</v>
@@ -5723,7 +5753,7 @@
         <v>4</v>
       </c>
       <c r="H94" s="6" t="s">
-        <v>159</v>
+        <v>173</v>
       </c>
       <c r="I94" s="6"/>
       <c r="J94" s="6">
@@ -5738,31 +5768,31 @@
       <c r="M94" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="N94" s="8"/>
+      <c r="N94" s="7" t="s">
+        <v>25</v>
+      </c>
       <c r="O94" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="P94" s="7" t="s">
-        <v>25</v>
-      </c>
+      <c r="P94" s="8"/>
       <c r="Q94" s="6"/>
       <c r="R94" s="8"/>
       <c r="S94" s="6"/>
       <c r="T94" s="8"/>
       <c r="U94" s="6"/>
       <c r="V94" s="6" t="s">
-        <v>129</v>
+        <v>143</v>
       </c>
       <c r="W94" s="6" t="s">
-        <v>130</v>
+        <v>144</v>
       </c>
     </row>
     <row r="95" spans="1:23" outlineLevel="1">
       <c r="A95" s="5" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="B95" s="5" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
       <c r="C95" s="5">
         <v>0</v>
@@ -5776,7 +5806,7 @@
         <v>6</v>
       </c>
       <c r="H95" s="6" t="s">
-        <v>160</v>
+        <v>174</v>
       </c>
       <c r="I95" s="6"/>
       <c r="J95" s="6">
@@ -5791,31 +5821,31 @@
       <c r="M95" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="N95" s="8"/>
+      <c r="N95" s="7" t="s">
+        <v>25</v>
+      </c>
       <c r="O95" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="P95" s="7" t="s">
-        <v>25</v>
-      </c>
+      <c r="P95" s="8"/>
       <c r="Q95" s="6"/>
       <c r="R95" s="8"/>
       <c r="S95" s="6"/>
       <c r="T95" s="8"/>
       <c r="U95" s="6"/>
       <c r="V95" s="6" t="s">
-        <v>129</v>
+        <v>143</v>
       </c>
       <c r="W95" s="6" t="s">
-        <v>130</v>
+        <v>144</v>
       </c>
     </row>
     <row r="96" spans="1:23" outlineLevel="1">
       <c r="A96" s="5" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="B96" s="5" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
       <c r="C96" s="5">
         <v>0</v>
@@ -5829,7 +5859,7 @@
         <v>0</v>
       </c>
       <c r="H96" s="6" t="s">
-        <v>165</v>
+        <v>175</v>
       </c>
       <c r="I96" s="6"/>
       <c r="J96" s="6">
@@ -5844,31 +5874,31 @@
       <c r="M96" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="N96" s="8"/>
+      <c r="N96" s="7" t="s">
+        <v>25</v>
+      </c>
       <c r="O96" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="P96" s="7" t="s">
-        <v>25</v>
-      </c>
+      <c r="P96" s="8"/>
       <c r="Q96" s="6"/>
       <c r="R96" s="8"/>
       <c r="S96" s="6"/>
       <c r="T96" s="8"/>
       <c r="U96" s="6"/>
       <c r="V96" s="6" t="s">
-        <v>129</v>
+        <v>143</v>
       </c>
       <c r="W96" s="6" t="s">
-        <v>130</v>
+        <v>144</v>
       </c>
     </row>
     <row r="97" spans="1:23" outlineLevel="1">
       <c r="A97" s="5" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="B97" s="5" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
       <c r="C97" s="5">
         <v>0</v>
@@ -5882,7 +5912,7 @@
         <v>2</v>
       </c>
       <c r="H97" s="6" t="s">
-        <v>166</v>
+        <v>176</v>
       </c>
       <c r="I97" s="6"/>
       <c r="J97" s="6">
@@ -5897,31 +5927,31 @@
       <c r="M97" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="N97" s="8"/>
+      <c r="N97" s="7" t="s">
+        <v>25</v>
+      </c>
       <c r="O97" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="P97" s="7" t="s">
-        <v>25</v>
-      </c>
+      <c r="P97" s="8"/>
       <c r="Q97" s="6"/>
       <c r="R97" s="8"/>
       <c r="S97" s="6"/>
       <c r="T97" s="8"/>
       <c r="U97" s="6"/>
       <c r="V97" s="6" t="s">
-        <v>129</v>
+        <v>143</v>
       </c>
       <c r="W97" s="6" t="s">
-        <v>130</v>
+        <v>144</v>
       </c>
     </row>
     <row r="98" spans="1:23">
       <c r="A98" s="2" t="s">
-        <v>167</v>
+        <v>177</v>
       </c>
       <c r="B98" s="2" t="s">
-        <v>168</v>
+        <v>178</v>
       </c>
       <c r="C98" s="2">
         <v>0</v>
@@ -5935,11 +5965,11 @@
         <v>0</v>
       </c>
       <c r="H98" s="2" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="I98" s="2"/>
       <c r="J98" s="2">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="K98" s="2">
         <v>0</v>
@@ -5963,16 +5993,18 @@
       <c r="T98" s="4"/>
       <c r="U98" s="2"/>
       <c r="V98" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="W98" s="2"/>
+        <v>143</v>
+      </c>
+      <c r="W98" s="2" t="s">
+        <v>144</v>
+      </c>
     </row>
     <row r="99" spans="1:23" outlineLevel="1">
       <c r="A99" s="5" t="s">
-        <v>167</v>
+        <v>177</v>
       </c>
       <c r="B99" s="5" t="s">
-        <v>168</v>
+        <v>178</v>
       </c>
       <c r="C99" s="5">
         <v>0</v>
@@ -5980,17 +6012,17 @@
       <c r="D99" s="5"/>
       <c r="E99" s="5"/>
       <c r="F99" s="6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G99" s="6">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H99" s="6" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="I99" s="6"/>
       <c r="J99" s="6">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="K99" s="6">
         <v>0</v>
@@ -6014,65 +6046,71 @@
       <c r="T99" s="8"/>
       <c r="U99" s="6"/>
       <c r="V99" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="W99" s="6"/>
-    </row>
-    <row r="100" spans="1:23">
-      <c r="A100" s="2" t="s">
-        <v>171</v>
-      </c>
-      <c r="B100" s="2" t="s">
-        <v>172</v>
-      </c>
-      <c r="C100" s="2">
-        <v>0</v>
-      </c>
-      <c r="D100" s="2"/>
-      <c r="E100" s="2"/>
-      <c r="F100" s="2">
-        <v>1</v>
-      </c>
-      <c r="G100" s="2">
-        <v>0</v>
-      </c>
-      <c r="H100" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="W99" s="6" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="100" spans="1:23" outlineLevel="1">
+      <c r="A100" s="5" t="s">
+        <v>177</v>
+      </c>
+      <c r="B100" s="5" t="s">
+        <v>178</v>
+      </c>
+      <c r="C100" s="5">
+        <v>0</v>
+      </c>
+      <c r="D100" s="5"/>
+      <c r="E100" s="5"/>
+      <c r="F100" s="6">
+        <v>3</v>
+      </c>
+      <c r="G100" s="6">
+        <v>4</v>
+      </c>
+      <c r="H100" s="6" t="s">
         <v>173</v>
       </c>
-      <c r="I100" s="2"/>
-      <c r="J100" s="2">
-        <v>1</v>
-      </c>
-      <c r="K100" s="2">
-        <v>0</v>
-      </c>
-      <c r="L100" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="M100" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="N100" s="4"/>
-      <c r="O100" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="P100" s="4"/>
-      <c r="Q100" s="2"/>
-      <c r="R100" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="S100" s="2"/>
-      <c r="T100" s="4"/>
-      <c r="U100" s="2"/>
-      <c r="V100" s="2"/>
-      <c r="W100" s="2"/>
+      <c r="I100" s="6"/>
+      <c r="J100" s="6">
+        <v>10</v>
+      </c>
+      <c r="K100" s="6">
+        <v>0</v>
+      </c>
+      <c r="L100" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="M100" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="N100" s="8"/>
+      <c r="O100" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="P100" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q100" s="6"/>
+      <c r="R100" s="8"/>
+      <c r="S100" s="6"/>
+      <c r="T100" s="8"/>
+      <c r="U100" s="6"/>
+      <c r="V100" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="W100" s="6" t="s">
+        <v>144</v>
+      </c>
     </row>
     <row r="101" spans="1:23" outlineLevel="1">
       <c r="A101" s="5" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="B101" s="5" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
       <c r="C101" s="5">
         <v>0</v>
@@ -6080,17 +6118,17 @@
       <c r="D101" s="5"/>
       <c r="E101" s="5"/>
       <c r="F101" s="6">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G101" s="6">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="H101" s="6" t="s">
         <v>174</v>
       </c>
       <c r="I101" s="6"/>
       <c r="J101" s="6">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="K101" s="6">
         <v>0</v>
@@ -6105,23 +6143,27 @@
       <c r="O101" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="P101" s="8"/>
+      <c r="P101" s="7" t="s">
+        <v>25</v>
+      </c>
       <c r="Q101" s="6"/>
-      <c r="R101" s="7" t="s">
-        <v>25</v>
-      </c>
+      <c r="R101" s="8"/>
       <c r="S101" s="6"/>
       <c r="T101" s="8"/>
       <c r="U101" s="6"/>
-      <c r="V101" s="6"/>
-      <c r="W101" s="6"/>
+      <c r="V101" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="W101" s="6" t="s">
+        <v>144</v>
+      </c>
     </row>
     <row r="102" spans="1:23" outlineLevel="1">
       <c r="A102" s="5" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="B102" s="5" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
       <c r="C102" s="5">
         <v>0</v>
@@ -6129,17 +6171,17 @@
       <c r="D102" s="5"/>
       <c r="E102" s="5"/>
       <c r="F102" s="6">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="G102" s="6">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H102" s="6" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="I102" s="6"/>
       <c r="J102" s="6">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="K102" s="6">
         <v>0</v>
@@ -6154,23 +6196,27 @@
       <c r="O102" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="P102" s="8"/>
+      <c r="P102" s="7" t="s">
+        <v>25</v>
+      </c>
       <c r="Q102" s="6"/>
-      <c r="R102" s="7" t="s">
-        <v>25</v>
-      </c>
+      <c r="R102" s="8"/>
       <c r="S102" s="6"/>
       <c r="T102" s="8"/>
       <c r="U102" s="6"/>
-      <c r="V102" s="6"/>
-      <c r="W102" s="6"/>
+      <c r="V102" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="W102" s="6" t="s">
+        <v>144</v>
+      </c>
     </row>
     <row r="103" spans="1:23" outlineLevel="1">
       <c r="A103" s="5" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="B103" s="5" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
       <c r="C103" s="5">
         <v>0</v>
@@ -6178,17 +6224,17 @@
       <c r="D103" s="5"/>
       <c r="E103" s="5"/>
       <c r="F103" s="6">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="G103" s="6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H103" s="6" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="I103" s="6"/>
       <c r="J103" s="6">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="K103" s="6">
         <v>0</v>
@@ -6203,19 +6249,321 @@
       <c r="O103" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="P103" s="8"/>
+      <c r="P103" s="7" t="s">
+        <v>25</v>
+      </c>
       <c r="Q103" s="6"/>
-      <c r="R103" s="7" t="s">
-        <v>25</v>
-      </c>
+      <c r="R103" s="8"/>
       <c r="S103" s="6"/>
       <c r="T103" s="8"/>
       <c r="U103" s="6"/>
-      <c r="V103" s="6"/>
-      <c r="W103" s="6"/>
+      <c r="V103" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="W103" s="6" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="104" spans="1:23">
+      <c r="A104" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="B104" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="C104" s="2">
+        <v>0</v>
+      </c>
+      <c r="D104" s="2"/>
+      <c r="E104" s="2"/>
+      <c r="F104" s="2">
+        <v>1</v>
+      </c>
+      <c r="G104" s="2">
+        <v>0</v>
+      </c>
+      <c r="H104" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="I104" s="2"/>
+      <c r="J104" s="2">
+        <v>16</v>
+      </c>
+      <c r="K104" s="2">
+        <v>0</v>
+      </c>
+      <c r="L104" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="M104" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="N104" s="4"/>
+      <c r="O104" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="P104" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q104" s="2"/>
+      <c r="R104" s="4"/>
+      <c r="S104" s="2"/>
+      <c r="T104" s="4"/>
+      <c r="U104" s="2"/>
+      <c r="V104" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="W104" s="2"/>
+    </row>
+    <row r="105" spans="1:23" outlineLevel="1">
+      <c r="A105" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="B105" s="5" t="s">
+        <v>182</v>
+      </c>
+      <c r="C105" s="5">
+        <v>0</v>
+      </c>
+      <c r="D105" s="5"/>
+      <c r="E105" s="5"/>
+      <c r="F105" s="6">
+        <v>3</v>
+      </c>
+      <c r="G105" s="6">
+        <v>0</v>
+      </c>
+      <c r="H105" s="6" t="s">
+        <v>184</v>
+      </c>
+      <c r="I105" s="6"/>
+      <c r="J105" s="6">
+        <v>16</v>
+      </c>
+      <c r="K105" s="6">
+        <v>0</v>
+      </c>
+      <c r="L105" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="M105" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="N105" s="8"/>
+      <c r="O105" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="P105" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q105" s="6"/>
+      <c r="R105" s="8"/>
+      <c r="S105" s="6"/>
+      <c r="T105" s="8"/>
+      <c r="U105" s="6"/>
+      <c r="V105" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="W105" s="6"/>
+    </row>
+    <row r="106" spans="1:23">
+      <c r="A106" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="B106" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="C106" s="2">
+        <v>0</v>
+      </c>
+      <c r="D106" s="2"/>
+      <c r="E106" s="2"/>
+      <c r="F106" s="2">
+        <v>1</v>
+      </c>
+      <c r="G106" s="2">
+        <v>0</v>
+      </c>
+      <c r="H106" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="I106" s="2"/>
+      <c r="J106" s="2">
+        <v>1</v>
+      </c>
+      <c r="K106" s="2">
+        <v>0</v>
+      </c>
+      <c r="L106" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="M106" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="N106" s="4"/>
+      <c r="O106" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="P106" s="4"/>
+      <c r="Q106" s="2"/>
+      <c r="R106" s="4"/>
+      <c r="S106" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="T106" s="4"/>
+      <c r="U106" s="2"/>
+      <c r="V106" s="2"/>
+      <c r="W106" s="2"/>
+    </row>
+    <row r="107" spans="1:23" outlineLevel="1">
+      <c r="A107" s="5" t="s">
+        <v>185</v>
+      </c>
+      <c r="B107" s="5" t="s">
+        <v>186</v>
+      </c>
+      <c r="C107" s="5">
+        <v>0</v>
+      </c>
+      <c r="D107" s="5"/>
+      <c r="E107" s="5"/>
+      <c r="F107" s="6">
+        <v>1</v>
+      </c>
+      <c r="G107" s="6">
+        <v>1</v>
+      </c>
+      <c r="H107" s="6" t="s">
+        <v>188</v>
+      </c>
+      <c r="I107" s="6"/>
+      <c r="J107" s="6">
+        <v>1</v>
+      </c>
+      <c r="K107" s="6">
+        <v>0</v>
+      </c>
+      <c r="L107" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="M107" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="N107" s="8"/>
+      <c r="O107" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="P107" s="8"/>
+      <c r="Q107" s="6"/>
+      <c r="R107" s="8"/>
+      <c r="S107" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="T107" s="8"/>
+      <c r="U107" s="6"/>
+      <c r="V107" s="6"/>
+      <c r="W107" s="6"/>
+    </row>
+    <row r="108" spans="1:23" outlineLevel="1">
+      <c r="A108" s="5" t="s">
+        <v>185</v>
+      </c>
+      <c r="B108" s="5" t="s">
+        <v>186</v>
+      </c>
+      <c r="C108" s="5">
+        <v>0</v>
+      </c>
+      <c r="D108" s="5"/>
+      <c r="E108" s="5"/>
+      <c r="F108" s="6">
+        <v>1</v>
+      </c>
+      <c r="G108" s="6">
+        <v>2</v>
+      </c>
+      <c r="H108" s="6" t="s">
+        <v>189</v>
+      </c>
+      <c r="I108" s="6"/>
+      <c r="J108" s="6">
+        <v>1</v>
+      </c>
+      <c r="K108" s="6">
+        <v>0</v>
+      </c>
+      <c r="L108" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="M108" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="N108" s="8"/>
+      <c r="O108" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="P108" s="8"/>
+      <c r="Q108" s="6"/>
+      <c r="R108" s="8"/>
+      <c r="S108" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="T108" s="8"/>
+      <c r="U108" s="6"/>
+      <c r="V108" s="6"/>
+      <c r="W108" s="6"/>
+    </row>
+    <row r="109" spans="1:23" outlineLevel="1">
+      <c r="A109" s="5" t="s">
+        <v>185</v>
+      </c>
+      <c r="B109" s="5" t="s">
+        <v>186</v>
+      </c>
+      <c r="C109" s="5">
+        <v>0</v>
+      </c>
+      <c r="D109" s="5"/>
+      <c r="E109" s="5"/>
+      <c r="F109" s="6">
+        <v>1</v>
+      </c>
+      <c r="G109" s="6">
+        <v>3</v>
+      </c>
+      <c r="H109" s="6" t="s">
+        <v>190</v>
+      </c>
+      <c r="I109" s="6"/>
+      <c r="J109" s="6">
+        <v>1</v>
+      </c>
+      <c r="K109" s="6">
+        <v>0</v>
+      </c>
+      <c r="L109" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="M109" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="N109" s="8"/>
+      <c r="O109" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="P109" s="8"/>
+      <c r="Q109" s="6"/>
+      <c r="R109" s="8"/>
+      <c r="S109" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="T109" s="8"/>
+      <c r="U109" s="6"/>
+      <c r="V109" s="6"/>
+      <c r="W109" s="6"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AH104"/>
+  <autoFilter ref="A1:AH110"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
generated from SC22EVO/MCB.json at 5dadd53
</commit_message>
<xml_diff>
--- a/SC22EVO/artifacts/MCB.xlsx
+++ b/SC22EVO/artifacts/MCB.xlsx
@@ -10,14 +10,14 @@
     <sheet name="K-Matrix " sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'K-Matrix '!$A$1:$AH$110</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'K-Matrix '!$A$1:$AH$130</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="883" uniqueCount="191">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1022" uniqueCount="211">
   <si>
     <t>ID</t>
   </si>
@@ -436,7 +436,67 @@
     <t>isRelayOpen</t>
   </si>
   <si>
-    <t>BMSLV_StatusMessage</t>
+    <t>cell1_OV</t>
+  </si>
+  <si>
+    <t>cell2_OV</t>
+  </si>
+  <si>
+    <t>cell3_OV</t>
+  </si>
+  <si>
+    <t>cell4_OV</t>
+  </si>
+  <si>
+    <t>cell5_OV</t>
+  </si>
+  <si>
+    <t>cell6_OV</t>
+  </si>
+  <si>
+    <t>cell7_OV</t>
+  </si>
+  <si>
+    <t>cell1_UV</t>
+  </si>
+  <si>
+    <t>cell2_UV</t>
+  </si>
+  <si>
+    <t>cell3_UV</t>
+  </si>
+  <si>
+    <t>cell4_UV</t>
+  </si>
+  <si>
+    <t>cell5_UV</t>
+  </si>
+  <si>
+    <t>cell6_UV</t>
+  </si>
+  <si>
+    <t>cell7_UV</t>
+  </si>
+  <si>
+    <t>cell1_OT</t>
+  </si>
+  <si>
+    <t>cell2_OT</t>
+  </si>
+  <si>
+    <t>cell3_OT</t>
+  </si>
+  <si>
+    <t>cell4_OT</t>
+  </si>
+  <si>
+    <t>cell5_OT</t>
+  </si>
+  <si>
+    <t>cell6_OT</t>
+  </si>
+  <si>
+    <t>cell7_OT</t>
   </si>
   <si>
     <t>104h</t>
@@ -978,7 +1038,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W109"/>
+  <dimension ref="A1:W129"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="1"/>
   <cols>
     <col min="1" max="1" width="4.28515625" customWidth="1"/>
@@ -4405,7 +4465,7 @@
       </c>
       <c r="I68" s="6"/>
       <c r="J68" s="6">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="K68" s="6">
         <v>0</v>
@@ -4428,70 +4488,64 @@
       <c r="S68" s="6"/>
       <c r="T68" s="8"/>
       <c r="U68" s="6"/>
-      <c r="V68" s="6" t="s">
-        <v>54</v>
-      </c>
+      <c r="V68" s="6"/>
       <c r="W68" s="6"/>
     </row>
-    <row r="69" spans="1:23">
-      <c r="A69" s="2" t="s">
+    <row r="69" spans="1:23" outlineLevel="1">
+      <c r="A69" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="B69" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="C69" s="5">
+        <v>0</v>
+      </c>
+      <c r="D69" s="5"/>
+      <c r="E69" s="5"/>
+      <c r="F69" s="6">
+        <v>1</v>
+      </c>
+      <c r="G69" s="6">
+        <v>2</v>
+      </c>
+      <c r="H69" s="6" t="s">
         <v>140</v>
       </c>
-      <c r="B69" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="C69" s="2">
-        <v>0</v>
-      </c>
-      <c r="D69" s="2"/>
-      <c r="E69" s="2"/>
-      <c r="F69" s="2">
-        <v>1</v>
-      </c>
-      <c r="G69" s="2">
-        <v>1</v>
-      </c>
-      <c r="H69" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="I69" s="2"/>
-      <c r="J69" s="2">
-        <v>10</v>
-      </c>
-      <c r="K69" s="2">
-        <v>0</v>
-      </c>
-      <c r="L69" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="M69" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="N69" s="4"/>
-      <c r="O69" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="P69" s="4"/>
-      <c r="Q69" s="2"/>
-      <c r="R69" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="S69" s="2"/>
-      <c r="T69" s="4"/>
-      <c r="U69" s="2"/>
-      <c r="V69" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="W69" s="2" t="s">
-        <v>144</v>
-      </c>
+      <c r="I69" s="6"/>
+      <c r="J69" s="6">
+        <v>1</v>
+      </c>
+      <c r="K69" s="6">
+        <v>0</v>
+      </c>
+      <c r="L69" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="M69" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="N69" s="8"/>
+      <c r="O69" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="P69" s="8"/>
+      <c r="Q69" s="6"/>
+      <c r="R69" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="S69" s="6"/>
+      <c r="T69" s="8"/>
+      <c r="U69" s="6"/>
+      <c r="V69" s="6"/>
+      <c r="W69" s="6"/>
     </row>
     <row r="70" spans="1:23" outlineLevel="1">
       <c r="A70" s="5" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="B70" s="5" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="C70" s="5">
         <v>0</v>
@@ -4499,17 +4553,17 @@
       <c r="D70" s="5"/>
       <c r="E70" s="5"/>
       <c r="F70" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G70" s="6">
         <v>3</v>
       </c>
       <c r="H70" s="6" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="I70" s="6"/>
       <c r="J70" s="6">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="K70" s="6">
         <v>0</v>
@@ -4532,19 +4586,15 @@
       <c r="S70" s="6"/>
       <c r="T70" s="8"/>
       <c r="U70" s="6"/>
-      <c r="V70" s="6" t="s">
-        <v>143</v>
-      </c>
-      <c r="W70" s="6" t="s">
-        <v>144</v>
-      </c>
+      <c r="V70" s="6"/>
+      <c r="W70" s="6"/>
     </row>
     <row r="71" spans="1:23" outlineLevel="1">
       <c r="A71" s="5" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="B71" s="5" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="C71" s="5">
         <v>0</v>
@@ -4552,17 +4602,17 @@
       <c r="D71" s="5"/>
       <c r="E71" s="5"/>
       <c r="F71" s="6">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G71" s="6">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H71" s="6" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="I71" s="6"/>
       <c r="J71" s="6">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="K71" s="6">
         <v>0</v>
@@ -4585,19 +4635,15 @@
       <c r="S71" s="6"/>
       <c r="T71" s="8"/>
       <c r="U71" s="6"/>
-      <c r="V71" s="6" t="s">
-        <v>143</v>
-      </c>
-      <c r="W71" s="6" t="s">
-        <v>144</v>
-      </c>
+      <c r="V71" s="6"/>
+      <c r="W71" s="6"/>
     </row>
     <row r="72" spans="1:23" outlineLevel="1">
       <c r="A72" s="5" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="B72" s="5" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="C72" s="5">
         <v>0</v>
@@ -4605,17 +4651,17 @@
       <c r="D72" s="5"/>
       <c r="E72" s="5"/>
       <c r="F72" s="6">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G72" s="6">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="H72" s="6" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="I72" s="6"/>
       <c r="J72" s="6">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="K72" s="6">
         <v>0</v>
@@ -4638,19 +4684,15 @@
       <c r="S72" s="6"/>
       <c r="T72" s="8"/>
       <c r="U72" s="6"/>
-      <c r="V72" s="6" t="s">
-        <v>143</v>
-      </c>
-      <c r="W72" s="6" t="s">
-        <v>144</v>
-      </c>
+      <c r="V72" s="6"/>
+      <c r="W72" s="6"/>
     </row>
     <row r="73" spans="1:23" outlineLevel="1">
       <c r="A73" s="5" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="B73" s="5" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="C73" s="5">
         <v>0</v>
@@ -4658,17 +4700,17 @@
       <c r="D73" s="5"/>
       <c r="E73" s="5"/>
       <c r="F73" s="6">
+        <v>1</v>
+      </c>
+      <c r="G73" s="6">
         <v>6</v>
       </c>
-      <c r="G73" s="6">
-        <v>1</v>
-      </c>
       <c r="H73" s="6" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="I73" s="6"/>
       <c r="J73" s="6">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="K73" s="6">
         <v>0</v>
@@ -4691,19 +4733,15 @@
       <c r="S73" s="6"/>
       <c r="T73" s="8"/>
       <c r="U73" s="6"/>
-      <c r="V73" s="6" t="s">
-        <v>143</v>
-      </c>
-      <c r="W73" s="6" t="s">
-        <v>144</v>
-      </c>
+      <c r="V73" s="6"/>
+      <c r="W73" s="6"/>
     </row>
     <row r="74" spans="1:23" outlineLevel="1">
       <c r="A74" s="5" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="B74" s="5" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="C74" s="5">
         <v>0</v>
@@ -4711,17 +4749,17 @@
       <c r="D74" s="5"/>
       <c r="E74" s="5"/>
       <c r="F74" s="6">
+        <v>1</v>
+      </c>
+      <c r="G74" s="6">
         <v>7</v>
       </c>
-      <c r="G74" s="6">
-        <v>6</v>
-      </c>
       <c r="H74" s="6" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="I74" s="6"/>
       <c r="J74" s="6">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="K74" s="6">
         <v>0</v>
@@ -4744,72 +4782,64 @@
       <c r="S74" s="6"/>
       <c r="T74" s="8"/>
       <c r="U74" s="6"/>
-      <c r="V74" s="6" t="s">
-        <v>143</v>
-      </c>
-      <c r="W74" s="6" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="75" spans="1:23">
-      <c r="A75" s="2" t="s">
-        <v>150</v>
-      </c>
-      <c r="B75" s="2" t="s">
-        <v>151</v>
-      </c>
-      <c r="C75" s="2">
-        <v>0</v>
-      </c>
-      <c r="D75" s="2"/>
-      <c r="E75" s="2"/>
-      <c r="F75" s="2">
-        <v>1</v>
-      </c>
-      <c r="G75" s="2">
-        <v>1</v>
-      </c>
-      <c r="H75" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="I75" s="2"/>
-      <c r="J75" s="2">
-        <v>10</v>
-      </c>
-      <c r="K75" s="2">
-        <v>0</v>
-      </c>
-      <c r="L75" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="M75" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="N75" s="4"/>
-      <c r="O75" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="P75" s="4"/>
-      <c r="Q75" s="2"/>
-      <c r="R75" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="S75" s="2"/>
-      <c r="T75" s="4"/>
-      <c r="U75" s="2"/>
-      <c r="V75" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="W75" s="2" t="s">
-        <v>144</v>
-      </c>
+      <c r="V74" s="6"/>
+      <c r="W74" s="6"/>
+    </row>
+    <row r="75" spans="1:23" outlineLevel="1">
+      <c r="A75" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="B75" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="C75" s="5">
+        <v>0</v>
+      </c>
+      <c r="D75" s="5"/>
+      <c r="E75" s="5"/>
+      <c r="F75" s="6">
+        <v>2</v>
+      </c>
+      <c r="G75" s="6">
+        <v>0</v>
+      </c>
+      <c r="H75" s="6" t="s">
+        <v>146</v>
+      </c>
+      <c r="I75" s="6"/>
+      <c r="J75" s="6">
+        <v>1</v>
+      </c>
+      <c r="K75" s="6">
+        <v>0</v>
+      </c>
+      <c r="L75" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="M75" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="N75" s="8"/>
+      <c r="O75" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="P75" s="8"/>
+      <c r="Q75" s="6"/>
+      <c r="R75" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="S75" s="6"/>
+      <c r="T75" s="8"/>
+      <c r="U75" s="6"/>
+      <c r="V75" s="6"/>
+      <c r="W75" s="6"/>
     </row>
     <row r="76" spans="1:23" outlineLevel="1">
       <c r="A76" s="5" t="s">
-        <v>150</v>
+        <v>136</v>
       </c>
       <c r="B76" s="5" t="s">
-        <v>151</v>
+        <v>137</v>
       </c>
       <c r="C76" s="5">
         <v>0</v>
@@ -4820,14 +4850,14 @@
         <v>2</v>
       </c>
       <c r="G76" s="6">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H76" s="6" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="I76" s="6"/>
       <c r="J76" s="6">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="K76" s="6">
         <v>0</v>
@@ -4850,19 +4880,15 @@
       <c r="S76" s="6"/>
       <c r="T76" s="8"/>
       <c r="U76" s="6"/>
-      <c r="V76" s="6" t="s">
-        <v>143</v>
-      </c>
-      <c r="W76" s="6" t="s">
-        <v>144</v>
-      </c>
+      <c r="V76" s="6"/>
+      <c r="W76" s="6"/>
     </row>
     <row r="77" spans="1:23" outlineLevel="1">
       <c r="A77" s="5" t="s">
-        <v>150</v>
+        <v>136</v>
       </c>
       <c r="B77" s="5" t="s">
-        <v>151</v>
+        <v>137</v>
       </c>
       <c r="C77" s="5">
         <v>0</v>
@@ -4870,17 +4896,17 @@
       <c r="D77" s="5"/>
       <c r="E77" s="5"/>
       <c r="F77" s="6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G77" s="6">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H77" s="6" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="I77" s="6"/>
       <c r="J77" s="6">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="K77" s="6">
         <v>0</v>
@@ -4903,19 +4929,15 @@
       <c r="S77" s="6"/>
       <c r="T77" s="8"/>
       <c r="U77" s="6"/>
-      <c r="V77" s="6" t="s">
-        <v>143</v>
-      </c>
-      <c r="W77" s="6" t="s">
-        <v>144</v>
-      </c>
+      <c r="V77" s="6"/>
+      <c r="W77" s="6"/>
     </row>
     <row r="78" spans="1:23" outlineLevel="1">
       <c r="A78" s="5" t="s">
-        <v>150</v>
+        <v>136</v>
       </c>
       <c r="B78" s="5" t="s">
-        <v>151</v>
+        <v>137</v>
       </c>
       <c r="C78" s="5">
         <v>0</v>
@@ -4923,17 +4945,17 @@
       <c r="D78" s="5"/>
       <c r="E78" s="5"/>
       <c r="F78" s="6">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G78" s="6">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="H78" s="6" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="I78" s="6"/>
       <c r="J78" s="6">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="K78" s="6">
         <v>0</v>
@@ -4956,19 +4978,15 @@
       <c r="S78" s="6"/>
       <c r="T78" s="8"/>
       <c r="U78" s="6"/>
-      <c r="V78" s="6" t="s">
-        <v>143</v>
-      </c>
-      <c r="W78" s="6" t="s">
-        <v>144</v>
-      </c>
+      <c r="V78" s="6"/>
+      <c r="W78" s="6"/>
     </row>
     <row r="79" spans="1:23" outlineLevel="1">
       <c r="A79" s="5" t="s">
-        <v>150</v>
+        <v>136</v>
       </c>
       <c r="B79" s="5" t="s">
-        <v>151</v>
+        <v>137</v>
       </c>
       <c r="C79" s="5">
         <v>0</v>
@@ -4976,17 +4994,17 @@
       <c r="D79" s="5"/>
       <c r="E79" s="5"/>
       <c r="F79" s="6">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G79" s="6">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H79" s="6" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="I79" s="6"/>
       <c r="J79" s="6">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="K79" s="6">
         <v>0</v>
@@ -5009,19 +5027,15 @@
       <c r="S79" s="6"/>
       <c r="T79" s="8"/>
       <c r="U79" s="6"/>
-      <c r="V79" s="6" t="s">
-        <v>143</v>
-      </c>
-      <c r="W79" s="6" t="s">
-        <v>144</v>
-      </c>
+      <c r="V79" s="6"/>
+      <c r="W79" s="6"/>
     </row>
     <row r="80" spans="1:23" outlineLevel="1">
       <c r="A80" s="5" t="s">
-        <v>150</v>
+        <v>136</v>
       </c>
       <c r="B80" s="5" t="s">
-        <v>151</v>
+        <v>137</v>
       </c>
       <c r="C80" s="5">
         <v>0</v>
@@ -5029,17 +5043,17 @@
       <c r="D80" s="5"/>
       <c r="E80" s="5"/>
       <c r="F80" s="6">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="G80" s="6">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H80" s="6" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="I80" s="6"/>
       <c r="J80" s="6">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="K80" s="6">
         <v>0</v>
@@ -5062,70 +5076,64 @@
       <c r="S80" s="6"/>
       <c r="T80" s="8"/>
       <c r="U80" s="6"/>
-      <c r="V80" s="6" t="s">
-        <v>143</v>
-      </c>
-      <c r="W80" s="6" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="81" spans="1:23">
-      <c r="A81" s="2" t="s">
+      <c r="V80" s="6"/>
+      <c r="W80" s="6"/>
+    </row>
+    <row r="81" spans="1:23" outlineLevel="1">
+      <c r="A81" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="B81" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="C81" s="5">
+        <v>0</v>
+      </c>
+      <c r="D81" s="5"/>
+      <c r="E81" s="5"/>
+      <c r="F81" s="6">
+        <v>2</v>
+      </c>
+      <c r="G81" s="6">
+        <v>6</v>
+      </c>
+      <c r="H81" s="6" t="s">
         <v>152</v>
       </c>
-      <c r="B81" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="C81" s="2">
-        <v>0</v>
-      </c>
-      <c r="D81" s="2"/>
-      <c r="E81" s="2"/>
-      <c r="F81" s="2">
-        <v>1</v>
-      </c>
-      <c r="G81" s="2">
-        <v>0</v>
-      </c>
-      <c r="H81" s="2" t="s">
-        <v>154</v>
-      </c>
-      <c r="I81" s="2"/>
-      <c r="J81" s="2">
-        <v>16</v>
-      </c>
-      <c r="K81" s="2">
-        <v>0</v>
-      </c>
-      <c r="L81" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="M81" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="N81" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="O81" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="P81" s="4"/>
-      <c r="Q81" s="2"/>
-      <c r="R81" s="4"/>
-      <c r="S81" s="2"/>
-      <c r="T81" s="4"/>
-      <c r="U81" s="2"/>
-      <c r="V81" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="W81" s="2"/>
+      <c r="I81" s="6"/>
+      <c r="J81" s="6">
+        <v>1</v>
+      </c>
+      <c r="K81" s="6">
+        <v>0</v>
+      </c>
+      <c r="L81" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="M81" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="N81" s="8"/>
+      <c r="O81" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="P81" s="8"/>
+      <c r="Q81" s="6"/>
+      <c r="R81" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="S81" s="6"/>
+      <c r="T81" s="8"/>
+      <c r="U81" s="6"/>
+      <c r="V81" s="6"/>
+      <c r="W81" s="6"/>
     </row>
     <row r="82" spans="1:23" outlineLevel="1">
       <c r="A82" s="5" t="s">
-        <v>152</v>
+        <v>136</v>
       </c>
       <c r="B82" s="5" t="s">
-        <v>153</v>
+        <v>137</v>
       </c>
       <c r="C82" s="5">
         <v>0</v>
@@ -5133,17 +5141,17 @@
       <c r="D82" s="5"/>
       <c r="E82" s="5"/>
       <c r="F82" s="6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G82" s="6">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="H82" s="6" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="I82" s="6"/>
       <c r="J82" s="6">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="K82" s="6">
         <v>0</v>
@@ -5154,29 +5162,27 @@
       <c r="M82" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="N82" s="7" t="s">
-        <v>25</v>
-      </c>
+      <c r="N82" s="8"/>
       <c r="O82" s="6" t="s">
         <v>26</v>
       </c>
       <c r="P82" s="8"/>
       <c r="Q82" s="6"/>
-      <c r="R82" s="8"/>
+      <c r="R82" s="7" t="s">
+        <v>25</v>
+      </c>
       <c r="S82" s="6"/>
       <c r="T82" s="8"/>
       <c r="U82" s="6"/>
-      <c r="V82" s="6" t="s">
-        <v>30</v>
-      </c>
+      <c r="V82" s="6"/>
       <c r="W82" s="6"/>
     </row>
     <row r="83" spans="1:23" outlineLevel="1">
       <c r="A83" s="5" t="s">
-        <v>152</v>
+        <v>136</v>
       </c>
       <c r="B83" s="5" t="s">
-        <v>153</v>
+        <v>137</v>
       </c>
       <c r="C83" s="5">
         <v>0</v>
@@ -5184,17 +5190,17 @@
       <c r="D83" s="5"/>
       <c r="E83" s="5"/>
       <c r="F83" s="6">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G83" s="6">
         <v>0</v>
       </c>
       <c r="H83" s="6" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="I83" s="6"/>
       <c r="J83" s="6">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="K83" s="6">
         <v>0</v>
@@ -5205,29 +5211,27 @@
       <c r="M83" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="N83" s="7" t="s">
-        <v>25</v>
-      </c>
+      <c r="N83" s="8"/>
       <c r="O83" s="6" t="s">
         <v>26</v>
       </c>
       <c r="P83" s="8"/>
       <c r="Q83" s="6"/>
-      <c r="R83" s="8"/>
+      <c r="R83" s="7" t="s">
+        <v>25</v>
+      </c>
       <c r="S83" s="6"/>
       <c r="T83" s="8"/>
       <c r="U83" s="6"/>
-      <c r="V83" s="6" t="s">
-        <v>30</v>
-      </c>
+      <c r="V83" s="6"/>
       <c r="W83" s="6"/>
     </row>
     <row r="84" spans="1:23" outlineLevel="1">
       <c r="A84" s="5" t="s">
-        <v>152</v>
+        <v>136</v>
       </c>
       <c r="B84" s="5" t="s">
-        <v>153</v>
+        <v>137</v>
       </c>
       <c r="C84" s="5">
         <v>0</v>
@@ -5235,17 +5239,17 @@
       <c r="D84" s="5"/>
       <c r="E84" s="5"/>
       <c r="F84" s="6">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="G84" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H84" s="6" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="I84" s="6"/>
       <c r="J84" s="6">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="K84" s="6">
         <v>0</v>
@@ -5256,80 +5260,76 @@
       <c r="M84" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="N84" s="7" t="s">
-        <v>25</v>
-      </c>
+      <c r="N84" s="8"/>
       <c r="O84" s="6" t="s">
         <v>26</v>
       </c>
       <c r="P84" s="8"/>
       <c r="Q84" s="6"/>
-      <c r="R84" s="8"/>
+      <c r="R84" s="7" t="s">
+        <v>25</v>
+      </c>
       <c r="S84" s="6"/>
       <c r="T84" s="8"/>
       <c r="U84" s="6"/>
-      <c r="V84" s="6" t="s">
-        <v>30</v>
-      </c>
+      <c r="V84" s="6"/>
       <c r="W84" s="6"/>
     </row>
-    <row r="85" spans="1:23">
-      <c r="A85" s="2" t="s">
-        <v>158</v>
-      </c>
-      <c r="B85" s="2" t="s">
-        <v>159</v>
-      </c>
-      <c r="C85" s="2">
-        <v>0</v>
-      </c>
-      <c r="D85" s="2"/>
-      <c r="E85" s="2"/>
-      <c r="F85" s="2">
-        <v>1</v>
-      </c>
-      <c r="G85" s="2">
-        <v>0</v>
-      </c>
-      <c r="H85" s="2" t="s">
-        <v>160</v>
-      </c>
-      <c r="I85" s="2"/>
-      <c r="J85" s="2">
-        <v>16</v>
-      </c>
-      <c r="K85" s="2">
-        <v>0</v>
-      </c>
-      <c r="L85" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="M85" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="N85" s="4"/>
-      <c r="O85" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="P85" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q85" s="2"/>
-      <c r="R85" s="4"/>
-      <c r="S85" s="2"/>
-      <c r="T85" s="4"/>
-      <c r="U85" s="2"/>
-      <c r="V85" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="W85" s="2"/>
+    <row r="85" spans="1:23" outlineLevel="1">
+      <c r="A85" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="B85" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="C85" s="5">
+        <v>0</v>
+      </c>
+      <c r="D85" s="5"/>
+      <c r="E85" s="5"/>
+      <c r="F85" s="6">
+        <v>3</v>
+      </c>
+      <c r="G85" s="6">
+        <v>2</v>
+      </c>
+      <c r="H85" s="6" t="s">
+        <v>156</v>
+      </c>
+      <c r="I85" s="6"/>
+      <c r="J85" s="6">
+        <v>1</v>
+      </c>
+      <c r="K85" s="6">
+        <v>0</v>
+      </c>
+      <c r="L85" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="M85" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="N85" s="8"/>
+      <c r="O85" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="P85" s="8"/>
+      <c r="Q85" s="6"/>
+      <c r="R85" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="S85" s="6"/>
+      <c r="T85" s="8"/>
+      <c r="U85" s="6"/>
+      <c r="V85" s="6"/>
+      <c r="W85" s="6"/>
     </row>
     <row r="86" spans="1:23" outlineLevel="1">
       <c r="A86" s="5" t="s">
-        <v>158</v>
+        <v>136</v>
       </c>
       <c r="B86" s="5" t="s">
-        <v>159</v>
+        <v>137</v>
       </c>
       <c r="C86" s="5">
         <v>0</v>
@@ -5340,14 +5340,14 @@
         <v>3</v>
       </c>
       <c r="G86" s="6">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H86" s="6" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="I86" s="6"/>
       <c r="J86" s="6">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="K86" s="6">
         <v>0</v>
@@ -5362,25 +5362,23 @@
       <c r="O86" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="P86" s="7" t="s">
-        <v>25</v>
-      </c>
+      <c r="P86" s="8"/>
       <c r="Q86" s="6"/>
-      <c r="R86" s="8"/>
+      <c r="R86" s="7" t="s">
+        <v>25</v>
+      </c>
       <c r="S86" s="6"/>
       <c r="T86" s="8"/>
       <c r="U86" s="6"/>
-      <c r="V86" s="6" t="s">
-        <v>30</v>
-      </c>
+      <c r="V86" s="6"/>
       <c r="W86" s="6"/>
     </row>
     <row r="87" spans="1:23" outlineLevel="1">
       <c r="A87" s="5" t="s">
-        <v>158</v>
+        <v>136</v>
       </c>
       <c r="B87" s="5" t="s">
-        <v>159</v>
+        <v>137</v>
       </c>
       <c r="C87" s="5">
         <v>0</v>
@@ -5388,17 +5386,17 @@
       <c r="D87" s="5"/>
       <c r="E87" s="5"/>
       <c r="F87" s="6">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G87" s="6">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H87" s="6" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="I87" s="6"/>
       <c r="J87" s="6">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="K87" s="6">
         <v>0</v>
@@ -5413,25 +5411,23 @@
       <c r="O87" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="P87" s="7" t="s">
-        <v>25</v>
-      </c>
+      <c r="P87" s="8"/>
       <c r="Q87" s="6"/>
-      <c r="R87" s="8"/>
+      <c r="R87" s="7" t="s">
+        <v>25</v>
+      </c>
       <c r="S87" s="6"/>
       <c r="T87" s="8"/>
       <c r="U87" s="6"/>
-      <c r="V87" s="6" t="s">
-        <v>30</v>
-      </c>
+      <c r="V87" s="6"/>
       <c r="W87" s="6"/>
     </row>
     <row r="88" spans="1:23" outlineLevel="1">
       <c r="A88" s="5" t="s">
-        <v>158</v>
+        <v>136</v>
       </c>
       <c r="B88" s="5" t="s">
-        <v>159</v>
+        <v>137</v>
       </c>
       <c r="C88" s="5">
         <v>0</v>
@@ -5439,17 +5435,17 @@
       <c r="D88" s="5"/>
       <c r="E88" s="5"/>
       <c r="F88" s="6">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="G88" s="6">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H88" s="6" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="I88" s="6"/>
       <c r="J88" s="6">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="K88" s="6">
         <v>0</v>
@@ -5464,25 +5460,23 @@
       <c r="O88" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="P88" s="7" t="s">
-        <v>25</v>
-      </c>
+      <c r="P88" s="8"/>
       <c r="Q88" s="6"/>
-      <c r="R88" s="8"/>
+      <c r="R88" s="7" t="s">
+        <v>25</v>
+      </c>
       <c r="S88" s="6"/>
       <c r="T88" s="8"/>
       <c r="U88" s="6"/>
-      <c r="V88" s="6" t="s">
-        <v>30</v>
-      </c>
+      <c r="V88" s="6"/>
       <c r="W88" s="6"/>
     </row>
     <row r="89" spans="1:23">
       <c r="A89" s="2" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="B89" s="2" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="C89" s="2">
         <v>0</v>
@@ -5493,14 +5487,14 @@
         <v>1</v>
       </c>
       <c r="G89" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H89" s="2" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="I89" s="2"/>
       <c r="J89" s="2">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="K89" s="2">
         <v>0</v>
@@ -5512,26 +5506,30 @@
         <v>29</v>
       </c>
       <c r="N89" s="4"/>
-      <c r="O89" s="9" t="s">
-        <v>25</v>
+      <c r="O89" s="2" t="s">
+        <v>26</v>
       </c>
       <c r="P89" s="4"/>
       <c r="Q89" s="2"/>
-      <c r="R89" s="4"/>
-      <c r="S89" s="2" t="s">
-        <v>26</v>
-      </c>
+      <c r="R89" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="S89" s="2"/>
       <c r="T89" s="4"/>
       <c r="U89" s="2"/>
-      <c r="V89" s="2"/>
-      <c r="W89" s="2"/>
+      <c r="V89" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="W89" s="2" t="s">
+        <v>164</v>
+      </c>
     </row>
     <row r="90" spans="1:23" outlineLevel="1">
       <c r="A90" s="5" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="B90" s="5" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="C90" s="5">
         <v>0</v>
@@ -5542,14 +5540,14 @@
         <v>2</v>
       </c>
       <c r="G90" s="6">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H90" s="6" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="I90" s="6"/>
       <c r="J90" s="6">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="K90" s="6">
         <v>0</v>
@@ -5561,28 +5559,30 @@
         <v>29</v>
       </c>
       <c r="N90" s="8"/>
-      <c r="O90" s="10" t="s">
-        <v>25</v>
+      <c r="O90" s="6" t="s">
+        <v>26</v>
       </c>
       <c r="P90" s="8"/>
       <c r="Q90" s="6"/>
-      <c r="R90" s="8"/>
-      <c r="S90" s="6" t="s">
-        <v>26</v>
-      </c>
+      <c r="R90" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="S90" s="6"/>
       <c r="T90" s="8"/>
       <c r="U90" s="6"/>
       <c r="V90" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="W90" s="6"/>
+        <v>163</v>
+      </c>
+      <c r="W90" s="6" t="s">
+        <v>164</v>
+      </c>
     </row>
     <row r="91" spans="1:23" outlineLevel="1">
       <c r="A91" s="5" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="B91" s="5" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="C91" s="5">
         <v>0</v>
@@ -5593,14 +5593,14 @@
         <v>3</v>
       </c>
       <c r="G91" s="6">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H91" s="6" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="I91" s="6"/>
       <c r="J91" s="6">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="K91" s="6">
         <v>0</v>
@@ -5612,81 +5612,83 @@
         <v>29</v>
       </c>
       <c r="N91" s="8"/>
-      <c r="O91" s="10" t="s">
-        <v>25</v>
+      <c r="O91" s="6" t="s">
+        <v>26</v>
       </c>
       <c r="P91" s="8"/>
       <c r="Q91" s="6"/>
-      <c r="R91" s="8"/>
-      <c r="S91" s="6" t="s">
-        <v>26</v>
-      </c>
+      <c r="R91" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="S91" s="6"/>
       <c r="T91" s="8"/>
       <c r="U91" s="6"/>
       <c r="V91" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="W91" s="6"/>
-    </row>
-    <row r="92" spans="1:23">
-      <c r="A92" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="B92" s="2" t="s">
-        <v>170</v>
-      </c>
-      <c r="C92" s="2">
-        <v>0</v>
-      </c>
-      <c r="D92" s="2"/>
-      <c r="E92" s="2"/>
-      <c r="F92" s="2">
-        <v>1</v>
-      </c>
-      <c r="G92" s="2">
-        <v>0</v>
-      </c>
-      <c r="H92" s="2" t="s">
-        <v>171</v>
-      </c>
-      <c r="I92" s="2"/>
-      <c r="J92" s="2">
+        <v>163</v>
+      </c>
+      <c r="W91" s="6" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="92" spans="1:23" outlineLevel="1">
+      <c r="A92" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="B92" s="5" t="s">
+        <v>161</v>
+      </c>
+      <c r="C92" s="5">
+        <v>0</v>
+      </c>
+      <c r="D92" s="5"/>
+      <c r="E92" s="5"/>
+      <c r="F92" s="6">
+        <v>4</v>
+      </c>
+      <c r="G92" s="6">
+        <v>7</v>
+      </c>
+      <c r="H92" s="6" t="s">
+        <v>167</v>
+      </c>
+      <c r="I92" s="6"/>
+      <c r="J92" s="6">
         <v>10</v>
       </c>
-      <c r="K92" s="2">
-        <v>0</v>
-      </c>
-      <c r="L92" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="M92" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="N92" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="O92" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="P92" s="4"/>
-      <c r="Q92" s="2"/>
-      <c r="R92" s="4"/>
-      <c r="S92" s="2"/>
-      <c r="T92" s="4"/>
-      <c r="U92" s="2"/>
-      <c r="V92" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="W92" s="2" t="s">
-        <v>144</v>
+      <c r="K92" s="6">
+        <v>0</v>
+      </c>
+      <c r="L92" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="M92" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="N92" s="8"/>
+      <c r="O92" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="P92" s="8"/>
+      <c r="Q92" s="6"/>
+      <c r="R92" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="S92" s="6"/>
+      <c r="T92" s="8"/>
+      <c r="U92" s="6"/>
+      <c r="V92" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="W92" s="6" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="93" spans="1:23" outlineLevel="1">
       <c r="A93" s="5" t="s">
-        <v>169</v>
+        <v>160</v>
       </c>
       <c r="B93" s="5" t="s">
-        <v>170</v>
+        <v>161</v>
       </c>
       <c r="C93" s="5">
         <v>0</v>
@@ -5694,13 +5696,13 @@
       <c r="D93" s="5"/>
       <c r="E93" s="5"/>
       <c r="F93" s="6">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G93" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H93" s="6" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="I93" s="6"/>
       <c r="J93" s="6">
@@ -5715,31 +5717,31 @@
       <c r="M93" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="N93" s="7" t="s">
-        <v>25</v>
-      </c>
+      <c r="N93" s="8"/>
       <c r="O93" s="6" t="s">
         <v>26</v>
       </c>
       <c r="P93" s="8"/>
       <c r="Q93" s="6"/>
-      <c r="R93" s="8"/>
+      <c r="R93" s="7" t="s">
+        <v>25</v>
+      </c>
       <c r="S93" s="6"/>
       <c r="T93" s="8"/>
       <c r="U93" s="6"/>
       <c r="V93" s="6" t="s">
-        <v>143</v>
+        <v>163</v>
       </c>
       <c r="W93" s="6" t="s">
-        <v>144</v>
+        <v>164</v>
       </c>
     </row>
     <row r="94" spans="1:23" outlineLevel="1">
       <c r="A94" s="5" t="s">
-        <v>169</v>
+        <v>160</v>
       </c>
       <c r="B94" s="5" t="s">
-        <v>170</v>
+        <v>161</v>
       </c>
       <c r="C94" s="5">
         <v>0</v>
@@ -5747,13 +5749,13 @@
       <c r="D94" s="5"/>
       <c r="E94" s="5"/>
       <c r="F94" s="6">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="G94" s="6">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H94" s="6" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="I94" s="6"/>
       <c r="J94" s="6">
@@ -5768,84 +5770,84 @@
       <c r="M94" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="N94" s="7" t="s">
-        <v>25</v>
-      </c>
+      <c r="N94" s="8"/>
       <c r="O94" s="6" t="s">
         <v>26</v>
       </c>
       <c r="P94" s="8"/>
       <c r="Q94" s="6"/>
-      <c r="R94" s="8"/>
+      <c r="R94" s="7" t="s">
+        <v>25</v>
+      </c>
       <c r="S94" s="6"/>
       <c r="T94" s="8"/>
       <c r="U94" s="6"/>
       <c r="V94" s="6" t="s">
-        <v>143</v>
+        <v>163</v>
       </c>
       <c r="W94" s="6" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="95" spans="1:23" outlineLevel="1">
-      <c r="A95" s="5" t="s">
-        <v>169</v>
-      </c>
-      <c r="B95" s="5" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="95" spans="1:23">
+      <c r="A95" s="2" t="s">
         <v>170</v>
       </c>
-      <c r="C95" s="5">
-        <v>0</v>
-      </c>
-      <c r="D95" s="5"/>
-      <c r="E95" s="5"/>
-      <c r="F95" s="6">
-        <v>4</v>
-      </c>
-      <c r="G95" s="6">
-        <v>6</v>
-      </c>
-      <c r="H95" s="6" t="s">
-        <v>174</v>
-      </c>
-      <c r="I95" s="6"/>
-      <c r="J95" s="6">
+      <c r="B95" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="C95" s="2">
+        <v>0</v>
+      </c>
+      <c r="D95" s="2"/>
+      <c r="E95" s="2"/>
+      <c r="F95" s="2">
+        <v>1</v>
+      </c>
+      <c r="G95" s="2">
+        <v>1</v>
+      </c>
+      <c r="H95" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="I95" s="2"/>
+      <c r="J95" s="2">
         <v>10</v>
       </c>
-      <c r="K95" s="6">
-        <v>0</v>
-      </c>
-      <c r="L95" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="M95" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="N95" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="O95" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="P95" s="8"/>
-      <c r="Q95" s="6"/>
-      <c r="R95" s="8"/>
-      <c r="S95" s="6"/>
-      <c r="T95" s="8"/>
-      <c r="U95" s="6"/>
-      <c r="V95" s="6" t="s">
-        <v>143</v>
-      </c>
-      <c r="W95" s="6" t="s">
-        <v>144</v>
+      <c r="K95" s="2">
+        <v>0</v>
+      </c>
+      <c r="L95" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="M95" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="N95" s="4"/>
+      <c r="O95" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="P95" s="4"/>
+      <c r="Q95" s="2"/>
+      <c r="R95" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="S95" s="2"/>
+      <c r="T95" s="4"/>
+      <c r="U95" s="2"/>
+      <c r="V95" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="W95" s="2" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="96" spans="1:23" outlineLevel="1">
       <c r="A96" s="5" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="B96" s="5" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C96" s="5">
         <v>0</v>
@@ -5853,13 +5855,13 @@
       <c r="D96" s="5"/>
       <c r="E96" s="5"/>
       <c r="F96" s="6">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G96" s="6">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H96" s="6" t="s">
-        <v>175</v>
+        <v>165</v>
       </c>
       <c r="I96" s="6"/>
       <c r="J96" s="6">
@@ -5874,31 +5876,31 @@
       <c r="M96" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="N96" s="7" t="s">
-        <v>25</v>
-      </c>
+      <c r="N96" s="8"/>
       <c r="O96" s="6" t="s">
         <v>26</v>
       </c>
       <c r="P96" s="8"/>
       <c r="Q96" s="6"/>
-      <c r="R96" s="8"/>
+      <c r="R96" s="7" t="s">
+        <v>25</v>
+      </c>
       <c r="S96" s="6"/>
       <c r="T96" s="8"/>
       <c r="U96" s="6"/>
       <c r="V96" s="6" t="s">
-        <v>143</v>
+        <v>163</v>
       </c>
       <c r="W96" s="6" t="s">
-        <v>144</v>
+        <v>164</v>
       </c>
     </row>
     <row r="97" spans="1:23" outlineLevel="1">
       <c r="A97" s="5" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="B97" s="5" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C97" s="5">
         <v>0</v>
@@ -5906,13 +5908,13 @@
       <c r="D97" s="5"/>
       <c r="E97" s="5"/>
       <c r="F97" s="6">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="G97" s="6">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H97" s="6" t="s">
-        <v>176</v>
+        <v>166</v>
       </c>
       <c r="I97" s="6"/>
       <c r="J97" s="6">
@@ -5927,84 +5929,84 @@
       <c r="M97" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="N97" s="7" t="s">
-        <v>25</v>
-      </c>
+      <c r="N97" s="8"/>
       <c r="O97" s="6" t="s">
         <v>26</v>
       </c>
       <c r="P97" s="8"/>
       <c r="Q97" s="6"/>
-      <c r="R97" s="8"/>
+      <c r="R97" s="7" t="s">
+        <v>25</v>
+      </c>
       <c r="S97" s="6"/>
       <c r="T97" s="8"/>
       <c r="U97" s="6"/>
       <c r="V97" s="6" t="s">
-        <v>143</v>
+        <v>163</v>
       </c>
       <c r="W97" s="6" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="98" spans="1:23">
-      <c r="A98" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="B98" s="2" t="s">
-        <v>178</v>
-      </c>
-      <c r="C98" s="2">
-        <v>0</v>
-      </c>
-      <c r="D98" s="2"/>
-      <c r="E98" s="2"/>
-      <c r="F98" s="2">
-        <v>1</v>
-      </c>
-      <c r="G98" s="2">
-        <v>0</v>
-      </c>
-      <c r="H98" s="2" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="98" spans="1:23" outlineLevel="1">
+      <c r="A98" s="5" t="s">
+        <v>170</v>
+      </c>
+      <c r="B98" s="5" t="s">
         <v>171</v>
       </c>
-      <c r="I98" s="2"/>
-      <c r="J98" s="2">
+      <c r="C98" s="5">
+        <v>0</v>
+      </c>
+      <c r="D98" s="5"/>
+      <c r="E98" s="5"/>
+      <c r="F98" s="6">
+        <v>4</v>
+      </c>
+      <c r="G98" s="6">
+        <v>7</v>
+      </c>
+      <c r="H98" s="6" t="s">
+        <v>167</v>
+      </c>
+      <c r="I98" s="6"/>
+      <c r="J98" s="6">
         <v>10</v>
       </c>
-      <c r="K98" s="2">
-        <v>0</v>
-      </c>
-      <c r="L98" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="M98" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="N98" s="4"/>
-      <c r="O98" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="P98" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q98" s="2"/>
-      <c r="R98" s="4"/>
-      <c r="S98" s="2"/>
-      <c r="T98" s="4"/>
-      <c r="U98" s="2"/>
-      <c r="V98" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="W98" s="2" t="s">
-        <v>144</v>
+      <c r="K98" s="6">
+        <v>0</v>
+      </c>
+      <c r="L98" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="M98" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="N98" s="8"/>
+      <c r="O98" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="P98" s="8"/>
+      <c r="Q98" s="6"/>
+      <c r="R98" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="S98" s="6"/>
+      <c r="T98" s="8"/>
+      <c r="U98" s="6"/>
+      <c r="V98" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="W98" s="6" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="99" spans="1:23" outlineLevel="1">
       <c r="A99" s="5" t="s">
-        <v>177</v>
+        <v>170</v>
       </c>
       <c r="B99" s="5" t="s">
-        <v>178</v>
+        <v>171</v>
       </c>
       <c r="C99" s="5">
         <v>0</v>
@@ -6012,13 +6014,13 @@
       <c r="D99" s="5"/>
       <c r="E99" s="5"/>
       <c r="F99" s="6">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G99" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H99" s="6" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="I99" s="6"/>
       <c r="J99" s="6">
@@ -6037,27 +6039,27 @@
       <c r="O99" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="P99" s="7" t="s">
-        <v>25</v>
-      </c>
+      <c r="P99" s="8"/>
       <c r="Q99" s="6"/>
-      <c r="R99" s="8"/>
+      <c r="R99" s="7" t="s">
+        <v>25</v>
+      </c>
       <c r="S99" s="6"/>
       <c r="T99" s="8"/>
       <c r="U99" s="6"/>
       <c r="V99" s="6" t="s">
-        <v>143</v>
+        <v>163</v>
       </c>
       <c r="W99" s="6" t="s">
-        <v>144</v>
+        <v>164</v>
       </c>
     </row>
     <row r="100" spans="1:23" outlineLevel="1">
       <c r="A100" s="5" t="s">
-        <v>177</v>
+        <v>170</v>
       </c>
       <c r="B100" s="5" t="s">
-        <v>178</v>
+        <v>171</v>
       </c>
       <c r="C100" s="5">
         <v>0</v>
@@ -6065,13 +6067,13 @@
       <c r="D100" s="5"/>
       <c r="E100" s="5"/>
       <c r="F100" s="6">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="G100" s="6">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H100" s="6" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="I100" s="6"/>
       <c r="J100" s="6">
@@ -6090,80 +6092,78 @@
       <c r="O100" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="P100" s="7" t="s">
-        <v>25</v>
-      </c>
+      <c r="P100" s="8"/>
       <c r="Q100" s="6"/>
-      <c r="R100" s="8"/>
+      <c r="R100" s="7" t="s">
+        <v>25</v>
+      </c>
       <c r="S100" s="6"/>
       <c r="T100" s="8"/>
       <c r="U100" s="6"/>
       <c r="V100" s="6" t="s">
-        <v>143</v>
+        <v>163</v>
       </c>
       <c r="W100" s="6" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="101" spans="1:23" outlineLevel="1">
-      <c r="A101" s="5" t="s">
-        <v>177</v>
-      </c>
-      <c r="B101" s="5" t="s">
-        <v>178</v>
-      </c>
-      <c r="C101" s="5">
-        <v>0</v>
-      </c>
-      <c r="D101" s="5"/>
-      <c r="E101" s="5"/>
-      <c r="F101" s="6">
-        <v>4</v>
-      </c>
-      <c r="G101" s="6">
-        <v>6</v>
-      </c>
-      <c r="H101" s="6" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="101" spans="1:23">
+      <c r="A101" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="B101" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="C101" s="2">
+        <v>0</v>
+      </c>
+      <c r="D101" s="2"/>
+      <c r="E101" s="2"/>
+      <c r="F101" s="2">
+        <v>1</v>
+      </c>
+      <c r="G101" s="2">
+        <v>0</v>
+      </c>
+      <c r="H101" s="2" t="s">
         <v>174</v>
       </c>
-      <c r="I101" s="6"/>
-      <c r="J101" s="6">
-        <v>10</v>
-      </c>
-      <c r="K101" s="6">
-        <v>0</v>
-      </c>
-      <c r="L101" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="M101" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="N101" s="8"/>
-      <c r="O101" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="P101" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q101" s="6"/>
-      <c r="R101" s="8"/>
-      <c r="S101" s="6"/>
-      <c r="T101" s="8"/>
-      <c r="U101" s="6"/>
-      <c r="V101" s="6" t="s">
-        <v>143</v>
-      </c>
-      <c r="W101" s="6" t="s">
-        <v>144</v>
-      </c>
+      <c r="I101" s="2"/>
+      <c r="J101" s="2">
+        <v>16</v>
+      </c>
+      <c r="K101" s="2">
+        <v>0</v>
+      </c>
+      <c r="L101" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="M101" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="N101" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="O101" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="P101" s="4"/>
+      <c r="Q101" s="2"/>
+      <c r="R101" s="4"/>
+      <c r="S101" s="2"/>
+      <c r="T101" s="4"/>
+      <c r="U101" s="2"/>
+      <c r="V101" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="W101" s="2"/>
     </row>
     <row r="102" spans="1:23" outlineLevel="1">
       <c r="A102" s="5" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="B102" s="5" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
       <c r="C102" s="5">
         <v>0</v>
@@ -6171,17 +6171,17 @@
       <c r="D102" s="5"/>
       <c r="E102" s="5"/>
       <c r="F102" s="6">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G102" s="6">
         <v>0</v>
       </c>
       <c r="H102" s="6" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="I102" s="6"/>
       <c r="J102" s="6">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="K102" s="6">
         <v>0</v>
@@ -6192,31 +6192,29 @@
       <c r="M102" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="N102" s="8"/>
+      <c r="N102" s="7" t="s">
+        <v>25</v>
+      </c>
       <c r="O102" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="P102" s="7" t="s">
-        <v>25</v>
-      </c>
+      <c r="P102" s="8"/>
       <c r="Q102" s="6"/>
       <c r="R102" s="8"/>
       <c r="S102" s="6"/>
       <c r="T102" s="8"/>
       <c r="U102" s="6"/>
       <c r="V102" s="6" t="s">
-        <v>143</v>
-      </c>
-      <c r="W102" s="6" t="s">
-        <v>144</v>
-      </c>
+        <v>30</v>
+      </c>
+      <c r="W102" s="6"/>
     </row>
     <row r="103" spans="1:23" outlineLevel="1">
       <c r="A103" s="5" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="B103" s="5" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
       <c r="C103" s="5">
         <v>0</v>
@@ -6224,17 +6222,17 @@
       <c r="D103" s="5"/>
       <c r="E103" s="5"/>
       <c r="F103" s="6">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="G103" s="6">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H103" s="6" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="I103" s="6"/>
       <c r="J103" s="6">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="K103" s="6">
         <v>0</v>
@@ -6245,182 +6243,182 @@
       <c r="M103" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="N103" s="8"/>
+      <c r="N103" s="7" t="s">
+        <v>25</v>
+      </c>
       <c r="O103" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="P103" s="7" t="s">
-        <v>25</v>
-      </c>
+      <c r="P103" s="8"/>
       <c r="Q103" s="6"/>
       <c r="R103" s="8"/>
       <c r="S103" s="6"/>
       <c r="T103" s="8"/>
       <c r="U103" s="6"/>
       <c r="V103" s="6" t="s">
-        <v>143</v>
-      </c>
-      <c r="W103" s="6" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="104" spans="1:23">
-      <c r="A104" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="W103" s="6"/>
+    </row>
+    <row r="104" spans="1:23" outlineLevel="1">
+      <c r="A104" s="5" t="s">
+        <v>172</v>
+      </c>
+      <c r="B104" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="C104" s="5">
+        <v>0</v>
+      </c>
+      <c r="D104" s="5"/>
+      <c r="E104" s="5"/>
+      <c r="F104" s="6">
+        <v>7</v>
+      </c>
+      <c r="G104" s="6">
+        <v>0</v>
+      </c>
+      <c r="H104" s="6" t="s">
+        <v>177</v>
+      </c>
+      <c r="I104" s="6"/>
+      <c r="J104" s="6">
+        <v>16</v>
+      </c>
+      <c r="K104" s="6">
+        <v>0</v>
+      </c>
+      <c r="L104" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="M104" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="N104" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="O104" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="P104" s="8"/>
+      <c r="Q104" s="6"/>
+      <c r="R104" s="8"/>
+      <c r="S104" s="6"/>
+      <c r="T104" s="8"/>
+      <c r="U104" s="6"/>
+      <c r="V104" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="W104" s="6"/>
+    </row>
+    <row r="105" spans="1:23">
+      <c r="A105" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="B105" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="C105" s="2">
+        <v>0</v>
+      </c>
+      <c r="D105" s="2"/>
+      <c r="E105" s="2"/>
+      <c r="F105" s="2">
+        <v>1</v>
+      </c>
+      <c r="G105" s="2">
+        <v>0</v>
+      </c>
+      <c r="H105" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="I105" s="2"/>
+      <c r="J105" s="2">
+        <v>16</v>
+      </c>
+      <c r="K105" s="2">
+        <v>0</v>
+      </c>
+      <c r="L105" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="M105" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="N105" s="4"/>
+      <c r="O105" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="P105" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q105" s="2"/>
+      <c r="R105" s="4"/>
+      <c r="S105" s="2"/>
+      <c r="T105" s="4"/>
+      <c r="U105" s="2"/>
+      <c r="V105" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="W105" s="2"/>
+    </row>
+    <row r="106" spans="1:23" outlineLevel="1">
+      <c r="A106" s="5" t="s">
+        <v>178</v>
+      </c>
+      <c r="B106" s="5" t="s">
+        <v>179</v>
+      </c>
+      <c r="C106" s="5">
+        <v>0</v>
+      </c>
+      <c r="D106" s="5"/>
+      <c r="E106" s="5"/>
+      <c r="F106" s="6">
+        <v>3</v>
+      </c>
+      <c r="G106" s="6">
+        <v>0</v>
+      </c>
+      <c r="H106" s="6" t="s">
         <v>181</v>
       </c>
-      <c r="B104" s="2" t="s">
-        <v>182</v>
-      </c>
-      <c r="C104" s="2">
-        <v>0</v>
-      </c>
-      <c r="D104" s="2"/>
-      <c r="E104" s="2"/>
-      <c r="F104" s="2">
-        <v>1</v>
-      </c>
-      <c r="G104" s="2">
-        <v>0</v>
-      </c>
-      <c r="H104" s="2" t="s">
-        <v>183</v>
-      </c>
-      <c r="I104" s="2"/>
-      <c r="J104" s="2">
+      <c r="I106" s="6"/>
+      <c r="J106" s="6">
         <v>16</v>
       </c>
-      <c r="K104" s="2">
-        <v>0</v>
-      </c>
-      <c r="L104" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="M104" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="N104" s="4"/>
-      <c r="O104" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="P104" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q104" s="2"/>
-      <c r="R104" s="4"/>
-      <c r="S104" s="2"/>
-      <c r="T104" s="4"/>
-      <c r="U104" s="2"/>
-      <c r="V104" s="2" t="s">
+      <c r="K106" s="6">
+        <v>0</v>
+      </c>
+      <c r="L106" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="M106" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="N106" s="8"/>
+      <c r="O106" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="P106" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q106" s="6"/>
+      <c r="R106" s="8"/>
+      <c r="S106" s="6"/>
+      <c r="T106" s="8"/>
+      <c r="U106" s="6"/>
+      <c r="V106" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="W104" s="2"/>
-    </row>
-    <row r="105" spans="1:23" outlineLevel="1">
-      <c r="A105" s="5" t="s">
-        <v>181</v>
-      </c>
-      <c r="B105" s="5" t="s">
-        <v>182</v>
-      </c>
-      <c r="C105" s="5">
-        <v>0</v>
-      </c>
-      <c r="D105" s="5"/>
-      <c r="E105" s="5"/>
-      <c r="F105" s="6">
-        <v>3</v>
-      </c>
-      <c r="G105" s="6">
-        <v>0</v>
-      </c>
-      <c r="H105" s="6" t="s">
-        <v>184</v>
-      </c>
-      <c r="I105" s="6"/>
-      <c r="J105" s="6">
-        <v>16</v>
-      </c>
-      <c r="K105" s="6">
-        <v>0</v>
-      </c>
-      <c r="L105" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="M105" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="N105" s="8"/>
-      <c r="O105" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="P105" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q105" s="6"/>
-      <c r="R105" s="8"/>
-      <c r="S105" s="6"/>
-      <c r="T105" s="8"/>
-      <c r="U105" s="6"/>
-      <c r="V105" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="W105" s="6"/>
-    </row>
-    <row r="106" spans="1:23">
-      <c r="A106" s="2" t="s">
-        <v>185</v>
-      </c>
-      <c r="B106" s="2" t="s">
-        <v>186</v>
-      </c>
-      <c r="C106" s="2">
-        <v>0</v>
-      </c>
-      <c r="D106" s="2"/>
-      <c r="E106" s="2"/>
-      <c r="F106" s="2">
-        <v>1</v>
-      </c>
-      <c r="G106" s="2">
-        <v>0</v>
-      </c>
-      <c r="H106" s="2" t="s">
-        <v>187</v>
-      </c>
-      <c r="I106" s="2"/>
-      <c r="J106" s="2">
-        <v>1</v>
-      </c>
-      <c r="K106" s="2">
-        <v>0</v>
-      </c>
-      <c r="L106" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="M106" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="N106" s="4"/>
-      <c r="O106" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="P106" s="4"/>
-      <c r="Q106" s="2"/>
-      <c r="R106" s="4"/>
-      <c r="S106" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="T106" s="4"/>
-      <c r="U106" s="2"/>
-      <c r="V106" s="2"/>
-      <c r="W106" s="2"/>
+      <c r="W106" s="6"/>
     </row>
     <row r="107" spans="1:23" outlineLevel="1">
       <c r="A107" s="5" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
       <c r="B107" s="5" t="s">
-        <v>186</v>
+        <v>179</v>
       </c>
       <c r="C107" s="5">
         <v>0</v>
@@ -6428,17 +6426,17 @@
       <c r="D107" s="5"/>
       <c r="E107" s="5"/>
       <c r="F107" s="6">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G107" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H107" s="6" t="s">
-        <v>188</v>
+        <v>182</v>
       </c>
       <c r="I107" s="6"/>
       <c r="J107" s="6">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="K107" s="6">
         <v>0</v>
@@ -6453,23 +6451,25 @@
       <c r="O107" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="P107" s="8"/>
+      <c r="P107" s="7" t="s">
+        <v>25</v>
+      </c>
       <c r="Q107" s="6"/>
       <c r="R107" s="8"/>
-      <c r="S107" s="10" t="s">
-        <v>25</v>
-      </c>
+      <c r="S107" s="6"/>
       <c r="T107" s="8"/>
       <c r="U107" s="6"/>
-      <c r="V107" s="6"/>
+      <c r="V107" s="6" t="s">
+        <v>30</v>
+      </c>
       <c r="W107" s="6"/>
     </row>
     <row r="108" spans="1:23" outlineLevel="1">
       <c r="A108" s="5" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
       <c r="B108" s="5" t="s">
-        <v>186</v>
+        <v>179</v>
       </c>
       <c r="C108" s="5">
         <v>0</v>
@@ -6477,17 +6477,17 @@
       <c r="D108" s="5"/>
       <c r="E108" s="5"/>
       <c r="F108" s="6">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="G108" s="6">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H108" s="6" t="s">
-        <v>189</v>
+        <v>183</v>
       </c>
       <c r="I108" s="6"/>
       <c r="J108" s="6">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="K108" s="6">
         <v>0</v>
@@ -6502,68 +6502,1106 @@
       <c r="O108" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="P108" s="8"/>
+      <c r="P108" s="7" t="s">
+        <v>25</v>
+      </c>
       <c r="Q108" s="6"/>
       <c r="R108" s="8"/>
-      <c r="S108" s="10" t="s">
-        <v>25</v>
-      </c>
+      <c r="S108" s="6"/>
       <c r="T108" s="8"/>
       <c r="U108" s="6"/>
-      <c r="V108" s="6"/>
+      <c r="V108" s="6" t="s">
+        <v>30</v>
+      </c>
       <c r="W108" s="6"/>
     </row>
-    <row r="109" spans="1:23" outlineLevel="1">
-      <c r="A109" s="5" t="s">
+    <row r="109" spans="1:23">
+      <c r="A109" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="B109" s="2" t="s">
         <v>185</v>
       </c>
-      <c r="B109" s="5" t="s">
+      <c r="C109" s="2">
+        <v>0</v>
+      </c>
+      <c r="D109" s="2"/>
+      <c r="E109" s="2"/>
+      <c r="F109" s="2">
+        <v>1</v>
+      </c>
+      <c r="G109" s="2">
+        <v>0</v>
+      </c>
+      <c r="H109" s="2" t="s">
         <v>186</v>
       </c>
-      <c r="C109" s="5">
-        <v>0</v>
-      </c>
-      <c r="D109" s="5"/>
-      <c r="E109" s="5"/>
-      <c r="F109" s="6">
-        <v>1</v>
-      </c>
-      <c r="G109" s="6">
+      <c r="I109" s="2"/>
+      <c r="J109" s="2">
+        <v>1</v>
+      </c>
+      <c r="K109" s="2">
+        <v>0</v>
+      </c>
+      <c r="L109" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="M109" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="N109" s="4"/>
+      <c r="O109" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="P109" s="4"/>
+      <c r="Q109" s="2"/>
+      <c r="R109" s="4"/>
+      <c r="S109" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="T109" s="4"/>
+      <c r="U109" s="2"/>
+      <c r="V109" s="2"/>
+      <c r="W109" s="2"/>
+    </row>
+    <row r="110" spans="1:23" outlineLevel="1">
+      <c r="A110" s="5" t="s">
+        <v>184</v>
+      </c>
+      <c r="B110" s="5" t="s">
+        <v>185</v>
+      </c>
+      <c r="C110" s="5">
+        <v>0</v>
+      </c>
+      <c r="D110" s="5"/>
+      <c r="E110" s="5"/>
+      <c r="F110" s="6">
+        <v>2</v>
+      </c>
+      <c r="G110" s="6">
+        <v>0</v>
+      </c>
+      <c r="H110" s="6" t="s">
+        <v>187</v>
+      </c>
+      <c r="I110" s="6"/>
+      <c r="J110" s="6">
+        <v>8</v>
+      </c>
+      <c r="K110" s="6">
+        <v>0</v>
+      </c>
+      <c r="L110" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="M110" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="N110" s="8"/>
+      <c r="O110" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="P110" s="8"/>
+      <c r="Q110" s="6"/>
+      <c r="R110" s="8"/>
+      <c r="S110" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="T110" s="8"/>
+      <c r="U110" s="6"/>
+      <c r="V110" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="W110" s="6"/>
+    </row>
+    <row r="111" spans="1:23" outlineLevel="1">
+      <c r="A111" s="5" t="s">
+        <v>184</v>
+      </c>
+      <c r="B111" s="5" t="s">
+        <v>185</v>
+      </c>
+      <c r="C111" s="5">
+        <v>0</v>
+      </c>
+      <c r="D111" s="5"/>
+      <c r="E111" s="5"/>
+      <c r="F111" s="6">
         <v>3</v>
       </c>
-      <c r="H109" s="6" t="s">
+      <c r="G111" s="6">
+        <v>0</v>
+      </c>
+      <c r="H111" s="6" t="s">
+        <v>188</v>
+      </c>
+      <c r="I111" s="6"/>
+      <c r="J111" s="6">
+        <v>8</v>
+      </c>
+      <c r="K111" s="6">
+        <v>0</v>
+      </c>
+      <c r="L111" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="M111" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="N111" s="8"/>
+      <c r="O111" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="P111" s="8"/>
+      <c r="Q111" s="6"/>
+      <c r="R111" s="8"/>
+      <c r="S111" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="T111" s="8"/>
+      <c r="U111" s="6"/>
+      <c r="V111" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="W111" s="6"/>
+    </row>
+    <row r="112" spans="1:23">
+      <c r="A112" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="B112" s="2" t="s">
         <v>190</v>
       </c>
-      <c r="I109" s="6"/>
-      <c r="J109" s="6">
-        <v>1</v>
-      </c>
-      <c r="K109" s="6">
-        <v>0</v>
-      </c>
-      <c r="L109" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="M109" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="N109" s="8"/>
-      <c r="O109" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="P109" s="8"/>
-      <c r="Q109" s="6"/>
-      <c r="R109" s="8"/>
-      <c r="S109" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="T109" s="8"/>
-      <c r="U109" s="6"/>
-      <c r="V109" s="6"/>
-      <c r="W109" s="6"/>
+      <c r="C112" s="2">
+        <v>0</v>
+      </c>
+      <c r="D112" s="2"/>
+      <c r="E112" s="2"/>
+      <c r="F112" s="2">
+        <v>1</v>
+      </c>
+      <c r="G112" s="2">
+        <v>0</v>
+      </c>
+      <c r="H112" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="I112" s="2"/>
+      <c r="J112" s="2">
+        <v>10</v>
+      </c>
+      <c r="K112" s="2">
+        <v>0</v>
+      </c>
+      <c r="L112" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="M112" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="N112" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="O112" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="P112" s="4"/>
+      <c r="Q112" s="2"/>
+      <c r="R112" s="4"/>
+      <c r="S112" s="2"/>
+      <c r="T112" s="4"/>
+      <c r="U112" s="2"/>
+      <c r="V112" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="W112" s="2" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="113" spans="1:23" outlineLevel="1">
+      <c r="A113" s="5" t="s">
+        <v>189</v>
+      </c>
+      <c r="B113" s="5" t="s">
+        <v>190</v>
+      </c>
+      <c r="C113" s="5">
+        <v>0</v>
+      </c>
+      <c r="D113" s="5"/>
+      <c r="E113" s="5"/>
+      <c r="F113" s="6">
+        <v>2</v>
+      </c>
+      <c r="G113" s="6">
+        <v>2</v>
+      </c>
+      <c r="H113" s="6" t="s">
+        <v>192</v>
+      </c>
+      <c r="I113" s="6"/>
+      <c r="J113" s="6">
+        <v>10</v>
+      </c>
+      <c r="K113" s="6">
+        <v>0</v>
+      </c>
+      <c r="L113" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="M113" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="N113" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="O113" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="P113" s="8"/>
+      <c r="Q113" s="6"/>
+      <c r="R113" s="8"/>
+      <c r="S113" s="6"/>
+      <c r="T113" s="8"/>
+      <c r="U113" s="6"/>
+      <c r="V113" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="W113" s="6" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="114" spans="1:23" outlineLevel="1">
+      <c r="A114" s="5" t="s">
+        <v>189</v>
+      </c>
+      <c r="B114" s="5" t="s">
+        <v>190</v>
+      </c>
+      <c r="C114" s="5">
+        <v>0</v>
+      </c>
+      <c r="D114" s="5"/>
+      <c r="E114" s="5"/>
+      <c r="F114" s="6">
+        <v>3</v>
+      </c>
+      <c r="G114" s="6">
+        <v>4</v>
+      </c>
+      <c r="H114" s="6" t="s">
+        <v>193</v>
+      </c>
+      <c r="I114" s="6"/>
+      <c r="J114" s="6">
+        <v>10</v>
+      </c>
+      <c r="K114" s="6">
+        <v>0</v>
+      </c>
+      <c r="L114" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="M114" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="N114" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="O114" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="P114" s="8"/>
+      <c r="Q114" s="6"/>
+      <c r="R114" s="8"/>
+      <c r="S114" s="6"/>
+      <c r="T114" s="8"/>
+      <c r="U114" s="6"/>
+      <c r="V114" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="W114" s="6" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="115" spans="1:23" outlineLevel="1">
+      <c r="A115" s="5" t="s">
+        <v>189</v>
+      </c>
+      <c r="B115" s="5" t="s">
+        <v>190</v>
+      </c>
+      <c r="C115" s="5">
+        <v>0</v>
+      </c>
+      <c r="D115" s="5"/>
+      <c r="E115" s="5"/>
+      <c r="F115" s="6">
+        <v>4</v>
+      </c>
+      <c r="G115" s="6">
+        <v>6</v>
+      </c>
+      <c r="H115" s="6" t="s">
+        <v>194</v>
+      </c>
+      <c r="I115" s="6"/>
+      <c r="J115" s="6">
+        <v>10</v>
+      </c>
+      <c r="K115" s="6">
+        <v>0</v>
+      </c>
+      <c r="L115" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="M115" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="N115" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="O115" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="P115" s="8"/>
+      <c r="Q115" s="6"/>
+      <c r="R115" s="8"/>
+      <c r="S115" s="6"/>
+      <c r="T115" s="8"/>
+      <c r="U115" s="6"/>
+      <c r="V115" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="W115" s="6" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="116" spans="1:23" outlineLevel="1">
+      <c r="A116" s="5" t="s">
+        <v>189</v>
+      </c>
+      <c r="B116" s="5" t="s">
+        <v>190</v>
+      </c>
+      <c r="C116" s="5">
+        <v>0</v>
+      </c>
+      <c r="D116" s="5"/>
+      <c r="E116" s="5"/>
+      <c r="F116" s="6">
+        <v>6</v>
+      </c>
+      <c r="G116" s="6">
+        <v>0</v>
+      </c>
+      <c r="H116" s="6" t="s">
+        <v>195</v>
+      </c>
+      <c r="I116" s="6"/>
+      <c r="J116" s="6">
+        <v>10</v>
+      </c>
+      <c r="K116" s="6">
+        <v>0</v>
+      </c>
+      <c r="L116" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="M116" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="N116" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="O116" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="P116" s="8"/>
+      <c r="Q116" s="6"/>
+      <c r="R116" s="8"/>
+      <c r="S116" s="6"/>
+      <c r="T116" s="8"/>
+      <c r="U116" s="6"/>
+      <c r="V116" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="W116" s="6" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="117" spans="1:23" outlineLevel="1">
+      <c r="A117" s="5" t="s">
+        <v>189</v>
+      </c>
+      <c r="B117" s="5" t="s">
+        <v>190</v>
+      </c>
+      <c r="C117" s="5">
+        <v>0</v>
+      </c>
+      <c r="D117" s="5"/>
+      <c r="E117" s="5"/>
+      <c r="F117" s="6">
+        <v>7</v>
+      </c>
+      <c r="G117" s="6">
+        <v>2</v>
+      </c>
+      <c r="H117" s="6" t="s">
+        <v>196</v>
+      </c>
+      <c r="I117" s="6"/>
+      <c r="J117" s="6">
+        <v>10</v>
+      </c>
+      <c r="K117" s="6">
+        <v>0</v>
+      </c>
+      <c r="L117" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="M117" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="N117" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="O117" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="P117" s="8"/>
+      <c r="Q117" s="6"/>
+      <c r="R117" s="8"/>
+      <c r="S117" s="6"/>
+      <c r="T117" s="8"/>
+      <c r="U117" s="6"/>
+      <c r="V117" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="W117" s="6" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="118" spans="1:23">
+      <c r="A118" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="B118" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="C118" s="2">
+        <v>0</v>
+      </c>
+      <c r="D118" s="2"/>
+      <c r="E118" s="2"/>
+      <c r="F118" s="2">
+        <v>1</v>
+      </c>
+      <c r="G118" s="2">
+        <v>0</v>
+      </c>
+      <c r="H118" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="I118" s="2"/>
+      <c r="J118" s="2">
+        <v>10</v>
+      </c>
+      <c r="K118" s="2">
+        <v>0</v>
+      </c>
+      <c r="L118" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="M118" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="N118" s="4"/>
+      <c r="O118" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="P118" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q118" s="2"/>
+      <c r="R118" s="4"/>
+      <c r="S118" s="2"/>
+      <c r="T118" s="4"/>
+      <c r="U118" s="2"/>
+      <c r="V118" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="W118" s="2" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="119" spans="1:23" outlineLevel="1">
+      <c r="A119" s="5" t="s">
+        <v>197</v>
+      </c>
+      <c r="B119" s="5" t="s">
+        <v>198</v>
+      </c>
+      <c r="C119" s="5">
+        <v>0</v>
+      </c>
+      <c r="D119" s="5"/>
+      <c r="E119" s="5"/>
+      <c r="F119" s="6">
+        <v>2</v>
+      </c>
+      <c r="G119" s="6">
+        <v>2</v>
+      </c>
+      <c r="H119" s="6" t="s">
+        <v>192</v>
+      </c>
+      <c r="I119" s="6"/>
+      <c r="J119" s="6">
+        <v>10</v>
+      </c>
+      <c r="K119" s="6">
+        <v>0</v>
+      </c>
+      <c r="L119" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="M119" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="N119" s="8"/>
+      <c r="O119" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="P119" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q119" s="6"/>
+      <c r="R119" s="8"/>
+      <c r="S119" s="6"/>
+      <c r="T119" s="8"/>
+      <c r="U119" s="6"/>
+      <c r="V119" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="W119" s="6" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="120" spans="1:23" outlineLevel="1">
+      <c r="A120" s="5" t="s">
+        <v>197</v>
+      </c>
+      <c r="B120" s="5" t="s">
+        <v>198</v>
+      </c>
+      <c r="C120" s="5">
+        <v>0</v>
+      </c>
+      <c r="D120" s="5"/>
+      <c r="E120" s="5"/>
+      <c r="F120" s="6">
+        <v>3</v>
+      </c>
+      <c r="G120" s="6">
+        <v>4</v>
+      </c>
+      <c r="H120" s="6" t="s">
+        <v>193</v>
+      </c>
+      <c r="I120" s="6"/>
+      <c r="J120" s="6">
+        <v>10</v>
+      </c>
+      <c r="K120" s="6">
+        <v>0</v>
+      </c>
+      <c r="L120" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="M120" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="N120" s="8"/>
+      <c r="O120" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="P120" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q120" s="6"/>
+      <c r="R120" s="8"/>
+      <c r="S120" s="6"/>
+      <c r="T120" s="8"/>
+      <c r="U120" s="6"/>
+      <c r="V120" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="W120" s="6" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="121" spans="1:23" outlineLevel="1">
+      <c r="A121" s="5" t="s">
+        <v>197</v>
+      </c>
+      <c r="B121" s="5" t="s">
+        <v>198</v>
+      </c>
+      <c r="C121" s="5">
+        <v>0</v>
+      </c>
+      <c r="D121" s="5"/>
+      <c r="E121" s="5"/>
+      <c r="F121" s="6">
+        <v>4</v>
+      </c>
+      <c r="G121" s="6">
+        <v>6</v>
+      </c>
+      <c r="H121" s="6" t="s">
+        <v>194</v>
+      </c>
+      <c r="I121" s="6"/>
+      <c r="J121" s="6">
+        <v>10</v>
+      </c>
+      <c r="K121" s="6">
+        <v>0</v>
+      </c>
+      <c r="L121" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="M121" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="N121" s="8"/>
+      <c r="O121" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="P121" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q121" s="6"/>
+      <c r="R121" s="8"/>
+      <c r="S121" s="6"/>
+      <c r="T121" s="8"/>
+      <c r="U121" s="6"/>
+      <c r="V121" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="W121" s="6" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="122" spans="1:23" outlineLevel="1">
+      <c r="A122" s="5" t="s">
+        <v>197</v>
+      </c>
+      <c r="B122" s="5" t="s">
+        <v>198</v>
+      </c>
+      <c r="C122" s="5">
+        <v>0</v>
+      </c>
+      <c r="D122" s="5"/>
+      <c r="E122" s="5"/>
+      <c r="F122" s="6">
+        <v>6</v>
+      </c>
+      <c r="G122" s="6">
+        <v>0</v>
+      </c>
+      <c r="H122" s="6" t="s">
+        <v>199</v>
+      </c>
+      <c r="I122" s="6"/>
+      <c r="J122" s="6">
+        <v>10</v>
+      </c>
+      <c r="K122" s="6">
+        <v>0</v>
+      </c>
+      <c r="L122" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="M122" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="N122" s="8"/>
+      <c r="O122" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="P122" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q122" s="6"/>
+      <c r="R122" s="8"/>
+      <c r="S122" s="6"/>
+      <c r="T122" s="8"/>
+      <c r="U122" s="6"/>
+      <c r="V122" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="W122" s="6" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="123" spans="1:23" outlineLevel="1">
+      <c r="A123" s="5" t="s">
+        <v>197</v>
+      </c>
+      <c r="B123" s="5" t="s">
+        <v>198</v>
+      </c>
+      <c r="C123" s="5">
+        <v>0</v>
+      </c>
+      <c r="D123" s="5"/>
+      <c r="E123" s="5"/>
+      <c r="F123" s="6">
+        <v>7</v>
+      </c>
+      <c r="G123" s="6">
+        <v>2</v>
+      </c>
+      <c r="H123" s="6" t="s">
+        <v>200</v>
+      </c>
+      <c r="I123" s="6"/>
+      <c r="J123" s="6">
+        <v>10</v>
+      </c>
+      <c r="K123" s="6">
+        <v>0</v>
+      </c>
+      <c r="L123" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="M123" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="N123" s="8"/>
+      <c r="O123" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="P123" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q123" s="6"/>
+      <c r="R123" s="8"/>
+      <c r="S123" s="6"/>
+      <c r="T123" s="8"/>
+      <c r="U123" s="6"/>
+      <c r="V123" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="W123" s="6" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="124" spans="1:23">
+      <c r="A124" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="B124" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="C124" s="2">
+        <v>0</v>
+      </c>
+      <c r="D124" s="2"/>
+      <c r="E124" s="2"/>
+      <c r="F124" s="2">
+        <v>1</v>
+      </c>
+      <c r="G124" s="2">
+        <v>0</v>
+      </c>
+      <c r="H124" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="I124" s="2"/>
+      <c r="J124" s="2">
+        <v>16</v>
+      </c>
+      <c r="K124" s="2">
+        <v>0</v>
+      </c>
+      <c r="L124" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="M124" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="N124" s="4"/>
+      <c r="O124" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="P124" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q124" s="2"/>
+      <c r="R124" s="4"/>
+      <c r="S124" s="2"/>
+      <c r="T124" s="4"/>
+      <c r="U124" s="2"/>
+      <c r="V124" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="W124" s="2"/>
+    </row>
+    <row r="125" spans="1:23" outlineLevel="1">
+      <c r="A125" s="5" t="s">
+        <v>201</v>
+      </c>
+      <c r="B125" s="5" t="s">
+        <v>202</v>
+      </c>
+      <c r="C125" s="5">
+        <v>0</v>
+      </c>
+      <c r="D125" s="5"/>
+      <c r="E125" s="5"/>
+      <c r="F125" s="6">
+        <v>3</v>
+      </c>
+      <c r="G125" s="6">
+        <v>0</v>
+      </c>
+      <c r="H125" s="6" t="s">
+        <v>204</v>
+      </c>
+      <c r="I125" s="6"/>
+      <c r="J125" s="6">
+        <v>16</v>
+      </c>
+      <c r="K125" s="6">
+        <v>0</v>
+      </c>
+      <c r="L125" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="M125" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="N125" s="8"/>
+      <c r="O125" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="P125" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q125" s="6"/>
+      <c r="R125" s="8"/>
+      <c r="S125" s="6"/>
+      <c r="T125" s="8"/>
+      <c r="U125" s="6"/>
+      <c r="V125" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="W125" s="6"/>
+    </row>
+    <row r="126" spans="1:23">
+      <c r="A126" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="B126" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="C126" s="2">
+        <v>0</v>
+      </c>
+      <c r="D126" s="2"/>
+      <c r="E126" s="2"/>
+      <c r="F126" s="2">
+        <v>1</v>
+      </c>
+      <c r="G126" s="2">
+        <v>0</v>
+      </c>
+      <c r="H126" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="I126" s="2"/>
+      <c r="J126" s="2">
+        <v>1</v>
+      </c>
+      <c r="K126" s="2">
+        <v>0</v>
+      </c>
+      <c r="L126" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="M126" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="N126" s="4"/>
+      <c r="O126" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="P126" s="4"/>
+      <c r="Q126" s="2"/>
+      <c r="R126" s="4"/>
+      <c r="S126" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="T126" s="4"/>
+      <c r="U126" s="2"/>
+      <c r="V126" s="2"/>
+      <c r="W126" s="2"/>
+    </row>
+    <row r="127" spans="1:23" outlineLevel="1">
+      <c r="A127" s="5" t="s">
+        <v>205</v>
+      </c>
+      <c r="B127" s="5" t="s">
+        <v>206</v>
+      </c>
+      <c r="C127" s="5">
+        <v>0</v>
+      </c>
+      <c r="D127" s="5"/>
+      <c r="E127" s="5"/>
+      <c r="F127" s="6">
+        <v>1</v>
+      </c>
+      <c r="G127" s="6">
+        <v>1</v>
+      </c>
+      <c r="H127" s="6" t="s">
+        <v>208</v>
+      </c>
+      <c r="I127" s="6"/>
+      <c r="J127" s="6">
+        <v>1</v>
+      </c>
+      <c r="K127" s="6">
+        <v>0</v>
+      </c>
+      <c r="L127" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="M127" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="N127" s="8"/>
+      <c r="O127" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="P127" s="8"/>
+      <c r="Q127" s="6"/>
+      <c r="R127" s="8"/>
+      <c r="S127" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="T127" s="8"/>
+      <c r="U127" s="6"/>
+      <c r="V127" s="6"/>
+      <c r="W127" s="6"/>
+    </row>
+    <row r="128" spans="1:23" outlineLevel="1">
+      <c r="A128" s="5" t="s">
+        <v>205</v>
+      </c>
+      <c r="B128" s="5" t="s">
+        <v>206</v>
+      </c>
+      <c r="C128" s="5">
+        <v>0</v>
+      </c>
+      <c r="D128" s="5"/>
+      <c r="E128" s="5"/>
+      <c r="F128" s="6">
+        <v>1</v>
+      </c>
+      <c r="G128" s="6">
+        <v>2</v>
+      </c>
+      <c r="H128" s="6" t="s">
+        <v>209</v>
+      </c>
+      <c r="I128" s="6"/>
+      <c r="J128" s="6">
+        <v>1</v>
+      </c>
+      <c r="K128" s="6">
+        <v>0</v>
+      </c>
+      <c r="L128" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="M128" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="N128" s="8"/>
+      <c r="O128" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="P128" s="8"/>
+      <c r="Q128" s="6"/>
+      <c r="R128" s="8"/>
+      <c r="S128" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="T128" s="8"/>
+      <c r="U128" s="6"/>
+      <c r="V128" s="6"/>
+      <c r="W128" s="6"/>
+    </row>
+    <row r="129" spans="1:23" outlineLevel="1">
+      <c r="A129" s="5" t="s">
+        <v>205</v>
+      </c>
+      <c r="B129" s="5" t="s">
+        <v>206</v>
+      </c>
+      <c r="C129" s="5">
+        <v>0</v>
+      </c>
+      <c r="D129" s="5"/>
+      <c r="E129" s="5"/>
+      <c r="F129" s="6">
+        <v>1</v>
+      </c>
+      <c r="G129" s="6">
+        <v>3</v>
+      </c>
+      <c r="H129" s="6" t="s">
+        <v>210</v>
+      </c>
+      <c r="I129" s="6"/>
+      <c r="J129" s="6">
+        <v>1</v>
+      </c>
+      <c r="K129" s="6">
+        <v>0</v>
+      </c>
+      <c r="L129" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="M129" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="N129" s="8"/>
+      <c r="O129" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="P129" s="8"/>
+      <c r="Q129" s="6"/>
+      <c r="R129" s="8"/>
+      <c r="S129" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="T129" s="8"/>
+      <c r="U129" s="6"/>
+      <c r="V129" s="6"/>
+      <c r="W129" s="6"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AH110"/>
+  <autoFilter ref="A1:AH130"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
generated from SC22EVO/MCB.json at bad310d
</commit_message>
<xml_diff>
--- a/SC22EVO/artifacts/MCB.xlsx
+++ b/SC22EVO/artifacts/MCB.xlsx
@@ -10,14 +10,14 @@
     <sheet name="K-Matrix " sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'K-Matrix '!$A$1:$AH$130</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'K-Matrix '!$A$1:$AH$135</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1022" uniqueCount="211">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1057" uniqueCount="216">
   <si>
     <t>ID</t>
   </si>
@@ -478,25 +478,40 @@
     <t>cell7_UV</t>
   </si>
   <si>
-    <t>cell1_OT</t>
-  </si>
-  <si>
-    <t>cell2_OT</t>
-  </si>
-  <si>
-    <t>cell3_OT</t>
-  </si>
-  <si>
-    <t>cell4_OT</t>
-  </si>
-  <si>
-    <t>cell5_OT</t>
-  </si>
-  <si>
-    <t>cell6_OT</t>
-  </si>
-  <si>
-    <t>cell7_OT</t>
+    <t>temp1_OT</t>
+  </si>
+  <si>
+    <t>temp2_OT</t>
+  </si>
+  <si>
+    <t>temp3_OT</t>
+  </si>
+  <si>
+    <t>temp4_OT</t>
+  </si>
+  <si>
+    <t>temp5_OT</t>
+  </si>
+  <si>
+    <t>temp6_OT</t>
+  </si>
+  <si>
+    <t>temp7_OT</t>
+  </si>
+  <si>
+    <t>temp8_OT</t>
+  </si>
+  <si>
+    <t>temp9_OT</t>
+  </si>
+  <si>
+    <t>temp10_OT</t>
+  </si>
+  <si>
+    <t>temp11_OT</t>
+  </si>
+  <si>
+    <t>temp12_OT</t>
   </si>
   <si>
     <t>104h</t>
@@ -1038,7 +1053,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W129"/>
+  <dimension ref="A1:W134"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="1"/>
   <cols>
     <col min="1" max="1" width="4.28515625" customWidth="1"/>
@@ -5471,65 +5486,61 @@
       <c r="V88" s="6"/>
       <c r="W88" s="6"/>
     </row>
-    <row r="89" spans="1:23">
-      <c r="A89" s="2" t="s">
+    <row r="89" spans="1:23" outlineLevel="1">
+      <c r="A89" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="B89" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="C89" s="5">
+        <v>0</v>
+      </c>
+      <c r="D89" s="5"/>
+      <c r="E89" s="5"/>
+      <c r="F89" s="6">
+        <v>3</v>
+      </c>
+      <c r="G89" s="6">
+        <v>6</v>
+      </c>
+      <c r="H89" s="6" t="s">
         <v>160</v>
       </c>
-      <c r="B89" s="2" t="s">
-        <v>161</v>
-      </c>
-      <c r="C89" s="2">
-        <v>0</v>
-      </c>
-      <c r="D89" s="2"/>
-      <c r="E89" s="2"/>
-      <c r="F89" s="2">
-        <v>1</v>
-      </c>
-      <c r="G89" s="2">
-        <v>1</v>
-      </c>
-      <c r="H89" s="2" t="s">
-        <v>162</v>
-      </c>
-      <c r="I89" s="2"/>
-      <c r="J89" s="2">
-        <v>10</v>
-      </c>
-      <c r="K89" s="2">
-        <v>0</v>
-      </c>
-      <c r="L89" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="M89" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="N89" s="4"/>
-      <c r="O89" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="P89" s="4"/>
-      <c r="Q89" s="2"/>
-      <c r="R89" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="S89" s="2"/>
-      <c r="T89" s="4"/>
-      <c r="U89" s="2"/>
-      <c r="V89" s="2" t="s">
-        <v>163</v>
-      </c>
-      <c r="W89" s="2" t="s">
-        <v>164</v>
-      </c>
+      <c r="I89" s="6"/>
+      <c r="J89" s="6">
+        <v>1</v>
+      </c>
+      <c r="K89" s="6">
+        <v>0</v>
+      </c>
+      <c r="L89" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="M89" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="N89" s="8"/>
+      <c r="O89" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="P89" s="8"/>
+      <c r="Q89" s="6"/>
+      <c r="R89" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="S89" s="6"/>
+      <c r="T89" s="8"/>
+      <c r="U89" s="6"/>
+      <c r="V89" s="6"/>
+      <c r="W89" s="6"/>
     </row>
     <row r="90" spans="1:23" outlineLevel="1">
       <c r="A90" s="5" t="s">
-        <v>160</v>
+        <v>136</v>
       </c>
       <c r="B90" s="5" t="s">
-        <v>161</v>
+        <v>137</v>
       </c>
       <c r="C90" s="5">
         <v>0</v>
@@ -5537,17 +5548,17 @@
       <c r="D90" s="5"/>
       <c r="E90" s="5"/>
       <c r="F90" s="6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G90" s="6">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="H90" s="6" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="I90" s="6"/>
       <c r="J90" s="6">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="K90" s="6">
         <v>0</v>
@@ -5570,19 +5581,15 @@
       <c r="S90" s="6"/>
       <c r="T90" s="8"/>
       <c r="U90" s="6"/>
-      <c r="V90" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="W90" s="6" t="s">
-        <v>164</v>
-      </c>
+      <c r="V90" s="6"/>
+      <c r="W90" s="6"/>
     </row>
     <row r="91" spans="1:23" outlineLevel="1">
       <c r="A91" s="5" t="s">
-        <v>160</v>
+        <v>136</v>
       </c>
       <c r="B91" s="5" t="s">
-        <v>161</v>
+        <v>137</v>
       </c>
       <c r="C91" s="5">
         <v>0</v>
@@ -5590,17 +5597,17 @@
       <c r="D91" s="5"/>
       <c r="E91" s="5"/>
       <c r="F91" s="6">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G91" s="6">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="H91" s="6" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="I91" s="6"/>
       <c r="J91" s="6">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="K91" s="6">
         <v>0</v>
@@ -5623,19 +5630,15 @@
       <c r="S91" s="6"/>
       <c r="T91" s="8"/>
       <c r="U91" s="6"/>
-      <c r="V91" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="W91" s="6" t="s">
-        <v>164</v>
-      </c>
+      <c r="V91" s="6"/>
+      <c r="W91" s="6"/>
     </row>
     <row r="92" spans="1:23" outlineLevel="1">
       <c r="A92" s="5" t="s">
-        <v>160</v>
+        <v>136</v>
       </c>
       <c r="B92" s="5" t="s">
-        <v>161</v>
+        <v>137</v>
       </c>
       <c r="C92" s="5">
         <v>0</v>
@@ -5646,14 +5649,14 @@
         <v>4</v>
       </c>
       <c r="G92" s="6">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="H92" s="6" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="I92" s="6"/>
       <c r="J92" s="6">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="K92" s="6">
         <v>0</v>
@@ -5676,19 +5679,15 @@
       <c r="S92" s="6"/>
       <c r="T92" s="8"/>
       <c r="U92" s="6"/>
-      <c r="V92" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="W92" s="6" t="s">
-        <v>164</v>
-      </c>
+      <c r="V92" s="6"/>
+      <c r="W92" s="6"/>
     </row>
     <row r="93" spans="1:23" outlineLevel="1">
       <c r="A93" s="5" t="s">
-        <v>160</v>
+        <v>136</v>
       </c>
       <c r="B93" s="5" t="s">
-        <v>161</v>
+        <v>137</v>
       </c>
       <c r="C93" s="5">
         <v>0</v>
@@ -5696,17 +5695,17 @@
       <c r="D93" s="5"/>
       <c r="E93" s="5"/>
       <c r="F93" s="6">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G93" s="6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H93" s="6" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="I93" s="6"/>
       <c r="J93" s="6">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="K93" s="6">
         <v>0</v>
@@ -5729,125 +5728,121 @@
       <c r="S93" s="6"/>
       <c r="T93" s="8"/>
       <c r="U93" s="6"/>
-      <c r="V93" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="W93" s="6" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="94" spans="1:23" outlineLevel="1">
-      <c r="A94" s="5" t="s">
-        <v>160</v>
-      </c>
-      <c r="B94" s="5" t="s">
-        <v>161</v>
-      </c>
-      <c r="C94" s="5">
-        <v>0</v>
-      </c>
-      <c r="D94" s="5"/>
-      <c r="E94" s="5"/>
-      <c r="F94" s="6">
-        <v>7</v>
-      </c>
-      <c r="G94" s="6">
-        <v>6</v>
-      </c>
-      <c r="H94" s="6" t="s">
+      <c r="V93" s="6"/>
+      <c r="W93" s="6"/>
+    </row>
+    <row r="94" spans="1:23">
+      <c r="A94" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="B94" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="C94" s="2">
+        <v>0</v>
+      </c>
+      <c r="D94" s="2"/>
+      <c r="E94" s="2"/>
+      <c r="F94" s="2">
+        <v>1</v>
+      </c>
+      <c r="G94" s="2">
+        <v>1</v>
+      </c>
+      <c r="H94" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="I94" s="2"/>
+      <c r="J94" s="2">
+        <v>10</v>
+      </c>
+      <c r="K94" s="2">
+        <v>0</v>
+      </c>
+      <c r="L94" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="M94" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="N94" s="4"/>
+      <c r="O94" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="P94" s="4"/>
+      <c r="Q94" s="2"/>
+      <c r="R94" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="S94" s="2"/>
+      <c r="T94" s="4"/>
+      <c r="U94" s="2"/>
+      <c r="V94" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="W94" s="2" t="s">
         <v>169</v>
       </c>
-      <c r="I94" s="6"/>
-      <c r="J94" s="6">
+    </row>
+    <row r="95" spans="1:23" outlineLevel="1">
+      <c r="A95" s="5" t="s">
+        <v>165</v>
+      </c>
+      <c r="B95" s="5" t="s">
+        <v>166</v>
+      </c>
+      <c r="C95" s="5">
+        <v>0</v>
+      </c>
+      <c r="D95" s="5"/>
+      <c r="E95" s="5"/>
+      <c r="F95" s="6">
+        <v>2</v>
+      </c>
+      <c r="G95" s="6">
+        <v>3</v>
+      </c>
+      <c r="H95" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="I95" s="6"/>
+      <c r="J95" s="6">
         <v>10</v>
       </c>
-      <c r="K94" s="6">
-        <v>0</v>
-      </c>
-      <c r="L94" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="M94" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="N94" s="8"/>
-      <c r="O94" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="P94" s="8"/>
-      <c r="Q94" s="6"/>
-      <c r="R94" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="S94" s="6"/>
-      <c r="T94" s="8"/>
-      <c r="U94" s="6"/>
-      <c r="V94" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="W94" s="6" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="95" spans="1:23">
-      <c r="A95" s="2" t="s">
-        <v>170</v>
-      </c>
-      <c r="B95" s="2" t="s">
-        <v>171</v>
-      </c>
-      <c r="C95" s="2">
-        <v>0</v>
-      </c>
-      <c r="D95" s="2"/>
-      <c r="E95" s="2"/>
-      <c r="F95" s="2">
-        <v>1</v>
-      </c>
-      <c r="G95" s="2">
-        <v>1</v>
-      </c>
-      <c r="H95" s="2" t="s">
-        <v>162</v>
-      </c>
-      <c r="I95" s="2"/>
-      <c r="J95" s="2">
-        <v>10</v>
-      </c>
-      <c r="K95" s="2">
-        <v>0</v>
-      </c>
-      <c r="L95" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="M95" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="N95" s="4"/>
-      <c r="O95" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="P95" s="4"/>
-      <c r="Q95" s="2"/>
-      <c r="R95" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="S95" s="2"/>
-      <c r="T95" s="4"/>
-      <c r="U95" s="2"/>
-      <c r="V95" s="2" t="s">
-        <v>163</v>
-      </c>
-      <c r="W95" s="2" t="s">
-        <v>164</v>
+      <c r="K95" s="6">
+        <v>0</v>
+      </c>
+      <c r="L95" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="M95" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="N95" s="8"/>
+      <c r="O95" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="P95" s="8"/>
+      <c r="Q95" s="6"/>
+      <c r="R95" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="S95" s="6"/>
+      <c r="T95" s="8"/>
+      <c r="U95" s="6"/>
+      <c r="V95" s="6" t="s">
+        <v>168</v>
+      </c>
+      <c r="W95" s="6" t="s">
+        <v>169</v>
       </c>
     </row>
     <row r="96" spans="1:23" outlineLevel="1">
       <c r="A96" s="5" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="B96" s="5" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="C96" s="5">
         <v>0</v>
@@ -5855,13 +5850,13 @@
       <c r="D96" s="5"/>
       <c r="E96" s="5"/>
       <c r="F96" s="6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G96" s="6">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H96" s="6" t="s">
-        <v>165</v>
+        <v>171</v>
       </c>
       <c r="I96" s="6"/>
       <c r="J96" s="6">
@@ -5889,18 +5884,18 @@
       <c r="T96" s="8"/>
       <c r="U96" s="6"/>
       <c r="V96" s="6" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="W96" s="6" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
     </row>
     <row r="97" spans="1:23" outlineLevel="1">
       <c r="A97" s="5" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="B97" s="5" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="C97" s="5">
         <v>0</v>
@@ -5908,13 +5903,13 @@
       <c r="D97" s="5"/>
       <c r="E97" s="5"/>
       <c r="F97" s="6">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G97" s="6">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H97" s="6" t="s">
-        <v>166</v>
+        <v>172</v>
       </c>
       <c r="I97" s="6"/>
       <c r="J97" s="6">
@@ -5942,18 +5937,18 @@
       <c r="T97" s="8"/>
       <c r="U97" s="6"/>
       <c r="V97" s="6" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="W97" s="6" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
     </row>
     <row r="98" spans="1:23" outlineLevel="1">
       <c r="A98" s="5" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="B98" s="5" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="C98" s="5">
         <v>0</v>
@@ -5961,13 +5956,13 @@
       <c r="D98" s="5"/>
       <c r="E98" s="5"/>
       <c r="F98" s="6">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G98" s="6">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="H98" s="6" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
       <c r="I98" s="6"/>
       <c r="J98" s="6">
@@ -5995,18 +5990,18 @@
       <c r="T98" s="8"/>
       <c r="U98" s="6"/>
       <c r="V98" s="6" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="W98" s="6" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
     </row>
     <row r="99" spans="1:23" outlineLevel="1">
       <c r="A99" s="5" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="B99" s="5" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="C99" s="5">
         <v>0</v>
@@ -6014,13 +6009,13 @@
       <c r="D99" s="5"/>
       <c r="E99" s="5"/>
       <c r="F99" s="6">
+        <v>7</v>
+      </c>
+      <c r="G99" s="6">
         <v>6</v>
       </c>
-      <c r="G99" s="6">
-        <v>1</v>
-      </c>
       <c r="H99" s="6" t="s">
-        <v>168</v>
+        <v>174</v>
       </c>
       <c r="I99" s="6"/>
       <c r="J99" s="6">
@@ -6048,122 +6043,124 @@
       <c r="T99" s="8"/>
       <c r="U99" s="6"/>
       <c r="V99" s="6" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="W99" s="6" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="100" spans="1:23" outlineLevel="1">
-      <c r="A100" s="5" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="100" spans="1:23">
+      <c r="A100" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="B100" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="C100" s="2">
+        <v>0</v>
+      </c>
+      <c r="D100" s="2"/>
+      <c r="E100" s="2"/>
+      <c r="F100" s="2">
+        <v>1</v>
+      </c>
+      <c r="G100" s="2">
+        <v>1</v>
+      </c>
+      <c r="H100" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="I100" s="2"/>
+      <c r="J100" s="2">
+        <v>10</v>
+      </c>
+      <c r="K100" s="2">
+        <v>0</v>
+      </c>
+      <c r="L100" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="M100" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="N100" s="4"/>
+      <c r="O100" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="P100" s="4"/>
+      <c r="Q100" s="2"/>
+      <c r="R100" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="S100" s="2"/>
+      <c r="T100" s="4"/>
+      <c r="U100" s="2"/>
+      <c r="V100" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="W100" s="2" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="101" spans="1:23" outlineLevel="1">
+      <c r="A101" s="5" t="s">
+        <v>175</v>
+      </c>
+      <c r="B101" s="5" t="s">
+        <v>176</v>
+      </c>
+      <c r="C101" s="5">
+        <v>0</v>
+      </c>
+      <c r="D101" s="5"/>
+      <c r="E101" s="5"/>
+      <c r="F101" s="6">
+        <v>2</v>
+      </c>
+      <c r="G101" s="6">
+        <v>3</v>
+      </c>
+      <c r="H101" s="6" t="s">
         <v>170</v>
       </c>
-      <c r="B100" s="5" t="s">
-        <v>171</v>
-      </c>
-      <c r="C100" s="5">
-        <v>0</v>
-      </c>
-      <c r="D100" s="5"/>
-      <c r="E100" s="5"/>
-      <c r="F100" s="6">
-        <v>7</v>
-      </c>
-      <c r="G100" s="6">
-        <v>6</v>
-      </c>
-      <c r="H100" s="6" t="s">
+      <c r="I101" s="6"/>
+      <c r="J101" s="6">
+        <v>10</v>
+      </c>
+      <c r="K101" s="6">
+        <v>0</v>
+      </c>
+      <c r="L101" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="M101" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="N101" s="8"/>
+      <c r="O101" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="P101" s="8"/>
+      <c r="Q101" s="6"/>
+      <c r="R101" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="S101" s="6"/>
+      <c r="T101" s="8"/>
+      <c r="U101" s="6"/>
+      <c r="V101" s="6" t="s">
+        <v>168</v>
+      </c>
+      <c r="W101" s="6" t="s">
         <v>169</v>
       </c>
-      <c r="I100" s="6"/>
-      <c r="J100" s="6">
-        <v>10</v>
-      </c>
-      <c r="K100" s="6">
-        <v>0</v>
-      </c>
-      <c r="L100" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="M100" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="N100" s="8"/>
-      <c r="O100" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="P100" s="8"/>
-      <c r="Q100" s="6"/>
-      <c r="R100" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="S100" s="6"/>
-      <c r="T100" s="8"/>
-      <c r="U100" s="6"/>
-      <c r="V100" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="W100" s="6" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="101" spans="1:23">
-      <c r="A101" s="2" t="s">
-        <v>172</v>
-      </c>
-      <c r="B101" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="C101" s="2">
-        <v>0</v>
-      </c>
-      <c r="D101" s="2"/>
-      <c r="E101" s="2"/>
-      <c r="F101" s="2">
-        <v>1</v>
-      </c>
-      <c r="G101" s="2">
-        <v>0</v>
-      </c>
-      <c r="H101" s="2" t="s">
-        <v>174</v>
-      </c>
-      <c r="I101" s="2"/>
-      <c r="J101" s="2">
-        <v>16</v>
-      </c>
-      <c r="K101" s="2">
-        <v>0</v>
-      </c>
-      <c r="L101" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="M101" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="N101" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="O101" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="P101" s="4"/>
-      <c r="Q101" s="2"/>
-      <c r="R101" s="4"/>
-      <c r="S101" s="2"/>
-      <c r="T101" s="4"/>
-      <c r="U101" s="2"/>
-      <c r="V101" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="W101" s="2"/>
     </row>
     <row r="102" spans="1:23" outlineLevel="1">
       <c r="A102" s="5" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="B102" s="5" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="C102" s="5">
         <v>0</v>
@@ -6174,14 +6171,14 @@
         <v>3</v>
       </c>
       <c r="G102" s="6">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H102" s="6" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="I102" s="6"/>
       <c r="J102" s="6">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="K102" s="6">
         <v>0</v>
@@ -6192,29 +6189,31 @@
       <c r="M102" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="N102" s="7" t="s">
-        <v>25</v>
-      </c>
+      <c r="N102" s="8"/>
       <c r="O102" s="6" t="s">
         <v>26</v>
       </c>
       <c r="P102" s="8"/>
       <c r="Q102" s="6"/>
-      <c r="R102" s="8"/>
+      <c r="R102" s="7" t="s">
+        <v>25</v>
+      </c>
       <c r="S102" s="6"/>
       <c r="T102" s="8"/>
       <c r="U102" s="6"/>
       <c r="V102" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="W102" s="6"/>
+        <v>168</v>
+      </c>
+      <c r="W102" s="6" t="s">
+        <v>169</v>
+      </c>
     </row>
     <row r="103" spans="1:23" outlineLevel="1">
       <c r="A103" s="5" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="B103" s="5" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="C103" s="5">
         <v>0</v>
@@ -6222,17 +6221,17 @@
       <c r="D103" s="5"/>
       <c r="E103" s="5"/>
       <c r="F103" s="6">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G103" s="6">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="H103" s="6" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="I103" s="6"/>
       <c r="J103" s="6">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="K103" s="6">
         <v>0</v>
@@ -6243,29 +6242,31 @@
       <c r="M103" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="N103" s="7" t="s">
-        <v>25</v>
-      </c>
+      <c r="N103" s="8"/>
       <c r="O103" s="6" t="s">
         <v>26</v>
       </c>
       <c r="P103" s="8"/>
       <c r="Q103" s="6"/>
-      <c r="R103" s="8"/>
+      <c r="R103" s="7" t="s">
+        <v>25</v>
+      </c>
       <c r="S103" s="6"/>
       <c r="T103" s="8"/>
       <c r="U103" s="6"/>
       <c r="V103" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="W103" s="6"/>
+        <v>168</v>
+      </c>
+      <c r="W103" s="6" t="s">
+        <v>169</v>
+      </c>
     </row>
     <row r="104" spans="1:23" outlineLevel="1">
       <c r="A104" s="5" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="B104" s="5" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="C104" s="5">
         <v>0</v>
@@ -6273,17 +6274,17 @@
       <c r="D104" s="5"/>
       <c r="E104" s="5"/>
       <c r="F104" s="6">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G104" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H104" s="6" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="I104" s="6"/>
       <c r="J104" s="6">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="K104" s="6">
         <v>0</v>
@@ -6294,131 +6295,135 @@
       <c r="M104" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="N104" s="7" t="s">
-        <v>25</v>
-      </c>
+      <c r="N104" s="8"/>
       <c r="O104" s="6" t="s">
         <v>26</v>
       </c>
       <c r="P104" s="8"/>
       <c r="Q104" s="6"/>
-      <c r="R104" s="8"/>
+      <c r="R104" s="7" t="s">
+        <v>25</v>
+      </c>
       <c r="S104" s="6"/>
       <c r="T104" s="8"/>
       <c r="U104" s="6"/>
       <c r="V104" s="6" t="s">
+        <v>168</v>
+      </c>
+      <c r="W104" s="6" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="105" spans="1:23" outlineLevel="1">
+      <c r="A105" s="5" t="s">
+        <v>175</v>
+      </c>
+      <c r="B105" s="5" t="s">
+        <v>176</v>
+      </c>
+      <c r="C105" s="5">
+        <v>0</v>
+      </c>
+      <c r="D105" s="5"/>
+      <c r="E105" s="5"/>
+      <c r="F105" s="6">
+        <v>7</v>
+      </c>
+      <c r="G105" s="6">
+        <v>6</v>
+      </c>
+      <c r="H105" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="I105" s="6"/>
+      <c r="J105" s="6">
+        <v>10</v>
+      </c>
+      <c r="K105" s="6">
+        <v>0</v>
+      </c>
+      <c r="L105" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="M105" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="N105" s="8"/>
+      <c r="O105" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="P105" s="8"/>
+      <c r="Q105" s="6"/>
+      <c r="R105" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="S105" s="6"/>
+      <c r="T105" s="8"/>
+      <c r="U105" s="6"/>
+      <c r="V105" s="6" t="s">
+        <v>168</v>
+      </c>
+      <c r="W105" s="6" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="106" spans="1:23">
+      <c r="A106" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="B106" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="C106" s="2">
+        <v>0</v>
+      </c>
+      <c r="D106" s="2"/>
+      <c r="E106" s="2"/>
+      <c r="F106" s="2">
+        <v>1</v>
+      </c>
+      <c r="G106" s="2">
+        <v>0</v>
+      </c>
+      <c r="H106" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="I106" s="2"/>
+      <c r="J106" s="2">
+        <v>16</v>
+      </c>
+      <c r="K106" s="2">
+        <v>0</v>
+      </c>
+      <c r="L106" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="M106" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="N106" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="O106" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="P106" s="4"/>
+      <c r="Q106" s="2"/>
+      <c r="R106" s="4"/>
+      <c r="S106" s="2"/>
+      <c r="T106" s="4"/>
+      <c r="U106" s="2"/>
+      <c r="V106" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="W104" s="6"/>
-    </row>
-    <row r="105" spans="1:23">
-      <c r="A105" s="2" t="s">
-        <v>178</v>
-      </c>
-      <c r="B105" s="2" t="s">
-        <v>179</v>
-      </c>
-      <c r="C105" s="2">
-        <v>0</v>
-      </c>
-      <c r="D105" s="2"/>
-      <c r="E105" s="2"/>
-      <c r="F105" s="2">
-        <v>1</v>
-      </c>
-      <c r="G105" s="2">
-        <v>0</v>
-      </c>
-      <c r="H105" s="2" t="s">
-        <v>180</v>
-      </c>
-      <c r="I105" s="2"/>
-      <c r="J105" s="2">
-        <v>16</v>
-      </c>
-      <c r="K105" s="2">
-        <v>0</v>
-      </c>
-      <c r="L105" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="M105" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="N105" s="4"/>
-      <c r="O105" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="P105" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q105" s="2"/>
-      <c r="R105" s="4"/>
-      <c r="S105" s="2"/>
-      <c r="T105" s="4"/>
-      <c r="U105" s="2"/>
-      <c r="V105" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="W105" s="2"/>
-    </row>
-    <row r="106" spans="1:23" outlineLevel="1">
-      <c r="A106" s="5" t="s">
-        <v>178</v>
-      </c>
-      <c r="B106" s="5" t="s">
-        <v>179</v>
-      </c>
-      <c r="C106" s="5">
-        <v>0</v>
-      </c>
-      <c r="D106" s="5"/>
-      <c r="E106" s="5"/>
-      <c r="F106" s="6">
-        <v>3</v>
-      </c>
-      <c r="G106" s="6">
-        <v>0</v>
-      </c>
-      <c r="H106" s="6" t="s">
-        <v>181</v>
-      </c>
-      <c r="I106" s="6"/>
-      <c r="J106" s="6">
-        <v>16</v>
-      </c>
-      <c r="K106" s="6">
-        <v>0</v>
-      </c>
-      <c r="L106" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="M106" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="N106" s="8"/>
-      <c r="O106" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="P106" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q106" s="6"/>
-      <c r="R106" s="8"/>
-      <c r="S106" s="6"/>
-      <c r="T106" s="8"/>
-      <c r="U106" s="6"/>
-      <c r="V106" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="W106" s="6"/>
+      <c r="W106" s="2"/>
     </row>
     <row r="107" spans="1:23" outlineLevel="1">
       <c r="A107" s="5" t="s">
+        <v>177</v>
+      </c>
+      <c r="B107" s="5" t="s">
         <v>178</v>
-      </c>
-      <c r="B107" s="5" t="s">
-        <v>179</v>
       </c>
       <c r="C107" s="5">
         <v>0</v>
@@ -6426,13 +6431,13 @@
       <c r="D107" s="5"/>
       <c r="E107" s="5"/>
       <c r="F107" s="6">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G107" s="6">
         <v>0</v>
       </c>
       <c r="H107" s="6" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="I107" s="6"/>
       <c r="J107" s="6">
@@ -6447,13 +6452,13 @@
       <c r="M107" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="N107" s="8"/>
+      <c r="N107" s="7" t="s">
+        <v>25</v>
+      </c>
       <c r="O107" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="P107" s="7" t="s">
-        <v>25</v>
-      </c>
+      <c r="P107" s="8"/>
       <c r="Q107" s="6"/>
       <c r="R107" s="8"/>
       <c r="S107" s="6"/>
@@ -6466,10 +6471,10 @@
     </row>
     <row r="108" spans="1:23" outlineLevel="1">
       <c r="A108" s="5" t="s">
+        <v>177</v>
+      </c>
+      <c r="B108" s="5" t="s">
         <v>178</v>
-      </c>
-      <c r="B108" s="5" t="s">
-        <v>179</v>
       </c>
       <c r="C108" s="5">
         <v>0</v>
@@ -6477,13 +6482,13 @@
       <c r="D108" s="5"/>
       <c r="E108" s="5"/>
       <c r="F108" s="6">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="G108" s="6">
         <v>0</v>
       </c>
       <c r="H108" s="6" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="I108" s="6"/>
       <c r="J108" s="6">
@@ -6498,13 +6503,13 @@
       <c r="M108" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="N108" s="8"/>
+      <c r="N108" s="7" t="s">
+        <v>25</v>
+      </c>
       <c r="O108" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="P108" s="7" t="s">
-        <v>25</v>
-      </c>
+      <c r="P108" s="8"/>
       <c r="Q108" s="6"/>
       <c r="R108" s="8"/>
       <c r="S108" s="6"/>
@@ -6515,112 +6520,114 @@
       </c>
       <c r="W108" s="6"/>
     </row>
-    <row r="109" spans="1:23">
-      <c r="A109" s="2" t="s">
+    <row r="109" spans="1:23" outlineLevel="1">
+      <c r="A109" s="5" t="s">
+        <v>177</v>
+      </c>
+      <c r="B109" s="5" t="s">
+        <v>178</v>
+      </c>
+      <c r="C109" s="5">
+        <v>0</v>
+      </c>
+      <c r="D109" s="5"/>
+      <c r="E109" s="5"/>
+      <c r="F109" s="6">
+        <v>7</v>
+      </c>
+      <c r="G109" s="6">
+        <v>0</v>
+      </c>
+      <c r="H109" s="6" t="s">
+        <v>182</v>
+      </c>
+      <c r="I109" s="6"/>
+      <c r="J109" s="6">
+        <v>16</v>
+      </c>
+      <c r="K109" s="6">
+        <v>0</v>
+      </c>
+      <c r="L109" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="M109" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="N109" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="O109" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="P109" s="8"/>
+      <c r="Q109" s="6"/>
+      <c r="R109" s="8"/>
+      <c r="S109" s="6"/>
+      <c r="T109" s="8"/>
+      <c r="U109" s="6"/>
+      <c r="V109" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="W109" s="6"/>
+    </row>
+    <row r="110" spans="1:23">
+      <c r="A110" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="B110" s="2" t="s">
         <v>184</v>
       </c>
-      <c r="B109" s="2" t="s">
+      <c r="C110" s="2">
+        <v>0</v>
+      </c>
+      <c r="D110" s="2"/>
+      <c r="E110" s="2"/>
+      <c r="F110" s="2">
+        <v>1</v>
+      </c>
+      <c r="G110" s="2">
+        <v>0</v>
+      </c>
+      <c r="H110" s="2" t="s">
         <v>185</v>
       </c>
-      <c r="C109" s="2">
-        <v>0</v>
-      </c>
-      <c r="D109" s="2"/>
-      <c r="E109" s="2"/>
-      <c r="F109" s="2">
-        <v>1</v>
-      </c>
-      <c r="G109" s="2">
-        <v>0</v>
-      </c>
-      <c r="H109" s="2" t="s">
-        <v>186</v>
-      </c>
-      <c r="I109" s="2"/>
-      <c r="J109" s="2">
-        <v>1</v>
-      </c>
-      <c r="K109" s="2">
-        <v>0</v>
-      </c>
-      <c r="L109" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="M109" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="N109" s="4"/>
-      <c r="O109" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="P109" s="4"/>
-      <c r="Q109" s="2"/>
-      <c r="R109" s="4"/>
-      <c r="S109" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="T109" s="4"/>
-      <c r="U109" s="2"/>
-      <c r="V109" s="2"/>
-      <c r="W109" s="2"/>
-    </row>
-    <row r="110" spans="1:23" outlineLevel="1">
-      <c r="A110" s="5" t="s">
-        <v>184</v>
-      </c>
-      <c r="B110" s="5" t="s">
-        <v>185</v>
-      </c>
-      <c r="C110" s="5">
-        <v>0</v>
-      </c>
-      <c r="D110" s="5"/>
-      <c r="E110" s="5"/>
-      <c r="F110" s="6">
-        <v>2</v>
-      </c>
-      <c r="G110" s="6">
-        <v>0</v>
-      </c>
-      <c r="H110" s="6" t="s">
-        <v>187</v>
-      </c>
-      <c r="I110" s="6"/>
-      <c r="J110" s="6">
-        <v>8</v>
-      </c>
-      <c r="K110" s="6">
-        <v>0</v>
-      </c>
-      <c r="L110" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="M110" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="N110" s="8"/>
-      <c r="O110" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="P110" s="8"/>
-      <c r="Q110" s="6"/>
-      <c r="R110" s="8"/>
-      <c r="S110" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="T110" s="8"/>
-      <c r="U110" s="6"/>
-      <c r="V110" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="W110" s="6"/>
+      <c r="I110" s="2"/>
+      <c r="J110" s="2">
+        <v>16</v>
+      </c>
+      <c r="K110" s="2">
+        <v>0</v>
+      </c>
+      <c r="L110" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="M110" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="N110" s="4"/>
+      <c r="O110" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="P110" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q110" s="2"/>
+      <c r="R110" s="4"/>
+      <c r="S110" s="2"/>
+      <c r="T110" s="4"/>
+      <c r="U110" s="2"/>
+      <c r="V110" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="W110" s="2"/>
     </row>
     <row r="111" spans="1:23" outlineLevel="1">
       <c r="A111" s="5" t="s">
+        <v>183</v>
+      </c>
+      <c r="B111" s="5" t="s">
         <v>184</v>
-      </c>
-      <c r="B111" s="5" t="s">
-        <v>185</v>
       </c>
       <c r="C111" s="5">
         <v>0</v>
@@ -6634,11 +6641,11 @@
         <v>0</v>
       </c>
       <c r="H111" s="6" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="I111" s="6"/>
       <c r="J111" s="6">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="K111" s="6">
         <v>0</v>
@@ -6650,81 +6657,79 @@
         <v>29</v>
       </c>
       <c r="N111" s="8"/>
-      <c r="O111" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="P111" s="8"/>
+      <c r="O111" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="P111" s="7" t="s">
+        <v>25</v>
+      </c>
       <c r="Q111" s="6"/>
       <c r="R111" s="8"/>
-      <c r="S111" s="6" t="s">
-        <v>26</v>
-      </c>
+      <c r="S111" s="6"/>
       <c r="T111" s="8"/>
       <c r="U111" s="6"/>
       <c r="V111" s="6" t="s">
-        <v>54</v>
+        <v>30</v>
       </c>
       <c r="W111" s="6"/>
     </row>
-    <row r="112" spans="1:23">
-      <c r="A112" s="2" t="s">
-        <v>189</v>
-      </c>
-      <c r="B112" s="2" t="s">
-        <v>190</v>
-      </c>
-      <c r="C112" s="2">
-        <v>0</v>
-      </c>
-      <c r="D112" s="2"/>
-      <c r="E112" s="2"/>
-      <c r="F112" s="2">
-        <v>1</v>
-      </c>
-      <c r="G112" s="2">
-        <v>0</v>
-      </c>
-      <c r="H112" s="2" t="s">
-        <v>191</v>
-      </c>
-      <c r="I112" s="2"/>
-      <c r="J112" s="2">
-        <v>10</v>
-      </c>
-      <c r="K112" s="2">
-        <v>0</v>
-      </c>
-      <c r="L112" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="M112" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="N112" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="O112" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="P112" s="4"/>
-      <c r="Q112" s="2"/>
-      <c r="R112" s="4"/>
-      <c r="S112" s="2"/>
-      <c r="T112" s="4"/>
-      <c r="U112" s="2"/>
-      <c r="V112" s="2" t="s">
-        <v>163</v>
-      </c>
-      <c r="W112" s="2" t="s">
-        <v>164</v>
-      </c>
+    <row r="112" spans="1:23" outlineLevel="1">
+      <c r="A112" s="5" t="s">
+        <v>183</v>
+      </c>
+      <c r="B112" s="5" t="s">
+        <v>184</v>
+      </c>
+      <c r="C112" s="5">
+        <v>0</v>
+      </c>
+      <c r="D112" s="5"/>
+      <c r="E112" s="5"/>
+      <c r="F112" s="6">
+        <v>5</v>
+      </c>
+      <c r="G112" s="6">
+        <v>0</v>
+      </c>
+      <c r="H112" s="6" t="s">
+        <v>187</v>
+      </c>
+      <c r="I112" s="6"/>
+      <c r="J112" s="6">
+        <v>16</v>
+      </c>
+      <c r="K112" s="6">
+        <v>0</v>
+      </c>
+      <c r="L112" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="M112" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="N112" s="8"/>
+      <c r="O112" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="P112" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q112" s="6"/>
+      <c r="R112" s="8"/>
+      <c r="S112" s="6"/>
+      <c r="T112" s="8"/>
+      <c r="U112" s="6"/>
+      <c r="V112" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="W112" s="6"/>
     </row>
     <row r="113" spans="1:23" outlineLevel="1">
       <c r="A113" s="5" t="s">
-        <v>189</v>
+        <v>183</v>
       </c>
       <c r="B113" s="5" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="C113" s="5">
         <v>0</v>
@@ -6732,17 +6737,17 @@
       <c r="D113" s="5"/>
       <c r="E113" s="5"/>
       <c r="F113" s="6">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="G113" s="6">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H113" s="6" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="I113" s="6"/>
       <c r="J113" s="6">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="K113" s="6">
         <v>0</v>
@@ -6753,77 +6758,71 @@
       <c r="M113" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="N113" s="7" t="s">
-        <v>25</v>
-      </c>
+      <c r="N113" s="8"/>
       <c r="O113" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="P113" s="8"/>
+      <c r="P113" s="7" t="s">
+        <v>25</v>
+      </c>
       <c r="Q113" s="6"/>
       <c r="R113" s="8"/>
       <c r="S113" s="6"/>
       <c r="T113" s="8"/>
       <c r="U113" s="6"/>
       <c r="V113" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="W113" s="6" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="114" spans="1:23" outlineLevel="1">
-      <c r="A114" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="W113" s="6"/>
+    </row>
+    <row r="114" spans="1:23">
+      <c r="A114" s="2" t="s">
         <v>189</v>
       </c>
-      <c r="B114" s="5" t="s">
+      <c r="B114" s="2" t="s">
         <v>190</v>
       </c>
-      <c r="C114" s="5">
-        <v>0</v>
-      </c>
-      <c r="D114" s="5"/>
-      <c r="E114" s="5"/>
-      <c r="F114" s="6">
-        <v>3</v>
-      </c>
-      <c r="G114" s="6">
-        <v>4</v>
-      </c>
-      <c r="H114" s="6" t="s">
-        <v>193</v>
-      </c>
-      <c r="I114" s="6"/>
-      <c r="J114" s="6">
-        <v>10</v>
-      </c>
-      <c r="K114" s="6">
-        <v>0</v>
-      </c>
-      <c r="L114" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="M114" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="N114" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="O114" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="P114" s="8"/>
-      <c r="Q114" s="6"/>
-      <c r="R114" s="8"/>
-      <c r="S114" s="6"/>
-      <c r="T114" s="8"/>
-      <c r="U114" s="6"/>
-      <c r="V114" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="W114" s="6" t="s">
-        <v>164</v>
-      </c>
+      <c r="C114" s="2">
+        <v>0</v>
+      </c>
+      <c r="D114" s="2"/>
+      <c r="E114" s="2"/>
+      <c r="F114" s="2">
+        <v>1</v>
+      </c>
+      <c r="G114" s="2">
+        <v>0</v>
+      </c>
+      <c r="H114" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="I114" s="2"/>
+      <c r="J114" s="2">
+        <v>1</v>
+      </c>
+      <c r="K114" s="2">
+        <v>0</v>
+      </c>
+      <c r="L114" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="M114" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="N114" s="4"/>
+      <c r="O114" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="P114" s="4"/>
+      <c r="Q114" s="2"/>
+      <c r="R114" s="4"/>
+      <c r="S114" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="T114" s="4"/>
+      <c r="U114" s="2"/>
+      <c r="V114" s="2"/>
+      <c r="W114" s="2"/>
     </row>
     <row r="115" spans="1:23" outlineLevel="1">
       <c r="A115" s="5" t="s">
@@ -6838,17 +6837,17 @@
       <c r="D115" s="5"/>
       <c r="E115" s="5"/>
       <c r="F115" s="6">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G115" s="6">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H115" s="6" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="I115" s="6"/>
       <c r="J115" s="6">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="K115" s="6">
         <v>0</v>
@@ -6859,24 +6858,22 @@
       <c r="M115" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="N115" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="O115" s="6" t="s">
-        <v>26</v>
+      <c r="N115" s="8"/>
+      <c r="O115" s="10" t="s">
+        <v>25</v>
       </c>
       <c r="P115" s="8"/>
       <c r="Q115" s="6"/>
       <c r="R115" s="8"/>
-      <c r="S115" s="6"/>
+      <c r="S115" s="6" t="s">
+        <v>26</v>
+      </c>
       <c r="T115" s="8"/>
       <c r="U115" s="6"/>
       <c r="V115" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="W115" s="6" t="s">
-        <v>164</v>
-      </c>
+        <v>54</v>
+      </c>
+      <c r="W115" s="6"/>
     </row>
     <row r="116" spans="1:23" outlineLevel="1">
       <c r="A116" s="5" t="s">
@@ -6891,17 +6888,17 @@
       <c r="D116" s="5"/>
       <c r="E116" s="5"/>
       <c r="F116" s="6">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G116" s="6">
         <v>0</v>
       </c>
       <c r="H116" s="6" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="I116" s="6"/>
       <c r="J116" s="6">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="K116" s="6">
         <v>0</v>
@@ -6912,137 +6909,135 @@
       <c r="M116" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="N116" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="O116" s="6" t="s">
-        <v>26</v>
+      <c r="N116" s="8"/>
+      <c r="O116" s="10" t="s">
+        <v>25</v>
       </c>
       <c r="P116" s="8"/>
       <c r="Q116" s="6"/>
       <c r="R116" s="8"/>
-      <c r="S116" s="6"/>
+      <c r="S116" s="6" t="s">
+        <v>26</v>
+      </c>
       <c r="T116" s="8"/>
       <c r="U116" s="6"/>
       <c r="V116" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="W116" s="6" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="117" spans="1:23" outlineLevel="1">
-      <c r="A117" s="5" t="s">
-        <v>189</v>
-      </c>
-      <c r="B117" s="5" t="s">
-        <v>190</v>
-      </c>
-      <c r="C117" s="5">
-        <v>0</v>
-      </c>
-      <c r="D117" s="5"/>
-      <c r="E117" s="5"/>
-      <c r="F117" s="6">
-        <v>7</v>
-      </c>
-      <c r="G117" s="6">
+        <v>54</v>
+      </c>
+      <c r="W116" s="6"/>
+    </row>
+    <row r="117" spans="1:23">
+      <c r="A117" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="B117" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="C117" s="2">
+        <v>0</v>
+      </c>
+      <c r="D117" s="2"/>
+      <c r="E117" s="2"/>
+      <c r="F117" s="2">
+        <v>1</v>
+      </c>
+      <c r="G117" s="2">
+        <v>0</v>
+      </c>
+      <c r="H117" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="I117" s="2"/>
+      <c r="J117" s="2">
+        <v>10</v>
+      </c>
+      <c r="K117" s="2">
+        <v>0</v>
+      </c>
+      <c r="L117" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="M117" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="N117" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="O117" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="P117" s="4"/>
+      <c r="Q117" s="2"/>
+      <c r="R117" s="4"/>
+      <c r="S117" s="2"/>
+      <c r="T117" s="4"/>
+      <c r="U117" s="2"/>
+      <c r="V117" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="W117" s="2" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="118" spans="1:23" outlineLevel="1">
+      <c r="A118" s="5" t="s">
+        <v>194</v>
+      </c>
+      <c r="B118" s="5" t="s">
+        <v>195</v>
+      </c>
+      <c r="C118" s="5">
+        <v>0</v>
+      </c>
+      <c r="D118" s="5"/>
+      <c r="E118" s="5"/>
+      <c r="F118" s="6">
         <v>2</v>
       </c>
-      <c r="H117" s="6" t="s">
-        <v>196</v>
-      </c>
-      <c r="I117" s="6"/>
-      <c r="J117" s="6">
+      <c r="G118" s="6">
+        <v>2</v>
+      </c>
+      <c r="H118" s="6" t="s">
+        <v>197</v>
+      </c>
+      <c r="I118" s="6"/>
+      <c r="J118" s="6">
         <v>10</v>
       </c>
-      <c r="K117" s="6">
-        <v>0</v>
-      </c>
-      <c r="L117" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="M117" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="N117" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="O117" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="P117" s="8"/>
-      <c r="Q117" s="6"/>
-      <c r="R117" s="8"/>
-      <c r="S117" s="6"/>
-      <c r="T117" s="8"/>
-      <c r="U117" s="6"/>
-      <c r="V117" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="W117" s="6" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="118" spans="1:23">
-      <c r="A118" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="B118" s="2" t="s">
-        <v>198</v>
-      </c>
-      <c r="C118" s="2">
-        <v>0</v>
-      </c>
-      <c r="D118" s="2"/>
-      <c r="E118" s="2"/>
-      <c r="F118" s="2">
-        <v>1</v>
-      </c>
-      <c r="G118" s="2">
-        <v>0</v>
-      </c>
-      <c r="H118" s="2" t="s">
-        <v>191</v>
-      </c>
-      <c r="I118" s="2"/>
-      <c r="J118" s="2">
-        <v>10</v>
-      </c>
-      <c r="K118" s="2">
-        <v>0</v>
-      </c>
-      <c r="L118" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="M118" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="N118" s="4"/>
-      <c r="O118" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="P118" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q118" s="2"/>
-      <c r="R118" s="4"/>
-      <c r="S118" s="2"/>
-      <c r="T118" s="4"/>
-      <c r="U118" s="2"/>
-      <c r="V118" s="2" t="s">
-        <v>163</v>
-      </c>
-      <c r="W118" s="2" t="s">
-        <v>164</v>
+      <c r="K118" s="6">
+        <v>0</v>
+      </c>
+      <c r="L118" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="M118" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="N118" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="O118" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="P118" s="8"/>
+      <c r="Q118" s="6"/>
+      <c r="R118" s="8"/>
+      <c r="S118" s="6"/>
+      <c r="T118" s="8"/>
+      <c r="U118" s="6"/>
+      <c r="V118" s="6" t="s">
+        <v>168</v>
+      </c>
+      <c r="W118" s="6" t="s">
+        <v>169</v>
       </c>
     </row>
     <row r="119" spans="1:23" outlineLevel="1">
       <c r="A119" s="5" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="B119" s="5" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="C119" s="5">
         <v>0</v>
@@ -7050,13 +7045,13 @@
       <c r="D119" s="5"/>
       <c r="E119" s="5"/>
       <c r="F119" s="6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G119" s="6">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H119" s="6" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
       <c r="I119" s="6"/>
       <c r="J119" s="6">
@@ -7071,31 +7066,31 @@
       <c r="M119" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="N119" s="8"/>
+      <c r="N119" s="7" t="s">
+        <v>25</v>
+      </c>
       <c r="O119" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="P119" s="7" t="s">
-        <v>25</v>
-      </c>
+      <c r="P119" s="8"/>
       <c r="Q119" s="6"/>
       <c r="R119" s="8"/>
       <c r="S119" s="6"/>
       <c r="T119" s="8"/>
       <c r="U119" s="6"/>
       <c r="V119" s="6" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="W119" s="6" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
     </row>
     <row r="120" spans="1:23" outlineLevel="1">
       <c r="A120" s="5" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="B120" s="5" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="C120" s="5">
         <v>0</v>
@@ -7103,13 +7098,13 @@
       <c r="D120" s="5"/>
       <c r="E120" s="5"/>
       <c r="F120" s="6">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G120" s="6">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H120" s="6" t="s">
-        <v>193</v>
+        <v>199</v>
       </c>
       <c r="I120" s="6"/>
       <c r="J120" s="6">
@@ -7124,31 +7119,31 @@
       <c r="M120" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="N120" s="8"/>
+      <c r="N120" s="7" t="s">
+        <v>25</v>
+      </c>
       <c r="O120" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="P120" s="7" t="s">
-        <v>25</v>
-      </c>
+      <c r="P120" s="8"/>
       <c r="Q120" s="6"/>
       <c r="R120" s="8"/>
       <c r="S120" s="6"/>
       <c r="T120" s="8"/>
       <c r="U120" s="6"/>
       <c r="V120" s="6" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="W120" s="6" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
     </row>
     <row r="121" spans="1:23" outlineLevel="1">
       <c r="A121" s="5" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="B121" s="5" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="C121" s="5">
         <v>0</v>
@@ -7156,13 +7151,13 @@
       <c r="D121" s="5"/>
       <c r="E121" s="5"/>
       <c r="F121" s="6">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G121" s="6">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H121" s="6" t="s">
-        <v>194</v>
+        <v>200</v>
       </c>
       <c r="I121" s="6"/>
       <c r="J121" s="6">
@@ -7177,31 +7172,31 @@
       <c r="M121" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="N121" s="8"/>
+      <c r="N121" s="7" t="s">
+        <v>25</v>
+      </c>
       <c r="O121" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="P121" s="7" t="s">
-        <v>25</v>
-      </c>
+      <c r="P121" s="8"/>
       <c r="Q121" s="6"/>
       <c r="R121" s="8"/>
       <c r="S121" s="6"/>
       <c r="T121" s="8"/>
       <c r="U121" s="6"/>
       <c r="V121" s="6" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="W121" s="6" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
     </row>
     <row r="122" spans="1:23" outlineLevel="1">
       <c r="A122" s="5" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="B122" s="5" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="C122" s="5">
         <v>0</v>
@@ -7209,13 +7204,13 @@
       <c r="D122" s="5"/>
       <c r="E122" s="5"/>
       <c r="F122" s="6">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G122" s="6">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H122" s="6" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="I122" s="6"/>
       <c r="J122" s="6">
@@ -7230,135 +7225,137 @@
       <c r="M122" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="N122" s="8"/>
+      <c r="N122" s="7" t="s">
+        <v>25</v>
+      </c>
       <c r="O122" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="P122" s="7" t="s">
-        <v>25</v>
-      </c>
+      <c r="P122" s="8"/>
       <c r="Q122" s="6"/>
       <c r="R122" s="8"/>
       <c r="S122" s="6"/>
       <c r="T122" s="8"/>
       <c r="U122" s="6"/>
       <c r="V122" s="6" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="W122" s="6" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="123" spans="1:23" outlineLevel="1">
-      <c r="A123" s="5" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="123" spans="1:23">
+      <c r="A123" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="B123" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="C123" s="2">
+        <v>0</v>
+      </c>
+      <c r="D123" s="2"/>
+      <c r="E123" s="2"/>
+      <c r="F123" s="2">
+        <v>1</v>
+      </c>
+      <c r="G123" s="2">
+        <v>0</v>
+      </c>
+      <c r="H123" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="I123" s="2"/>
+      <c r="J123" s="2">
+        <v>10</v>
+      </c>
+      <c r="K123" s="2">
+        <v>0</v>
+      </c>
+      <c r="L123" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="M123" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="N123" s="4"/>
+      <c r="O123" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="P123" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q123" s="2"/>
+      <c r="R123" s="4"/>
+      <c r="S123" s="2"/>
+      <c r="T123" s="4"/>
+      <c r="U123" s="2"/>
+      <c r="V123" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="W123" s="2" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="124" spans="1:23" outlineLevel="1">
+      <c r="A124" s="5" t="s">
+        <v>202</v>
+      </c>
+      <c r="B124" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="C124" s="5">
+        <v>0</v>
+      </c>
+      <c r="D124" s="5"/>
+      <c r="E124" s="5"/>
+      <c r="F124" s="6">
+        <v>2</v>
+      </c>
+      <c r="G124" s="6">
+        <v>2</v>
+      </c>
+      <c r="H124" s="6" t="s">
         <v>197</v>
       </c>
-      <c r="B123" s="5" t="s">
-        <v>198</v>
-      </c>
-      <c r="C123" s="5">
-        <v>0</v>
-      </c>
-      <c r="D123" s="5"/>
-      <c r="E123" s="5"/>
-      <c r="F123" s="6">
-        <v>7</v>
-      </c>
-      <c r="G123" s="6">
-        <v>2</v>
-      </c>
-      <c r="H123" s="6" t="s">
-        <v>200</v>
-      </c>
-      <c r="I123" s="6"/>
-      <c r="J123" s="6">
+      <c r="I124" s="6"/>
+      <c r="J124" s="6">
         <v>10</v>
       </c>
-      <c r="K123" s="6">
-        <v>0</v>
-      </c>
-      <c r="L123" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="M123" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="N123" s="8"/>
-      <c r="O123" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="P123" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q123" s="6"/>
-      <c r="R123" s="8"/>
-      <c r="S123" s="6"/>
-      <c r="T123" s="8"/>
-      <c r="U123" s="6"/>
-      <c r="V123" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="W123" s="6" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="124" spans="1:23">
-      <c r="A124" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="B124" s="2" t="s">
-        <v>202</v>
-      </c>
-      <c r="C124" s="2">
-        <v>0</v>
-      </c>
-      <c r="D124" s="2"/>
-      <c r="E124" s="2"/>
-      <c r="F124" s="2">
-        <v>1</v>
-      </c>
-      <c r="G124" s="2">
-        <v>0</v>
-      </c>
-      <c r="H124" s="2" t="s">
-        <v>203</v>
-      </c>
-      <c r="I124" s="2"/>
-      <c r="J124" s="2">
-        <v>16</v>
-      </c>
-      <c r="K124" s="2">
-        <v>0</v>
-      </c>
-      <c r="L124" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="M124" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="N124" s="4"/>
-      <c r="O124" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="P124" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q124" s="2"/>
-      <c r="R124" s="4"/>
-      <c r="S124" s="2"/>
-      <c r="T124" s="4"/>
-      <c r="U124" s="2"/>
-      <c r="V124" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="W124" s="2"/>
+      <c r="K124" s="6">
+        <v>0</v>
+      </c>
+      <c r="L124" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="M124" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="N124" s="8"/>
+      <c r="O124" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="P124" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q124" s="6"/>
+      <c r="R124" s="8"/>
+      <c r="S124" s="6"/>
+      <c r="T124" s="8"/>
+      <c r="U124" s="6"/>
+      <c r="V124" s="6" t="s">
+        <v>168</v>
+      </c>
+      <c r="W124" s="6" t="s">
+        <v>169</v>
+      </c>
     </row>
     <row r="125" spans="1:23" outlineLevel="1">
       <c r="A125" s="5" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B125" s="5" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C125" s="5">
         <v>0</v>
@@ -7369,14 +7366,14 @@
         <v>3</v>
       </c>
       <c r="G125" s="6">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H125" s="6" t="s">
-        <v>204</v>
+        <v>198</v>
       </c>
       <c r="I125" s="6"/>
       <c r="J125" s="6">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="K125" s="6">
         <v>0</v>
@@ -7400,65 +7397,71 @@
       <c r="T125" s="8"/>
       <c r="U125" s="6"/>
       <c r="V125" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="W125" s="6"/>
-    </row>
-    <row r="126" spans="1:23">
-      <c r="A126" s="2" t="s">
-        <v>205</v>
-      </c>
-      <c r="B126" s="2" t="s">
-        <v>206</v>
-      </c>
-      <c r="C126" s="2">
-        <v>0</v>
-      </c>
-      <c r="D126" s="2"/>
-      <c r="E126" s="2"/>
-      <c r="F126" s="2">
-        <v>1</v>
-      </c>
-      <c r="G126" s="2">
-        <v>0</v>
-      </c>
-      <c r="H126" s="2" t="s">
-        <v>207</v>
-      </c>
-      <c r="I126" s="2"/>
-      <c r="J126" s="2">
-        <v>1</v>
-      </c>
-      <c r="K126" s="2">
-        <v>0</v>
-      </c>
-      <c r="L126" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="M126" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="N126" s="4"/>
-      <c r="O126" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="P126" s="4"/>
-      <c r="Q126" s="2"/>
-      <c r="R126" s="4"/>
-      <c r="S126" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="T126" s="4"/>
-      <c r="U126" s="2"/>
-      <c r="V126" s="2"/>
-      <c r="W126" s="2"/>
+        <v>168</v>
+      </c>
+      <c r="W125" s="6" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="126" spans="1:23" outlineLevel="1">
+      <c r="A126" s="5" t="s">
+        <v>202</v>
+      </c>
+      <c r="B126" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="C126" s="5">
+        <v>0</v>
+      </c>
+      <c r="D126" s="5"/>
+      <c r="E126" s="5"/>
+      <c r="F126" s="6">
+        <v>4</v>
+      </c>
+      <c r="G126" s="6">
+        <v>6</v>
+      </c>
+      <c r="H126" s="6" t="s">
+        <v>199</v>
+      </c>
+      <c r="I126" s="6"/>
+      <c r="J126" s="6">
+        <v>10</v>
+      </c>
+      <c r="K126" s="6">
+        <v>0</v>
+      </c>
+      <c r="L126" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="M126" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="N126" s="8"/>
+      <c r="O126" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="P126" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q126" s="6"/>
+      <c r="R126" s="8"/>
+      <c r="S126" s="6"/>
+      <c r="T126" s="8"/>
+      <c r="U126" s="6"/>
+      <c r="V126" s="6" t="s">
+        <v>168</v>
+      </c>
+      <c r="W126" s="6" t="s">
+        <v>169</v>
+      </c>
     </row>
     <row r="127" spans="1:23" outlineLevel="1">
       <c r="A127" s="5" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="B127" s="5" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="C127" s="5">
         <v>0</v>
@@ -7466,17 +7469,17 @@
       <c r="D127" s="5"/>
       <c r="E127" s="5"/>
       <c r="F127" s="6">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="G127" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H127" s="6" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
       <c r="I127" s="6"/>
       <c r="J127" s="6">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="K127" s="6">
         <v>0</v>
@@ -7491,23 +7494,27 @@
       <c r="O127" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="P127" s="8"/>
+      <c r="P127" s="7" t="s">
+        <v>25</v>
+      </c>
       <c r="Q127" s="6"/>
       <c r="R127" s="8"/>
-      <c r="S127" s="10" t="s">
-        <v>25</v>
-      </c>
+      <c r="S127" s="6"/>
       <c r="T127" s="8"/>
       <c r="U127" s="6"/>
-      <c r="V127" s="6"/>
-      <c r="W127" s="6"/>
+      <c r="V127" s="6" t="s">
+        <v>168</v>
+      </c>
+      <c r="W127" s="6" t="s">
+        <v>169</v>
+      </c>
     </row>
     <row r="128" spans="1:23" outlineLevel="1">
       <c r="A128" s="5" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="B128" s="5" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="C128" s="5">
         <v>0</v>
@@ -7515,17 +7522,17 @@
       <c r="D128" s="5"/>
       <c r="E128" s="5"/>
       <c r="F128" s="6">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="G128" s="6">
         <v>2</v>
       </c>
       <c r="H128" s="6" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="I128" s="6"/>
       <c r="J128" s="6">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="K128" s="6">
         <v>0</v>
@@ -7540,68 +7547,321 @@
       <c r="O128" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="P128" s="8"/>
+      <c r="P128" s="7" t="s">
+        <v>25</v>
+      </c>
       <c r="Q128" s="6"/>
       <c r="R128" s="8"/>
-      <c r="S128" s="10" t="s">
-        <v>25</v>
-      </c>
+      <c r="S128" s="6"/>
       <c r="T128" s="8"/>
       <c r="U128" s="6"/>
-      <c r="V128" s="6"/>
-      <c r="W128" s="6"/>
-    </row>
-    <row r="129" spans="1:23" outlineLevel="1">
-      <c r="A129" s="5" t="s">
-        <v>205</v>
-      </c>
-      <c r="B129" s="5" t="s">
+      <c r="V128" s="6" t="s">
+        <v>168</v>
+      </c>
+      <c r="W128" s="6" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="129" spans="1:23">
+      <c r="A129" s="2" t="s">
         <v>206</v>
       </c>
-      <c r="C129" s="5">
-        <v>0</v>
-      </c>
-      <c r="D129" s="5"/>
-      <c r="E129" s="5"/>
-      <c r="F129" s="6">
-        <v>1</v>
-      </c>
-      <c r="G129" s="6">
+      <c r="B129" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="C129" s="2">
+        <v>0</v>
+      </c>
+      <c r="D129" s="2"/>
+      <c r="E129" s="2"/>
+      <c r="F129" s="2">
+        <v>1</v>
+      </c>
+      <c r="G129" s="2">
+        <v>0</v>
+      </c>
+      <c r="H129" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="I129" s="2"/>
+      <c r="J129" s="2">
+        <v>16</v>
+      </c>
+      <c r="K129" s="2">
+        <v>0</v>
+      </c>
+      <c r="L129" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="M129" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="N129" s="4"/>
+      <c r="O129" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="P129" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q129" s="2"/>
+      <c r="R129" s="4"/>
+      <c r="S129" s="2"/>
+      <c r="T129" s="4"/>
+      <c r="U129" s="2"/>
+      <c r="V129" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="W129" s="2"/>
+    </row>
+    <row r="130" spans="1:23" outlineLevel="1">
+      <c r="A130" s="5" t="s">
+        <v>206</v>
+      </c>
+      <c r="B130" s="5" t="s">
+        <v>207</v>
+      </c>
+      <c r="C130" s="5">
+        <v>0</v>
+      </c>
+      <c r="D130" s="5"/>
+      <c r="E130" s="5"/>
+      <c r="F130" s="6">
         <v>3</v>
       </c>
-      <c r="H129" s="6" t="s">
+      <c r="G130" s="6">
+        <v>0</v>
+      </c>
+      <c r="H130" s="6" t="s">
+        <v>209</v>
+      </c>
+      <c r="I130" s="6"/>
+      <c r="J130" s="6">
+        <v>16</v>
+      </c>
+      <c r="K130" s="6">
+        <v>0</v>
+      </c>
+      <c r="L130" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="M130" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="N130" s="8"/>
+      <c r="O130" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="P130" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q130" s="6"/>
+      <c r="R130" s="8"/>
+      <c r="S130" s="6"/>
+      <c r="T130" s="8"/>
+      <c r="U130" s="6"/>
+      <c r="V130" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="W130" s="6"/>
+    </row>
+    <row r="131" spans="1:23">
+      <c r="A131" s="2" t="s">
         <v>210</v>
       </c>
-      <c r="I129" s="6"/>
-      <c r="J129" s="6">
-        <v>1</v>
-      </c>
-      <c r="K129" s="6">
-        <v>0</v>
-      </c>
-      <c r="L129" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="M129" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="N129" s="8"/>
-      <c r="O129" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="P129" s="8"/>
-      <c r="Q129" s="6"/>
-      <c r="R129" s="8"/>
-      <c r="S129" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="T129" s="8"/>
-      <c r="U129" s="6"/>
-      <c r="V129" s="6"/>
-      <c r="W129" s="6"/>
+      <c r="B131" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="C131" s="2">
+        <v>0</v>
+      </c>
+      <c r="D131" s="2"/>
+      <c r="E131" s="2"/>
+      <c r="F131" s="2">
+        <v>1</v>
+      </c>
+      <c r="G131" s="2">
+        <v>0</v>
+      </c>
+      <c r="H131" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="I131" s="2"/>
+      <c r="J131" s="2">
+        <v>1</v>
+      </c>
+      <c r="K131" s="2">
+        <v>0</v>
+      </c>
+      <c r="L131" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="M131" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="N131" s="4"/>
+      <c r="O131" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="P131" s="4"/>
+      <c r="Q131" s="2"/>
+      <c r="R131" s="4"/>
+      <c r="S131" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="T131" s="4"/>
+      <c r="U131" s="2"/>
+      <c r="V131" s="2"/>
+      <c r="W131" s="2"/>
+    </row>
+    <row r="132" spans="1:23" outlineLevel="1">
+      <c r="A132" s="5" t="s">
+        <v>210</v>
+      </c>
+      <c r="B132" s="5" t="s">
+        <v>211</v>
+      </c>
+      <c r="C132" s="5">
+        <v>0</v>
+      </c>
+      <c r="D132" s="5"/>
+      <c r="E132" s="5"/>
+      <c r="F132" s="6">
+        <v>1</v>
+      </c>
+      <c r="G132" s="6">
+        <v>1</v>
+      </c>
+      <c r="H132" s="6" t="s">
+        <v>213</v>
+      </c>
+      <c r="I132" s="6"/>
+      <c r="J132" s="6">
+        <v>1</v>
+      </c>
+      <c r="K132" s="6">
+        <v>0</v>
+      </c>
+      <c r="L132" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="M132" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="N132" s="8"/>
+      <c r="O132" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="P132" s="8"/>
+      <c r="Q132" s="6"/>
+      <c r="R132" s="8"/>
+      <c r="S132" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="T132" s="8"/>
+      <c r="U132" s="6"/>
+      <c r="V132" s="6"/>
+      <c r="W132" s="6"/>
+    </row>
+    <row r="133" spans="1:23" outlineLevel="1">
+      <c r="A133" s="5" t="s">
+        <v>210</v>
+      </c>
+      <c r="B133" s="5" t="s">
+        <v>211</v>
+      </c>
+      <c r="C133" s="5">
+        <v>0</v>
+      </c>
+      <c r="D133" s="5"/>
+      <c r="E133" s="5"/>
+      <c r="F133" s="6">
+        <v>1</v>
+      </c>
+      <c r="G133" s="6">
+        <v>2</v>
+      </c>
+      <c r="H133" s="6" t="s">
+        <v>214</v>
+      </c>
+      <c r="I133" s="6"/>
+      <c r="J133" s="6">
+        <v>1</v>
+      </c>
+      <c r="K133" s="6">
+        <v>0</v>
+      </c>
+      <c r="L133" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="M133" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="N133" s="8"/>
+      <c r="O133" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="P133" s="8"/>
+      <c r="Q133" s="6"/>
+      <c r="R133" s="8"/>
+      <c r="S133" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="T133" s="8"/>
+      <c r="U133" s="6"/>
+      <c r="V133" s="6"/>
+      <c r="W133" s="6"/>
+    </row>
+    <row r="134" spans="1:23" outlineLevel="1">
+      <c r="A134" s="5" t="s">
+        <v>210</v>
+      </c>
+      <c r="B134" s="5" t="s">
+        <v>211</v>
+      </c>
+      <c r="C134" s="5">
+        <v>0</v>
+      </c>
+      <c r="D134" s="5"/>
+      <c r="E134" s="5"/>
+      <c r="F134" s="6">
+        <v>1</v>
+      </c>
+      <c r="G134" s="6">
+        <v>3</v>
+      </c>
+      <c r="H134" s="6" t="s">
+        <v>215</v>
+      </c>
+      <c r="I134" s="6"/>
+      <c r="J134" s="6">
+        <v>1</v>
+      </c>
+      <c r="K134" s="6">
+        <v>0</v>
+      </c>
+      <c r="L134" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="M134" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="N134" s="8"/>
+      <c r="O134" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="P134" s="8"/>
+      <c r="Q134" s="6"/>
+      <c r="R134" s="8"/>
+      <c r="S134" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="T134" s="8"/>
+      <c r="U134" s="6"/>
+      <c r="V134" s="6"/>
+      <c r="W134" s="6"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AH130"/>
+  <autoFilter ref="A1:AH135"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>